<commit_message>
claude og jeg i main
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
+++ b/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
@@ -1437,7 +1437,9 @@
       <c r="DE2" t="inlineStr"/>
       <c r="DF2" t="inlineStr"/>
       <c r="DG2" t="inlineStr"/>
-      <c r="DH2" t="inlineStr"/>
+      <c r="DH2" t="n">
+        <v>0.4168509209269715</v>
+      </c>
       <c r="DI2" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -1794,7 +1796,9 @@
       <c r="DE3" t="inlineStr"/>
       <c r="DF3" t="inlineStr"/>
       <c r="DG3" t="inlineStr"/>
-      <c r="DH3" t="inlineStr"/>
+      <c r="DH3" t="n">
+        <v>0.3510801462589335</v>
+      </c>
       <c r="DI3" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -2151,7 +2155,9 @@
       <c r="DE4" t="inlineStr"/>
       <c r="DF4" t="inlineStr"/>
       <c r="DG4" t="inlineStr"/>
-      <c r="DH4" t="inlineStr"/>
+      <c r="DH4" t="n">
+        <v>0.9710500856002894</v>
+      </c>
       <c r="DI4" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -2508,7 +2514,9 @@
       <c r="DE5" t="inlineStr"/>
       <c r="DF5" t="inlineStr"/>
       <c r="DG5" t="inlineStr"/>
-      <c r="DH5" t="inlineStr"/>
+      <c r="DH5" t="n">
+        <v>0.2390120541241804</v>
+      </c>
       <c r="DI5" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -2865,7 +2873,9 @@
       <c r="DE6" t="inlineStr"/>
       <c r="DF6" t="inlineStr"/>
       <c r="DG6" t="inlineStr"/>
-      <c r="DH6" t="inlineStr"/>
+      <c r="DH6" t="n">
+        <v>0.1498211582610251</v>
+      </c>
       <c r="DI6" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -3222,7 +3232,9 @@
       <c r="DE7" t="inlineStr"/>
       <c r="DF7" t="inlineStr"/>
       <c r="DG7" t="inlineStr"/>
-      <c r="DH7" t="inlineStr"/>
+      <c r="DH7" t="n">
+        <v>0.8869972338644152</v>
+      </c>
       <c r="DI7" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -3579,7 +3591,9 @@
       <c r="DE8" t="inlineStr"/>
       <c r="DF8" t="inlineStr"/>
       <c r="DG8" t="inlineStr"/>
-      <c r="DH8" t="inlineStr"/>
+      <c r="DH8" t="n">
+        <v>0.156624220701184</v>
+      </c>
       <c r="DI8" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -3936,7 +3950,9 @@
       <c r="DE9" t="inlineStr"/>
       <c r="DF9" t="inlineStr"/>
       <c r="DG9" t="inlineStr"/>
-      <c r="DH9" t="inlineStr"/>
+      <c r="DH9" t="n">
+        <v>0.2484155525087566</v>
+      </c>
       <c r="DI9" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -4293,7 +4309,9 @@
       <c r="DE10" t="inlineStr"/>
       <c r="DF10" t="inlineStr"/>
       <c r="DG10" t="inlineStr"/>
-      <c r="DH10" t="inlineStr"/>
+      <c r="DH10" t="n">
+        <v>0.3305528262613096</v>
+      </c>
       <c r="DI10" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -4650,7 +4668,9 @@
       <c r="DE11" t="inlineStr"/>
       <c r="DF11" t="inlineStr"/>
       <c r="DG11" t="inlineStr"/>
-      <c r="DH11" t="inlineStr"/>
+      <c r="DH11" t="n">
+        <v>0.177487554142807</v>
+      </c>
       <c r="DI11" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -5007,7 +5027,9 @@
       <c r="DE12" t="inlineStr"/>
       <c r="DF12" t="inlineStr"/>
       <c r="DG12" t="inlineStr"/>
-      <c r="DH12" t="inlineStr"/>
+      <c r="DH12" t="n">
+        <v>0.6650403051306145</v>
+      </c>
       <c r="DI12" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -5609,7 +5631,9 @@
       <c r="DE14" t="inlineStr"/>
       <c r="DF14" t="inlineStr"/>
       <c r="DG14" t="inlineStr"/>
-      <c r="DH14" t="inlineStr"/>
+      <c r="DH14" t="n">
+        <v>0.8121898302828405</v>
+      </c>
       <c r="DI14" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -6215,7 +6239,9 @@
       <c r="DE16" t="inlineStr"/>
       <c r="DF16" t="inlineStr"/>
       <c r="DG16" t="inlineStr"/>
-      <c r="DH16" t="inlineStr"/>
+      <c r="DH16" t="n">
+        <v>0.1711120015564108</v>
+      </c>
       <c r="DI16" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -6572,7 +6598,9 @@
       <c r="DE17" t="inlineStr"/>
       <c r="DF17" t="inlineStr"/>
       <c r="DG17" t="inlineStr"/>
-      <c r="DH17" t="inlineStr"/>
+      <c r="DH17" t="n">
+        <v>0.3377173610857986</v>
+      </c>
       <c r="DI17" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -6929,7 +6957,9 @@
       <c r="DE18" t="inlineStr"/>
       <c r="DF18" t="inlineStr"/>
       <c r="DG18" t="inlineStr"/>
-      <c r="DH18" t="inlineStr"/>
+      <c r="DH18" t="n">
+        <v>0.1985630424984809</v>
+      </c>
       <c r="DI18" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -7286,7 +7316,9 @@
       <c r="DE19" t="inlineStr"/>
       <c r="DF19" t="inlineStr"/>
       <c r="DG19" t="inlineStr"/>
-      <c r="DH19" t="inlineStr"/>
+      <c r="DH19" t="n">
+        <v>0.5011686247978796</v>
+      </c>
       <c r="DI19" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -7643,7 +7675,9 @@
       <c r="DE20" t="inlineStr"/>
       <c r="DF20" t="inlineStr"/>
       <c r="DG20" t="inlineStr"/>
-      <c r="DH20" t="inlineStr"/>
+      <c r="DH20" t="n">
+        <v>0.8250920994353811</v>
+      </c>
       <c r="DI20" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -8000,7 +8034,9 @@
       <c r="DE21" t="inlineStr"/>
       <c r="DF21" t="inlineStr"/>
       <c r="DG21" t="inlineStr"/>
-      <c r="DH21" t="inlineStr"/>
+      <c r="DH21" t="n">
+        <v>0.1115590813504107</v>
+      </c>
       <c r="DI21" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -8357,7 +8393,9 @@
       <c r="DE22" t="inlineStr"/>
       <c r="DF22" t="inlineStr"/>
       <c r="DG22" t="inlineStr"/>
-      <c r="DH22" t="inlineStr"/>
+      <c r="DH22" t="n">
+        <v>0.1800065046926276</v>
+      </c>
       <c r="DI22" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -8714,7 +8752,9 @@
       <c r="DE23" t="inlineStr"/>
       <c r="DF23" t="inlineStr"/>
       <c r="DG23" t="inlineStr"/>
-      <c r="DH23" t="inlineStr"/>
+      <c r="DH23" t="n">
+        <v>0.4259434984905918</v>
+      </c>
       <c r="DI23" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -9071,7 +9111,9 @@
       <c r="DE24" t="inlineStr"/>
       <c r="DF24" t="inlineStr"/>
       <c r="DG24" t="inlineStr"/>
-      <c r="DH24" t="inlineStr"/>
+      <c r="DH24" t="n">
+        <v>0.8713273200982731</v>
+      </c>
       <c r="DI24" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -9428,7 +9470,9 @@
       <c r="DE25" t="inlineStr"/>
       <c r="DF25" t="inlineStr"/>
       <c r="DG25" t="inlineStr"/>
-      <c r="DH25" t="inlineStr"/>
+      <c r="DH25" t="n">
+        <v>0.1814543706923444</v>
+      </c>
       <c r="DI25" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -9785,7 +9829,9 @@
       <c r="DE26" t="inlineStr"/>
       <c r="DF26" t="inlineStr"/>
       <c r="DG26" t="inlineStr"/>
-      <c r="DH26" t="inlineStr"/>
+      <c r="DH26" t="n">
+        <v>0.6578783270375694</v>
+      </c>
       <c r="DI26" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -10142,7 +10188,9 @@
       <c r="DE27" t="inlineStr"/>
       <c r="DF27" t="inlineStr"/>
       <c r="DG27" t="inlineStr"/>
-      <c r="DH27" t="inlineStr"/>
+      <c r="DH27" t="n">
+        <v>0.1928520351914384</v>
+      </c>
       <c r="DI27" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -10499,7 +10547,9 @@
       <c r="DE28" t="inlineStr"/>
       <c r="DF28" t="inlineStr"/>
       <c r="DG28" t="inlineStr"/>
-      <c r="DH28" t="inlineStr"/>
+      <c r="DH28" t="n">
+        <v>0.4874679417682617</v>
+      </c>
       <c r="DI28" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -11356,7 +11406,9 @@
       <c r="DE31" t="inlineStr"/>
       <c r="DF31" t="inlineStr"/>
       <c r="DG31" t="inlineStr"/>
-      <c r="DH31" t="inlineStr"/>
+      <c r="DH31" t="n">
+        <v>0.5457616688958367</v>
+      </c>
       <c r="DI31" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -11970,7 +12022,9 @@
       <c r="DE33" t="inlineStr"/>
       <c r="DF33" t="inlineStr"/>
       <c r="DG33" t="inlineStr"/>
-      <c r="DH33" t="inlineStr"/>
+      <c r="DH33" t="n">
+        <v>0.5916552355514699</v>
+      </c>
       <c r="DI33" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -12327,7 +12381,9 @@
       <c r="DE34" t="inlineStr"/>
       <c r="DF34" t="inlineStr"/>
       <c r="DG34" t="inlineStr"/>
-      <c r="DH34" t="inlineStr"/>
+      <c r="DH34" t="n">
+        <v>0.1358791260329088</v>
+      </c>
       <c r="DI34" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -12684,7 +12740,9 @@
       <c r="DE35" t="inlineStr"/>
       <c r="DF35" t="inlineStr"/>
       <c r="DG35" t="inlineStr"/>
-      <c r="DH35" t="inlineStr"/>
+      <c r="DH35" t="n">
+        <v>0.1345789722721871</v>
+      </c>
       <c r="DI35" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -13041,7 +13099,9 @@
       <c r="DE36" t="inlineStr"/>
       <c r="DF36" t="inlineStr"/>
       <c r="DG36" t="inlineStr"/>
-      <c r="DH36" t="inlineStr"/>
+      <c r="DH36" t="n">
+        <v>0.5285268589333408</v>
+      </c>
       <c r="DI36" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -13398,7 +13458,9 @@
       <c r="DE37" t="inlineStr"/>
       <c r="DF37" t="inlineStr"/>
       <c r="DG37" t="inlineStr"/>
-      <c r="DH37" t="inlineStr"/>
+      <c r="DH37" t="n">
+        <v>0.3232977061252653</v>
+      </c>
       <c r="DI37" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -13755,7 +13817,9 @@
       <c r="DE38" t="inlineStr"/>
       <c r="DF38" t="inlineStr"/>
       <c r="DG38" t="inlineStr"/>
-      <c r="DH38" t="inlineStr"/>
+      <c r="DH38" t="n">
+        <v>0.2968671593549307</v>
+      </c>
       <c r="DI38" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -14112,7 +14176,9 @@
       <c r="DE39" t="inlineStr"/>
       <c r="DF39" t="inlineStr"/>
       <c r="DG39" t="inlineStr"/>
-      <c r="DH39" t="inlineStr"/>
+      <c r="DH39" t="n">
+        <v>0.5424014389417392</v>
+      </c>
       <c r="DI39" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -14469,7 +14535,9 @@
       <c r="DE40" t="inlineStr"/>
       <c r="DF40" t="inlineStr"/>
       <c r="DG40" t="inlineStr"/>
-      <c r="DH40" t="inlineStr"/>
+      <c r="DH40" t="n">
+        <v>0.2956365413743471</v>
+      </c>
       <c r="DI40" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -14826,7 +14894,9 @@
       <c r="DE41" t="inlineStr"/>
       <c r="DF41" t="inlineStr"/>
       <c r="DG41" t="inlineStr"/>
-      <c r="DH41" t="inlineStr"/>
+      <c r="DH41" t="n">
+        <v>0.5267886890989452</v>
+      </c>
       <c r="DI41" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -15183,7 +15253,9 @@
       <c r="DE42" t="inlineStr"/>
       <c r="DF42" t="inlineStr"/>
       <c r="DG42" t="inlineStr"/>
-      <c r="DH42" t="inlineStr"/>
+      <c r="DH42" t="n">
+        <v>0.1512371502199017</v>
+      </c>
       <c r="DI42" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -15540,7 +15612,9 @@
       <c r="DE43" t="inlineStr"/>
       <c r="DF43" t="inlineStr"/>
       <c r="DG43" t="inlineStr"/>
-      <c r="DH43" t="inlineStr"/>
+      <c r="DH43" t="n">
+        <v>0.5156152317264465</v>
+      </c>
       <c r="DI43" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -15897,7 +15971,9 @@
       <c r="DE44" t="inlineStr"/>
       <c r="DF44" t="inlineStr"/>
       <c r="DG44" t="inlineStr"/>
-      <c r="DH44" t="inlineStr"/>
+      <c r="DH44" t="n">
+        <v>0.5085100106963746</v>
+      </c>
       <c r="DI44" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -16254,7 +16330,9 @@
       <c r="DE45" t="inlineStr"/>
       <c r="DF45" t="inlineStr"/>
       <c r="DG45" t="inlineStr"/>
-      <c r="DH45" t="inlineStr"/>
+      <c r="DH45" t="n">
+        <v>0.2569401170240794</v>
+      </c>
       <c r="DI45" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -16611,7 +16689,9 @@
       <c r="DE46" t="inlineStr"/>
       <c r="DF46" t="inlineStr"/>
       <c r="DG46" t="inlineStr"/>
-      <c r="DH46" t="inlineStr"/>
+      <c r="DH46" t="n">
+        <v>0.4536086363286888</v>
+      </c>
       <c r="DI46" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -16968,7 +17048,9 @@
       <c r="DE47" t="inlineStr"/>
       <c r="DF47" t="inlineStr"/>
       <c r="DG47" t="inlineStr"/>
-      <c r="DH47" t="inlineStr"/>
+      <c r="DH47" t="n">
+        <v>0.7402315880191129</v>
+      </c>
       <c r="DI47" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -17325,7 +17407,9 @@
       <c r="DE48" t="inlineStr"/>
       <c r="DF48" t="inlineStr"/>
       <c r="DG48" t="inlineStr"/>
-      <c r="DH48" t="inlineStr"/>
+      <c r="DH48" t="n">
+        <v>0.176591398891399</v>
+      </c>
       <c r="DI48" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -17682,7 +17766,9 @@
       <c r="DE49" t="inlineStr"/>
       <c r="DF49" t="inlineStr"/>
       <c r="DG49" t="inlineStr"/>
-      <c r="DH49" t="inlineStr"/>
+      <c r="DH49" t="n">
+        <v>0.1828275131397293</v>
+      </c>
       <c r="DI49" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -18039,7 +18125,9 @@
       <c r="DE50" t="inlineStr"/>
       <c r="DF50" t="inlineStr"/>
       <c r="DG50" t="inlineStr"/>
-      <c r="DH50" t="inlineStr"/>
+      <c r="DH50" t="n">
+        <v>0.2021097791470266</v>
+      </c>
       <c r="DI50" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -18396,7 +18484,9 @@
       <c r="DE51" t="inlineStr"/>
       <c r="DF51" t="inlineStr"/>
       <c r="DG51" t="inlineStr"/>
-      <c r="DH51" t="inlineStr"/>
+      <c r="DH51" t="n">
+        <v>0.1335347198043298</v>
+      </c>
       <c r="DI51" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -19002,7 +19092,9 @@
       <c r="DE53" t="inlineStr"/>
       <c r="DF53" t="inlineStr"/>
       <c r="DG53" t="inlineStr"/>
-      <c r="DH53" t="inlineStr"/>
+      <c r="DH53" t="n">
+        <v>0.671597538362207</v>
+      </c>
       <c r="DI53" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -19359,7 +19451,9 @@
       <c r="DE54" t="inlineStr"/>
       <c r="DF54" t="inlineStr"/>
       <c r="DG54" t="inlineStr"/>
-      <c r="DH54" t="inlineStr"/>
+      <c r="DH54" t="n">
+        <v>0.1520888189722116</v>
+      </c>
       <c r="DI54" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
@@ -19716,7 +19810,9 @@
       <c r="DE55" t="inlineStr"/>
       <c r="DF55" t="inlineStr"/>
       <c r="DG55" t="inlineStr"/>
-      <c r="DH55" t="inlineStr"/>
+      <c r="DH55" t="n">
+        <v>0.7270716869919048</v>
+      </c>
       <c r="DI55" t="inlineStr">
         <is>
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>

</xml_diff>

<commit_message>
claude: Refactor to position-based probe column naming: fix OUT/IN computation, PSD band amplitudes, swell scatter plot, grouper column detection, and probe ordering in all-probes plot
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
+++ b/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FI55"/>
+  <dimension ref="A1:FU55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1240,6 +1240,66 @@
       <c r="FI1" t="inlineStr">
         <is>
           <t>Probe 8804 Celerity (FFT)</t>
+        </is>
+      </c>
+      <c r="FJ1" t="inlineStr">
+        <is>
+          <t>Probe 9373/170 Swell Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>Probe 9373/170 Wind Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>Probe 9373/170 Total Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>Probe 12545 Swell Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>Probe 12545 Wind Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FO1" t="inlineStr">
+        <is>
+          <t>Probe 12545 Total Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FP1" t="inlineStr">
+        <is>
+          <t>Probe 9373/340 Swell Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FQ1" t="inlineStr">
+        <is>
+          <t>Probe 9373/340 Wind Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FR1" t="inlineStr">
+        <is>
+          <t>Probe 9373/340 Total Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>Probe 8804 Swell Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>Probe 8804 Wind Amplitude (PSD)</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>Probe 8804 Total Amplitude (PSD)</t>
         </is>
       </c>
     </row>
@@ -1601,6 +1661,42 @@
       <c r="FI2" t="n">
         <v>1.187816136416175</v>
       </c>
+      <c r="FJ2" t="n">
+        <v>1.771812410244804</v>
+      </c>
+      <c r="FK2" t="n">
+        <v>8.598773705927615</v>
+      </c>
+      <c r="FL2" t="n">
+        <v>8.77942073617899</v>
+      </c>
+      <c r="FM2" t="n">
+        <v>0.4767152619678585</v>
+      </c>
+      <c r="FN2" t="n">
+        <v>0.3485586506474362</v>
+      </c>
+      <c r="FO2" t="n">
+        <v>0.5905510764821663</v>
+      </c>
+      <c r="FP2" t="n">
+        <v>1.54665260274402</v>
+      </c>
+      <c r="FQ2" t="n">
+        <v>7.952300578192454</v>
+      </c>
+      <c r="FR2" t="n">
+        <v>8.10130969408619</v>
+      </c>
+      <c r="FS2" t="n">
+        <v>1.747733807722847</v>
+      </c>
+      <c r="FT2" t="n">
+        <v>8.412106630442134</v>
+      </c>
+      <c r="FU2" t="n">
+        <v>8.591746703935463</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1960,6 +2056,42 @@
       <c r="FI3" t="n">
         <v>1.098609364819519</v>
       </c>
+      <c r="FJ3" t="n">
+        <v>0.2569338702111716</v>
+      </c>
+      <c r="FK3" t="n">
+        <v>0.2345700357124621</v>
+      </c>
+      <c r="FL3" t="n">
+        <v>0.347905325219142</v>
+      </c>
+      <c r="FM3" t="n">
+        <v>0.01545724933767163</v>
+      </c>
+      <c r="FN3" t="n">
+        <v>0.01976122902583179</v>
+      </c>
+      <c r="FO3" t="n">
+        <v>0.0250884979562015</v>
+      </c>
+      <c r="FP3" t="n">
+        <v>0.4255443773470479</v>
+      </c>
+      <c r="FQ3" t="n">
+        <v>0.1244255942448564</v>
+      </c>
+      <c r="FR3" t="n">
+        <v>0.4433618675471226</v>
+      </c>
+      <c r="FS3" t="n">
+        <v>0.2126262547829662</v>
+      </c>
+      <c r="FT3" t="n">
+        <v>0.2343710435090477</v>
+      </c>
+      <c r="FU3" t="n">
+        <v>0.3164485902299942</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2319,6 +2451,42 @@
       <c r="FI4" t="n">
         <v>1.942684020882263</v>
       </c>
+      <c r="FJ4" t="n">
+        <v>14.0564722993424</v>
+      </c>
+      <c r="FK4" t="n">
+        <v>7.995156719522582</v>
+      </c>
+      <c r="FL4" t="n">
+        <v>16.17117634780807</v>
+      </c>
+      <c r="FM4" t="n">
+        <v>12.99024384442987</v>
+      </c>
+      <c r="FN4" t="n">
+        <v>0.6800318204706834</v>
+      </c>
+      <c r="FO4" t="n">
+        <v>13.00803130433659</v>
+      </c>
+      <c r="FP4" t="n">
+        <v>13.97812676542665</v>
+      </c>
+      <c r="FQ4" t="n">
+        <v>7.108740060065507</v>
+      </c>
+      <c r="FR4" t="n">
+        <v>15.68190718987703</v>
+      </c>
+      <c r="FS4" t="n">
+        <v>13.80005527182242</v>
+      </c>
+      <c r="FT4" t="n">
+        <v>5.51250276308433</v>
+      </c>
+      <c r="FU4" t="n">
+        <v>14.86032342240121</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2678,6 +2846,42 @@
       <c r="FI5" t="n">
         <v>1.162574609521982</v>
       </c>
+      <c r="FJ5" t="n">
+        <v>2.025178734246257</v>
+      </c>
+      <c r="FK5" t="n">
+        <v>7.1668182388075</v>
+      </c>
+      <c r="FL5" t="n">
+        <v>7.447458128364812</v>
+      </c>
+      <c r="FM5" t="n">
+        <v>0.5450108997857883</v>
+      </c>
+      <c r="FN5" t="n">
+        <v>0.4134341415568038</v>
+      </c>
+      <c r="FO5" t="n">
+        <v>0.6840794327343324</v>
+      </c>
+      <c r="FP5" t="n">
+        <v>1.813426907526454</v>
+      </c>
+      <c r="FQ5" t="n">
+        <v>8.101961467805477</v>
+      </c>
+      <c r="FR5" t="n">
+        <v>8.302427161664571</v>
+      </c>
+      <c r="FS5" t="n">
+        <v>1.332345883759544</v>
+      </c>
+      <c r="FT5" t="n">
+        <v>8.147531205159472</v>
+      </c>
+      <c r="FU5" t="n">
+        <v>8.255750135088778</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3037,6 +3241,42 @@
       <c r="FI6" t="n">
         <v>1.316954165864082</v>
       </c>
+      <c r="FJ6" t="n">
+        <v>0.5475865491460892</v>
+      </c>
+      <c r="FK6" t="n">
+        <v>0.2764354922289936</v>
+      </c>
+      <c r="FL6" t="n">
+        <v>0.6134065618899167</v>
+      </c>
+      <c r="FM6" t="n">
+        <v>0.2294291548178547</v>
+      </c>
+      <c r="FN6" t="n">
+        <v>0.0849581091622485</v>
+      </c>
+      <c r="FO6" t="n">
+        <v>0.2446540770002815</v>
+      </c>
+      <c r="FP6" t="n">
+        <v>0.5264746906613557</v>
+      </c>
+      <c r="FQ6" t="n">
+        <v>0.1271623896360732</v>
+      </c>
+      <c r="FR6" t="n">
+        <v>0.5416141368584525</v>
+      </c>
+      <c r="FS6" t="n">
+        <v>0.5662606067017698</v>
+      </c>
+      <c r="FT6" t="n">
+        <v>0.2930291225191731</v>
+      </c>
+      <c r="FU6" t="n">
+        <v>0.6375869676731268</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3396,6 +3636,42 @@
       <c r="FI7" t="n">
         <v>1.945721282483451</v>
       </c>
+      <c r="FJ7" t="n">
+        <v>14.09402088958368</v>
+      </c>
+      <c r="FK7" t="n">
+        <v>8.550948026541384</v>
+      </c>
+      <c r="FL7" t="n">
+        <v>16.4851489829068</v>
+      </c>
+      <c r="FM7" t="n">
+        <v>13.08951615222986</v>
+      </c>
+      <c r="FN7" t="n">
+        <v>0.7235472194145429</v>
+      </c>
+      <c r="FO7" t="n">
+        <v>13.10949860514158</v>
+      </c>
+      <c r="FP7" t="n">
+        <v>14.04152221769476</v>
+      </c>
+      <c r="FQ7" t="n">
+        <v>8.163236049751021</v>
+      </c>
+      <c r="FR7" t="n">
+        <v>16.24200631061231</v>
+      </c>
+      <c r="FS7" t="n">
+        <v>13.83678896156808</v>
+      </c>
+      <c r="FT7" t="n">
+        <v>7.219429265302268</v>
+      </c>
+      <c r="FU7" t="n">
+        <v>15.6069499801747</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3755,6 +4031,42 @@
       <c r="FI8" t="n">
         <v>0.8792368949489662</v>
       </c>
+      <c r="FJ8" t="n">
+        <v>1.718003466451163</v>
+      </c>
+      <c r="FK8" t="n">
+        <v>8.695563900853456</v>
+      </c>
+      <c r="FL8" t="n">
+        <v>8.863654295185704</v>
+      </c>
+      <c r="FM8" t="n">
+        <v>0.3886494977733614</v>
+      </c>
+      <c r="FN8" t="n">
+        <v>0.3018501677900433</v>
+      </c>
+      <c r="FO8" t="n">
+        <v>0.4920995386244163</v>
+      </c>
+      <c r="FP8" t="n">
+        <v>1.188752761078823</v>
+      </c>
+      <c r="FQ8" t="n">
+        <v>7.773673726218001</v>
+      </c>
+      <c r="FR8" t="n">
+        <v>7.864040712551313</v>
+      </c>
+      <c r="FS8" t="n">
+        <v>1.147961845373633</v>
+      </c>
+      <c r="FT8" t="n">
+        <v>6.590044362598596</v>
+      </c>
+      <c r="FU8" t="n">
+        <v>6.689282554912087</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4114,6 +4426,42 @@
       <c r="FI9" t="n">
         <v>1.193989394226231</v>
       </c>
+      <c r="FJ9" t="n">
+        <v>0.3902306106172115</v>
+      </c>
+      <c r="FK9" t="n">
+        <v>0.2229987190898928</v>
+      </c>
+      <c r="FL9" t="n">
+        <v>0.4494533993401481</v>
+      </c>
+      <c r="FM9" t="n">
+        <v>0.0778016722611917</v>
+      </c>
+      <c r="FN9" t="n">
+        <v>0.07070023050996813</v>
+      </c>
+      <c r="FO9" t="n">
+        <v>0.1051266988010206</v>
+      </c>
+      <c r="FP9" t="n">
+        <v>2.828753555709682</v>
+      </c>
+      <c r="FQ9" t="n">
+        <v>0.1521382735043302</v>
+      </c>
+      <c r="FR9" t="n">
+        <v>2.832841812245267</v>
+      </c>
+      <c r="FS9" t="n">
+        <v>0.8204041246228407</v>
+      </c>
+      <c r="FT9" t="n">
+        <v>0.246790575836475</v>
+      </c>
+      <c r="FU9" t="n">
+        <v>0.8567196250932207</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4473,6 +4821,42 @@
       <c r="FI10" t="n">
         <v>1.264890930902623</v>
       </c>
+      <c r="FJ10" t="n">
+        <v>0.2903306872937315</v>
+      </c>
+      <c r="FK10" t="n">
+        <v>0.2093755715201862</v>
+      </c>
+      <c r="FL10" t="n">
+        <v>0.3579525638039978</v>
+      </c>
+      <c r="FM10" t="n">
+        <v>0.02625741053391764</v>
+      </c>
+      <c r="FN10" t="n">
+        <v>0.02940512298865377</v>
+      </c>
+      <c r="FO10" t="n">
+        <v>0.03942223821556234</v>
+      </c>
+      <c r="FP10" t="n">
+        <v>0.5035641268235784</v>
+      </c>
+      <c r="FQ10" t="n">
+        <v>0.1630495318215809</v>
+      </c>
+      <c r="FR10" t="n">
+        <v>0.529303296466997</v>
+      </c>
+      <c r="FS10" t="n">
+        <v>0.1967877471169936</v>
+      </c>
+      <c r="FT10" t="n">
+        <v>0.2377984905751512</v>
+      </c>
+      <c r="FU10" t="n">
+        <v>0.3086641209068557</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4832,6 +5216,42 @@
       <c r="FI11" t="n">
         <v>1.133579292726939</v>
       </c>
+      <c r="FJ11" t="n">
+        <v>1.719461519003797</v>
+      </c>
+      <c r="FK11" t="n">
+        <v>0.2841784810126997</v>
+      </c>
+      <c r="FL11" t="n">
+        <v>1.742786654873605</v>
+      </c>
+      <c r="FM11" t="n">
+        <v>0.5842484917335113</v>
+      </c>
+      <c r="FN11" t="n">
+        <v>0.1565865740633791</v>
+      </c>
+      <c r="FO11" t="n">
+        <v>0.6048682958047884</v>
+      </c>
+      <c r="FP11" t="n">
+        <v>3.42462737929076</v>
+      </c>
+      <c r="FQ11" t="n">
+        <v>0.152219191568271</v>
+      </c>
+      <c r="FR11" t="n">
+        <v>3.428008659450789</v>
+      </c>
+      <c r="FS11" t="n">
+        <v>2.268570903168181</v>
+      </c>
+      <c r="FT11" t="n">
+        <v>0.2774050550331268</v>
+      </c>
+      <c r="FU11" t="n">
+        <v>2.285468771884496</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5190,6 +5610,42 @@
       </c>
       <c r="FI12" t="n">
         <v>0.902978760080029</v>
+      </c>
+      <c r="FJ12" t="n">
+        <v>2.163300689528062</v>
+      </c>
+      <c r="FK12" t="n">
+        <v>8.20211235029541</v>
+      </c>
+      <c r="FL12" t="n">
+        <v>8.482600832302618</v>
+      </c>
+      <c r="FM12" t="n">
+        <v>0.7275915278148936</v>
+      </c>
+      <c r="FN12" t="n">
+        <v>0.3673994834930855</v>
+      </c>
+      <c r="FO12" t="n">
+        <v>0.8150900636242582</v>
+      </c>
+      <c r="FP12" t="n">
+        <v>1.604624947868744</v>
+      </c>
+      <c r="FQ12" t="n">
+        <v>8.860765333108043</v>
+      </c>
+      <c r="FR12" t="n">
+        <v>9.004886646245586</v>
+      </c>
+      <c r="FS12" t="n">
+        <v>1.58546546939955</v>
+      </c>
+      <c r="FT12" t="n">
+        <v>7.420812162600787</v>
+      </c>
+      <c r="FU12" t="n">
+        <v>7.588290578731293</v>
       </c>
     </row>
     <row r="13">
@@ -5436,6 +5892,18 @@
       <c r="FG13" t="inlineStr"/>
       <c r="FH13" t="inlineStr"/>
       <c r="FI13" t="inlineStr"/>
+      <c r="FJ13" t="inlineStr"/>
+      <c r="FK13" t="inlineStr"/>
+      <c r="FL13" t="inlineStr"/>
+      <c r="FM13" t="inlineStr"/>
+      <c r="FN13" t="inlineStr"/>
+      <c r="FO13" t="inlineStr"/>
+      <c r="FP13" t="inlineStr"/>
+      <c r="FQ13" t="inlineStr"/>
+      <c r="FR13" t="inlineStr"/>
+      <c r="FS13" t="inlineStr"/>
+      <c r="FT13" t="inlineStr"/>
+      <c r="FU13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5794,6 +6262,42 @@
       </c>
       <c r="FI14" t="n">
         <v>1.816531755137202</v>
+      </c>
+      <c r="FJ14" t="n">
+        <v>15.01676412758177</v>
+      </c>
+      <c r="FK14" t="n">
+        <v>7.700016469256914</v>
+      </c>
+      <c r="FL14" t="n">
+        <v>16.87582467585672</v>
+      </c>
+      <c r="FM14" t="n">
+        <v>13.25210738849798</v>
+      </c>
+      <c r="FN14" t="n">
+        <v>0.7304940883582224</v>
+      </c>
+      <c r="FO14" t="n">
+        <v>13.27222558011312</v>
+      </c>
+      <c r="FP14" t="n">
+        <v>15.1099702219194</v>
+      </c>
+      <c r="FQ14" t="n">
+        <v>7.534918044826206</v>
+      </c>
+      <c r="FR14" t="n">
+        <v>16.88449555211936</v>
+      </c>
+      <c r="FS14" t="n">
+        <v>15.79009140208618</v>
+      </c>
+      <c r="FT14" t="n">
+        <v>7.165867638077138</v>
+      </c>
+      <c r="FU14" t="n">
+        <v>17.34003014682146</v>
       </c>
     </row>
     <row r="15">
@@ -6044,6 +6548,18 @@
       <c r="FG15" t="inlineStr"/>
       <c r="FH15" t="inlineStr"/>
       <c r="FI15" t="inlineStr"/>
+      <c r="FJ15" t="inlineStr"/>
+      <c r="FK15" t="inlineStr"/>
+      <c r="FL15" t="inlineStr"/>
+      <c r="FM15" t="inlineStr"/>
+      <c r="FN15" t="inlineStr"/>
+      <c r="FO15" t="inlineStr"/>
+      <c r="FP15" t="inlineStr"/>
+      <c r="FQ15" t="inlineStr"/>
+      <c r="FR15" t="inlineStr"/>
+      <c r="FS15" t="inlineStr"/>
+      <c r="FT15" t="inlineStr"/>
+      <c r="FU15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6403,6 +6919,42 @@
       <c r="FI16" t="n">
         <v>1.111569801678024</v>
       </c>
+      <c r="FJ16" t="n">
+        <v>3.01477424904373</v>
+      </c>
+      <c r="FK16" t="n">
+        <v>9.348880301134997</v>
+      </c>
+      <c r="FL16" t="n">
+        <v>9.822954069812562</v>
+      </c>
+      <c r="FM16" t="n">
+        <v>0.7768036454793847</v>
+      </c>
+      <c r="FN16" t="n">
+        <v>0.4613535076633608</v>
+      </c>
+      <c r="FO16" t="n">
+        <v>0.9034771511573209</v>
+      </c>
+      <c r="FP16" t="n">
+        <v>2.828161555938423</v>
+      </c>
+      <c r="FQ16" t="n">
+        <v>8.353385682618818</v>
+      </c>
+      <c r="FR16" t="n">
+        <v>8.819158131537788</v>
+      </c>
+      <c r="FS16" t="n">
+        <v>3.378385377053944</v>
+      </c>
+      <c r="FT16" t="n">
+        <v>7.560016786387846</v>
+      </c>
+      <c r="FU16" t="n">
+        <v>8.280539932055031</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6762,6 +7314,42 @@
       <c r="FI17" t="n">
         <v>0.7832869829762423</v>
       </c>
+      <c r="FJ17" t="n">
+        <v>1.789644410235752</v>
+      </c>
+      <c r="FK17" t="n">
+        <v>9.93360786109108</v>
+      </c>
+      <c r="FL17" t="n">
+        <v>10.09353219903808</v>
+      </c>
+      <c r="FM17" t="n">
+        <v>0.4505873265272665</v>
+      </c>
+      <c r="FN17" t="n">
+        <v>0.3282656333230807</v>
+      </c>
+      <c r="FO17" t="n">
+        <v>0.557482972697815</v>
+      </c>
+      <c r="FP17" t="n">
+        <v>4.592957685801953</v>
+      </c>
+      <c r="FQ17" t="n">
+        <v>10.29948734021632</v>
+      </c>
+      <c r="FR17" t="n">
+        <v>11.27717605497243</v>
+      </c>
+      <c r="FS17" t="n">
+        <v>1.17225316725956</v>
+      </c>
+      <c r="FT17" t="n">
+        <v>7.608283883341123</v>
+      </c>
+      <c r="FU17" t="n">
+        <v>7.698062167692487</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7121,6 +7709,42 @@
       <c r="FI18" t="n">
         <v>1.126073825131297</v>
       </c>
+      <c r="FJ18" t="n">
+        <v>2.037055843371123</v>
+      </c>
+      <c r="FK18" t="n">
+        <v>8.311816822236782</v>
+      </c>
+      <c r="FL18" t="n">
+        <v>8.557797344844689</v>
+      </c>
+      <c r="FM18" t="n">
+        <v>0.5882030740322445</v>
+      </c>
+      <c r="FN18" t="n">
+        <v>0.3350410203727163</v>
+      </c>
+      <c r="FO18" t="n">
+        <v>0.6769308248509391</v>
+      </c>
+      <c r="FP18" t="n">
+        <v>1.663241498382127</v>
+      </c>
+      <c r="FQ18" t="n">
+        <v>8.454416440251132</v>
+      </c>
+      <c r="FR18" t="n">
+        <v>8.616468512513061</v>
+      </c>
+      <c r="FS18" t="n">
+        <v>1.869291545452095</v>
+      </c>
+      <c r="FT18" t="n">
+        <v>8.095250423875644</v>
+      </c>
+      <c r="FU18" t="n">
+        <v>8.308268791219833</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7480,6 +8104,42 @@
       <c r="FI19" t="n">
         <v>1.165605882826456</v>
       </c>
+      <c r="FJ19" t="n">
+        <v>1.766881579579202</v>
+      </c>
+      <c r="FK19" t="n">
+        <v>7.572748940417865</v>
+      </c>
+      <c r="FL19" t="n">
+        <v>7.776142811886636</v>
+      </c>
+      <c r="FM19" t="n">
+        <v>0.5897388358710461</v>
+      </c>
+      <c r="FN19" t="n">
+        <v>0.3782209692922325</v>
+      </c>
+      <c r="FO19" t="n">
+        <v>0.7006018813469549</v>
+      </c>
+      <c r="FP19" t="n">
+        <v>1.387560386941324</v>
+      </c>
+      <c r="FQ19" t="n">
+        <v>8.781089284640954</v>
+      </c>
+      <c r="FR19" t="n">
+        <v>8.89004234254511</v>
+      </c>
+      <c r="FS19" t="n">
+        <v>1.426103575052908</v>
+      </c>
+      <c r="FT19" t="n">
+        <v>6.515489111837552</v>
+      </c>
+      <c r="FU19" t="n">
+        <v>6.669735360061326</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7839,6 +8499,42 @@
       <c r="FI20" t="n">
         <v>2.049595832795259</v>
       </c>
+      <c r="FJ20" t="n">
+        <v>12.36613674587938</v>
+      </c>
+      <c r="FK20" t="n">
+        <v>9.187062236518445</v>
+      </c>
+      <c r="FL20" t="n">
+        <v>15.40530592216369</v>
+      </c>
+      <c r="FM20" t="n">
+        <v>10.57947955407382</v>
+      </c>
+      <c r="FN20" t="n">
+        <v>0.56717924276562</v>
+      </c>
+      <c r="FO20" t="n">
+        <v>10.59467224261753</v>
+      </c>
+      <c r="FP20" t="n">
+        <v>12.19722697565197</v>
+      </c>
+      <c r="FQ20" t="n">
+        <v>8.216156395176062</v>
+      </c>
+      <c r="FR20" t="n">
+        <v>14.70637860948659</v>
+      </c>
+      <c r="FS20" t="n">
+        <v>11.32550141044773</v>
+      </c>
+      <c r="FT20" t="n">
+        <v>7.212419640668243</v>
+      </c>
+      <c r="FU20" t="n">
+        <v>13.42706145331698</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8198,6 +8894,42 @@
       <c r="FI21" t="n">
         <v>1.168255153011199</v>
       </c>
+      <c r="FJ21" t="n">
+        <v>4.740416437160764</v>
+      </c>
+      <c r="FK21" t="n">
+        <v>11.52555735153384</v>
+      </c>
+      <c r="FL21" t="n">
+        <v>12.46234409175095</v>
+      </c>
+      <c r="FM21" t="n">
+        <v>0.4638020221417332</v>
+      </c>
+      <c r="FN21" t="n">
+        <v>0.3348882238156782</v>
+      </c>
+      <c r="FO21" t="n">
+        <v>0.5720685607452838</v>
+      </c>
+      <c r="FP21" t="n">
+        <v>1.609771486501385</v>
+      </c>
+      <c r="FQ21" t="n">
+        <v>7.9762783084447</v>
+      </c>
+      <c r="FR21" t="n">
+        <v>8.137098985051018</v>
+      </c>
+      <c r="FS21" t="n">
+        <v>2.150965308606643</v>
+      </c>
+      <c r="FT21" t="n">
+        <v>8.090308881213199</v>
+      </c>
+      <c r="FU21" t="n">
+        <v>8.371364855999673</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8557,6 +9289,42 @@
       <c r="FI22" t="n">
         <v>1.180089393467238</v>
       </c>
+      <c r="FJ22" t="n">
+        <v>0.9291965770211569</v>
+      </c>
+      <c r="FK22" t="n">
+        <v>0.2587607754267011</v>
+      </c>
+      <c r="FL22" t="n">
+        <v>0.9645534809678842</v>
+      </c>
+      <c r="FM22" t="n">
+        <v>0.324757940083269</v>
+      </c>
+      <c r="FN22" t="n">
+        <v>0.1434555405949508</v>
+      </c>
+      <c r="FO22" t="n">
+        <v>0.3550312828111317</v>
+      </c>
+      <c r="FP22" t="n">
+        <v>2.385908682021681</v>
+      </c>
+      <c r="FQ22" t="n">
+        <v>0.1359783651054784</v>
+      </c>
+      <c r="FR22" t="n">
+        <v>2.389780398849065</v>
+      </c>
+      <c r="FS22" t="n">
+        <v>1.255450527966795</v>
+      </c>
+      <c r="FT22" t="n">
+        <v>0.2318212374026114</v>
+      </c>
+      <c r="FU22" t="n">
+        <v>1.27667423968802</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8916,6 +9684,42 @@
       <c r="FI23" t="n">
         <v>1.316621132854703</v>
       </c>
+      <c r="FJ23" t="n">
+        <v>0.2845731833293657</v>
+      </c>
+      <c r="FK23" t="n">
+        <v>0.2334350687847213</v>
+      </c>
+      <c r="FL23" t="n">
+        <v>0.3680676948724736</v>
+      </c>
+      <c r="FM23" t="n">
+        <v>0.1600367746637435</v>
+      </c>
+      <c r="FN23" t="n">
+        <v>0.0991157601665907</v>
+      </c>
+      <c r="FO23" t="n">
+        <v>0.1882437333835444</v>
+      </c>
+      <c r="FP23" t="n">
+        <v>0.4041538511857107</v>
+      </c>
+      <c r="FQ23" t="n">
+        <v>0.1125857640386134</v>
+      </c>
+      <c r="FR23" t="n">
+        <v>0.4195424766247154</v>
+      </c>
+      <c r="FS23" t="n">
+        <v>0.3255507576085295</v>
+      </c>
+      <c r="FT23" t="n">
+        <v>0.2277495243474225</v>
+      </c>
+      <c r="FU23" t="n">
+        <v>0.3973073641652829</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9275,6 +10079,42 @@
       <c r="FI24" t="n">
         <v>1.66895328415039</v>
       </c>
+      <c r="FJ24" t="n">
+        <v>15.60157140575128</v>
+      </c>
+      <c r="FK24" t="n">
+        <v>6.169847398040435</v>
+      </c>
+      <c r="FL24" t="n">
+        <v>16.7772479043454</v>
+      </c>
+      <c r="FM24" t="n">
+        <v>12.43077167354</v>
+      </c>
+      <c r="FN24" t="n">
+        <v>0.6563050964825067</v>
+      </c>
+      <c r="FO24" t="n">
+        <v>12.44808502458725</v>
+      </c>
+      <c r="FP24" t="n">
+        <v>15.72649156348198</v>
+      </c>
+      <c r="FQ24" t="n">
+        <v>7.509533828807492</v>
+      </c>
+      <c r="FR24" t="n">
+        <v>17.42743914699673</v>
+      </c>
+      <c r="FS24" t="n">
+        <v>16.05582227409923</v>
+      </c>
+      <c r="FT24" t="n">
+        <v>6.362997910360851</v>
+      </c>
+      <c r="FU24" t="n">
+        <v>17.27070268705699</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9634,6 +10474,42 @@
       <c r="FI25" t="n">
         <v>0.74917287252075</v>
       </c>
+      <c r="FJ25" t="n">
+        <v>1.645586784170358</v>
+      </c>
+      <c r="FK25" t="n">
+        <v>6.96403138270767</v>
+      </c>
+      <c r="FL25" t="n">
+        <v>7.155815045372081</v>
+      </c>
+      <c r="FM25" t="n">
+        <v>0.6294307236889297</v>
+      </c>
+      <c r="FN25" t="n">
+        <v>0.4474600122102669</v>
+      </c>
+      <c r="FO25" t="n">
+        <v>0.7722716480946209</v>
+      </c>
+      <c r="FP25" t="n">
+        <v>1.618622278670048</v>
+      </c>
+      <c r="FQ25" t="n">
+        <v>8.843641759120199</v>
+      </c>
+      <c r="FR25" t="n">
+        <v>8.99054712710309</v>
+      </c>
+      <c r="FS25" t="n">
+        <v>1.114370336550886</v>
+      </c>
+      <c r="FT25" t="n">
+        <v>5.887108264420349</v>
+      </c>
+      <c r="FU25" t="n">
+        <v>5.991649602904938</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9993,6 +10869,42 @@
       <c r="FI26" t="n">
         <v>1.192813932658235</v>
       </c>
+      <c r="FJ26" t="n">
+        <v>0.6671596805428824</v>
+      </c>
+      <c r="FK26" t="n">
+        <v>0.2869757337436439</v>
+      </c>
+      <c r="FL26" t="n">
+        <v>0.7262624257799545</v>
+      </c>
+      <c r="FM26" t="n">
+        <v>1.027048847843455</v>
+      </c>
+      <c r="FN26" t="n">
+        <v>0.1818497481191538</v>
+      </c>
+      <c r="FO26" t="n">
+        <v>1.043023809290836</v>
+      </c>
+      <c r="FP26" t="n">
+        <v>1.061138642535507</v>
+      </c>
+      <c r="FQ26" t="n">
+        <v>0.1686559759565866</v>
+      </c>
+      <c r="FR26" t="n">
+        <v>1.074458029384102</v>
+      </c>
+      <c r="FS26" t="n">
+        <v>1.490788532898586</v>
+      </c>
+      <c r="FT26" t="n">
+        <v>0.2896009968980653</v>
+      </c>
+      <c r="FU26" t="n">
+        <v>1.518657034101601</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10352,6 +11264,42 @@
       <c r="FI27" t="n">
         <v>1.157336579892411</v>
       </c>
+      <c r="FJ27" t="n">
+        <v>2.195763042146507</v>
+      </c>
+      <c r="FK27" t="n">
+        <v>7.93465853097363</v>
+      </c>
+      <c r="FL27" t="n">
+        <v>8.232871998301023</v>
+      </c>
+      <c r="FM27" t="n">
+        <v>0.4245887693714887</v>
+      </c>
+      <c r="FN27" t="n">
+        <v>0.4229918877081993</v>
+      </c>
+      <c r="FO27" t="n">
+        <v>0.5993310939233347</v>
+      </c>
+      <c r="FP27" t="n">
+        <v>2.054152681158393</v>
+      </c>
+      <c r="FQ27" t="n">
+        <v>6.657102894392769</v>
+      </c>
+      <c r="FR27" t="n">
+        <v>6.966818655888984</v>
+      </c>
+      <c r="FS27" t="n">
+        <v>2.397874661082844</v>
+      </c>
+      <c r="FT27" t="n">
+        <v>7.829977218890035</v>
+      </c>
+      <c r="FU27" t="n">
+        <v>8.188916053947562</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10710,6 +11658,42 @@
       </c>
       <c r="FI28" t="n">
         <v>1.360850120492653</v>
+      </c>
+      <c r="FJ28" t="n">
+        <v>1.207889824890587</v>
+      </c>
+      <c r="FK28" t="n">
+        <v>7.233536924432496</v>
+      </c>
+      <c r="FL28" t="n">
+        <v>7.333693085083568</v>
+      </c>
+      <c r="FM28" t="n">
+        <v>0.4401338394655961</v>
+      </c>
+      <c r="FN28" t="n">
+        <v>0.3524789322294102</v>
+      </c>
+      <c r="FO28" t="n">
+        <v>0.5638787053155248</v>
+      </c>
+      <c r="FP28" t="n">
+        <v>1.579760235714316</v>
+      </c>
+      <c r="FQ28" t="n">
+        <v>7.505963676319444</v>
+      </c>
+      <c r="FR28" t="n">
+        <v>7.670406319913636</v>
+      </c>
+      <c r="FS28" t="n">
+        <v>1.357367984015576</v>
+      </c>
+      <c r="FT28" t="n">
+        <v>7.417588146160777</v>
+      </c>
+      <c r="FU28" t="n">
+        <v>7.540760024698796</v>
       </c>
     </row>
     <row r="29">
@@ -10968,6 +11952,18 @@
       <c r="FG29" t="inlineStr"/>
       <c r="FH29" t="inlineStr"/>
       <c r="FI29" t="inlineStr"/>
+      <c r="FJ29" t="inlineStr"/>
+      <c r="FK29" t="inlineStr"/>
+      <c r="FL29" t="inlineStr"/>
+      <c r="FM29" t="inlineStr"/>
+      <c r="FN29" t="inlineStr"/>
+      <c r="FO29" t="inlineStr"/>
+      <c r="FP29" t="inlineStr"/>
+      <c r="FQ29" t="inlineStr"/>
+      <c r="FR29" t="inlineStr"/>
+      <c r="FS29" t="inlineStr"/>
+      <c r="FT29" t="inlineStr"/>
+      <c r="FU29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -11211,6 +12207,18 @@
       <c r="FG30" t="inlineStr"/>
       <c r="FH30" t="inlineStr"/>
       <c r="FI30" t="inlineStr"/>
+      <c r="FJ30" t="inlineStr"/>
+      <c r="FK30" t="inlineStr"/>
+      <c r="FL30" t="inlineStr"/>
+      <c r="FM30" t="inlineStr"/>
+      <c r="FN30" t="inlineStr"/>
+      <c r="FO30" t="inlineStr"/>
+      <c r="FP30" t="inlineStr"/>
+      <c r="FQ30" t="inlineStr"/>
+      <c r="FR30" t="inlineStr"/>
+      <c r="FS30" t="inlineStr"/>
+      <c r="FT30" t="inlineStr"/>
+      <c r="FU30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -11569,6 +12577,42 @@
       </c>
       <c r="FI31" t="n">
         <v>1.533165646509226</v>
+      </c>
+      <c r="FJ31" t="n">
+        <v>8.205973437845383</v>
+      </c>
+      <c r="FK31" t="n">
+        <v>8.676922370490557</v>
+      </c>
+      <c r="FL31" t="n">
+        <v>11.94265388789876</v>
+      </c>
+      <c r="FM31" t="n">
+        <v>3.463517113787987</v>
+      </c>
+      <c r="FN31" t="n">
+        <v>0.385797889440082</v>
+      </c>
+      <c r="FO31" t="n">
+        <v>3.484937705181929</v>
+      </c>
+      <c r="FP31" t="n">
+        <v>8.167505732488731</v>
+      </c>
+      <c r="FQ31" t="n">
+        <v>7.033335351011362</v>
+      </c>
+      <c r="FR31" t="n">
+        <v>10.77849507352592</v>
+      </c>
+      <c r="FS31" t="n">
+        <v>7.770374659783641</v>
+      </c>
+      <c r="FT31" t="n">
+        <v>7.043250583167478</v>
+      </c>
+      <c r="FU31" t="n">
+        <v>10.487425858174</v>
       </c>
     </row>
     <row r="32">
@@ -11827,6 +12871,18 @@
       <c r="FG32" t="inlineStr"/>
       <c r="FH32" t="inlineStr"/>
       <c r="FI32" t="inlineStr"/>
+      <c r="FJ32" t="inlineStr"/>
+      <c r="FK32" t="inlineStr"/>
+      <c r="FL32" t="inlineStr"/>
+      <c r="FM32" t="inlineStr"/>
+      <c r="FN32" t="inlineStr"/>
+      <c r="FO32" t="inlineStr"/>
+      <c r="FP32" t="inlineStr"/>
+      <c r="FQ32" t="inlineStr"/>
+      <c r="FR32" t="inlineStr"/>
+      <c r="FS32" t="inlineStr"/>
+      <c r="FT32" t="inlineStr"/>
+      <c r="FU32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -12186,6 +13242,42 @@
       <c r="FI33" t="n">
         <v>1.538145483781941</v>
       </c>
+      <c r="FJ33" t="n">
+        <v>7.907630174803121</v>
+      </c>
+      <c r="FK33" t="n">
+        <v>0.3498422027992996</v>
+      </c>
+      <c r="FL33" t="n">
+        <v>7.915365092547298</v>
+      </c>
+      <c r="FM33" t="n">
+        <v>5.116741486975672</v>
+      </c>
+      <c r="FN33" t="n">
+        <v>0.2435614185622338</v>
+      </c>
+      <c r="FO33" t="n">
+        <v>5.122535076419689</v>
+      </c>
+      <c r="FP33" t="n">
+        <v>7.804491682476962</v>
+      </c>
+      <c r="FQ33" t="n">
+        <v>0.2547591518605058</v>
+      </c>
+      <c r="FR33" t="n">
+        <v>7.808648580087899</v>
+      </c>
+      <c r="FS33" t="n">
+        <v>8.109782088392983</v>
+      </c>
+      <c r="FT33" t="n">
+        <v>0.2499005451643272</v>
+      </c>
+      <c r="FU33" t="n">
+        <v>8.113631480643736</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12545,6 +13637,42 @@
       <c r="FI34" t="n">
         <v>1.230971278407673</v>
       </c>
+      <c r="FJ34" t="n">
+        <v>2.216215003327047</v>
+      </c>
+      <c r="FK34" t="n">
+        <v>8.462068281931414</v>
+      </c>
+      <c r="FL34" t="n">
+        <v>8.747468693801743</v>
+      </c>
+      <c r="FM34" t="n">
+        <v>0.5966975086356637</v>
+      </c>
+      <c r="FN34" t="n">
+        <v>0.3285345574814942</v>
+      </c>
+      <c r="FO34" t="n">
+        <v>0.6811628823354728</v>
+      </c>
+      <c r="FP34" t="n">
+        <v>2.351949534429338</v>
+      </c>
+      <c r="FQ34" t="n">
+        <v>8.091376752411607</v>
+      </c>
+      <c r="FR34" t="n">
+        <v>8.426271082867522</v>
+      </c>
+      <c r="FS34" t="n">
+        <v>2.827709813147016</v>
+      </c>
+      <c r="FT34" t="n">
+        <v>7.36123698783431</v>
+      </c>
+      <c r="FU34" t="n">
+        <v>7.885667554394357</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12904,6 +14032,42 @@
       <c r="FI35" t="n">
         <v>1.188551314689845</v>
       </c>
+      <c r="FJ35" t="n">
+        <v>3.008649047303332</v>
+      </c>
+      <c r="FK35" t="n">
+        <v>0.3004355102852885</v>
+      </c>
+      <c r="FL35" t="n">
+        <v>3.0236121751441</v>
+      </c>
+      <c r="FM35" t="n">
+        <v>0.8427101835483108</v>
+      </c>
+      <c r="FN35" t="n">
+        <v>0.1546513635993811</v>
+      </c>
+      <c r="FO35" t="n">
+        <v>0.8567832267961224</v>
+      </c>
+      <c r="FP35" t="n">
+        <v>1.93182751967761</v>
+      </c>
+      <c r="FQ35" t="n">
+        <v>0.133464033658981</v>
+      </c>
+      <c r="FR35" t="n">
+        <v>1.936432341721309</v>
+      </c>
+      <c r="FS35" t="n">
+        <v>4.159548428751656</v>
+      </c>
+      <c r="FT35" t="n">
+        <v>0.2758088369536021</v>
+      </c>
+      <c r="FU35" t="n">
+        <v>4.168682483192031</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13263,6 +14427,42 @@
       <c r="FI36" t="n">
         <v>1.411100775691752</v>
       </c>
+      <c r="FJ36" t="n">
+        <v>12.99310764232061</v>
+      </c>
+      <c r="FK36" t="n">
+        <v>0.360892300418238</v>
+      </c>
+      <c r="FL36" t="n">
+        <v>12.99811868915773</v>
+      </c>
+      <c r="FM36" t="n">
+        <v>5.664363574900774</v>
+      </c>
+      <c r="FN36" t="n">
+        <v>0.2191090214655936</v>
+      </c>
+      <c r="FO36" t="n">
+        <v>5.668599780541072</v>
+      </c>
+      <c r="FP36" t="n">
+        <v>15.07782482479693</v>
+      </c>
+      <c r="FQ36" t="n">
+        <v>0.4337722473076037</v>
+      </c>
+      <c r="FR36" t="n">
+        <v>15.08406310679575</v>
+      </c>
+      <c r="FS36" t="n">
+        <v>14.28151795564476</v>
+      </c>
+      <c r="FT36" t="n">
+        <v>0.2847292462787374</v>
+      </c>
+      <c r="FU36" t="n">
+        <v>14.28435598342082</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13622,6 +14822,42 @@
       <c r="FI37" t="n">
         <v>1.311871197187217</v>
       </c>
+      <c r="FJ37" t="n">
+        <v>5.879751693630715</v>
+      </c>
+      <c r="FK37" t="n">
+        <v>0.2986201721670153</v>
+      </c>
+      <c r="FL37" t="n">
+        <v>5.88732995389067</v>
+      </c>
+      <c r="FM37" t="n">
+        <v>1.560217996677857</v>
+      </c>
+      <c r="FN37" t="n">
+        <v>0.1828350442791346</v>
+      </c>
+      <c r="FO37" t="n">
+        <v>1.570894283704037</v>
+      </c>
+      <c r="FP37" t="n">
+        <v>6.984554226112732</v>
+      </c>
+      <c r="FQ37" t="n">
+        <v>0.2683828443575317</v>
+      </c>
+      <c r="FR37" t="n">
+        <v>6.989708655491635</v>
+      </c>
+      <c r="FS37" t="n">
+        <v>6.333913038540704</v>
+      </c>
+      <c r="FT37" t="n">
+        <v>0.2236113102042181</v>
+      </c>
+      <c r="FU37" t="n">
+        <v>6.337858975856688</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13981,6 +15217,42 @@
       <c r="FI38" t="n">
         <v>1.314872069488793</v>
       </c>
+      <c r="FJ38" t="n">
+        <v>3.159090117559394</v>
+      </c>
+      <c r="FK38" t="n">
+        <v>8.713907186302237</v>
+      </c>
+      <c r="FL38" t="n">
+        <v>9.268874193900313</v>
+      </c>
+      <c r="FM38" t="n">
+        <v>0.8438660938037519</v>
+      </c>
+      <c r="FN38" t="n">
+        <v>0.3373738689417674</v>
+      </c>
+      <c r="FO38" t="n">
+        <v>0.9088075218198512</v>
+      </c>
+      <c r="FP38" t="n">
+        <v>3.109341077576107</v>
+      </c>
+      <c r="FQ38" t="n">
+        <v>7.5162894407559</v>
+      </c>
+      <c r="FR38" t="n">
+        <v>8.134040133532707</v>
+      </c>
+      <c r="FS38" t="n">
+        <v>6.321761427545957</v>
+      </c>
+      <c r="FT38" t="n">
+        <v>5.316850843196956</v>
+      </c>
+      <c r="FU38" t="n">
+        <v>8.260361398607937</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14340,6 +15612,42 @@
       <c r="FI39" t="n">
         <v>1.412295179821375</v>
       </c>
+      <c r="FJ39" t="n">
+        <v>13.30366779349172</v>
+      </c>
+      <c r="FK39" t="n">
+        <v>6.650540342233861</v>
+      </c>
+      <c r="FL39" t="n">
+        <v>14.87337431799754</v>
+      </c>
+      <c r="FM39" t="n">
+        <v>6.168476404595649</v>
+      </c>
+      <c r="FN39" t="n">
+        <v>0.4926844496021359</v>
+      </c>
+      <c r="FO39" t="n">
+        <v>6.188120806911662</v>
+      </c>
+      <c r="FP39" t="n">
+        <v>13.4447679930178</v>
+      </c>
+      <c r="FQ39" t="n">
+        <v>7.795970766868034</v>
+      </c>
+      <c r="FR39" t="n">
+        <v>15.54152330320091</v>
+      </c>
+      <c r="FS39" t="n">
+        <v>14.42616568462093</v>
+      </c>
+      <c r="FT39" t="n">
+        <v>5.144493413479315</v>
+      </c>
+      <c r="FU39" t="n">
+        <v>15.31600694833567</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14699,6 +16007,42 @@
       <c r="FI40" t="n">
         <v>1.316121510018907</v>
       </c>
+      <c r="FJ40" t="n">
+        <v>6.207780139359216</v>
+      </c>
+      <c r="FK40" t="n">
+        <v>8.05224645331074</v>
+      </c>
+      <c r="FL40" t="n">
+        <v>10.16735989347668</v>
+      </c>
+      <c r="FM40" t="n">
+        <v>1.409902383319888</v>
+      </c>
+      <c r="FN40" t="n">
+        <v>0.4121996719476386</v>
+      </c>
+      <c r="FO40" t="n">
+        <v>1.468922496268895</v>
+      </c>
+      <c r="FP40" t="n">
+        <v>6.360373469679094</v>
+      </c>
+      <c r="FQ40" t="n">
+        <v>8.485569481349666</v>
+      </c>
+      <c r="FR40" t="n">
+        <v>10.60468010345482</v>
+      </c>
+      <c r="FS40" t="n">
+        <v>12.68873338430673</v>
+      </c>
+      <c r="FT40" t="n">
+        <v>7.229725678505521</v>
+      </c>
+      <c r="FU40" t="n">
+        <v>14.60386552541697</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -15058,6 +16402,42 @@
       <c r="FI41" t="n">
         <v>1.408470098717027</v>
       </c>
+      <c r="FJ41" t="n">
+        <v>6.929899065990313</v>
+      </c>
+      <c r="FK41" t="n">
+        <v>9.766671742739202</v>
+      </c>
+      <c r="FL41" t="n">
+        <v>11.97544896842009</v>
+      </c>
+      <c r="FM41" t="n">
+        <v>3.022565977316682</v>
+      </c>
+      <c r="FN41" t="n">
+        <v>0.3734493556163624</v>
+      </c>
+      <c r="FO41" t="n">
+        <v>3.045549130853519</v>
+      </c>
+      <c r="FP41" t="n">
+        <v>6.670367062976138</v>
+      </c>
+      <c r="FQ41" t="n">
+        <v>7.230404417187239</v>
+      </c>
+      <c r="FR41" t="n">
+        <v>9.83730373582709</v>
+      </c>
+      <c r="FS41" t="n">
+        <v>7.462577168870305</v>
+      </c>
+      <c r="FT41" t="n">
+        <v>7.387891779104244</v>
+      </c>
+      <c r="FU41" t="n">
+        <v>10.50100009242455</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -15417,6 +16797,42 @@
       <c r="FI42" t="n">
         <v>1.201661839031998</v>
       </c>
+      <c r="FJ42" t="n">
+        <v>1.348276112070721</v>
+      </c>
+      <c r="FK42" t="n">
+        <v>0.2698604006183555</v>
+      </c>
+      <c r="FL42" t="n">
+        <v>1.375017494507775</v>
+      </c>
+      <c r="FM42" t="n">
+        <v>0.3944589798590894</v>
+      </c>
+      <c r="FN42" t="n">
+        <v>0.1540519940224033</v>
+      </c>
+      <c r="FO42" t="n">
+        <v>0.4234736162427974</v>
+      </c>
+      <c r="FP42" t="n">
+        <v>1.690320755450197</v>
+      </c>
+      <c r="FQ42" t="n">
+        <v>0.1514209516124925</v>
+      </c>
+      <c r="FR42" t="n">
+        <v>1.697089438094809</v>
+      </c>
+      <c r="FS42" t="n">
+        <v>1.980696601140864</v>
+      </c>
+      <c r="FT42" t="n">
+        <v>0.2182056221695956</v>
+      </c>
+      <c r="FU42" t="n">
+        <v>1.992679783436714</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -15776,6 +17192,42 @@
       <c r="FI43" t="n">
         <v>1.418016365693152</v>
       </c>
+      <c r="FJ43" t="n">
+        <v>6.471671254237674</v>
+      </c>
+      <c r="FK43" t="n">
+        <v>0.243472290091854</v>
+      </c>
+      <c r="FL43" t="n">
+        <v>6.476249499437834</v>
+      </c>
+      <c r="FM43" t="n">
+        <v>3.027027490559691</v>
+      </c>
+      <c r="FN43" t="n">
+        <v>0.1890722840056747</v>
+      </c>
+      <c r="FO43" t="n">
+        <v>3.032926599372827</v>
+      </c>
+      <c r="FP43" t="n">
+        <v>7.786909430202888</v>
+      </c>
+      <c r="FQ43" t="n">
+        <v>0.2179353154953514</v>
+      </c>
+      <c r="FR43" t="n">
+        <v>7.789958554185172</v>
+      </c>
+      <c r="FS43" t="n">
+        <v>7.055414547567674</v>
+      </c>
+      <c r="FT43" t="n">
+        <v>0.1916056053556205</v>
+      </c>
+      <c r="FU43" t="n">
+        <v>7.058015808003923</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16135,6 +17587,42 @@
       <c r="FI44" t="n">
         <v>1.421106980462218</v>
       </c>
+      <c r="FJ44" t="n">
+        <v>6.764670982784174</v>
+      </c>
+      <c r="FK44" t="n">
+        <v>6.539233102672244</v>
+      </c>
+      <c r="FL44" t="n">
+        <v>9.408631307284107</v>
+      </c>
+      <c r="FM44" t="n">
+        <v>2.72826928526404</v>
+      </c>
+      <c r="FN44" t="n">
+        <v>0.3640180266899998</v>
+      </c>
+      <c r="FO44" t="n">
+        <v>2.752446623764108</v>
+      </c>
+      <c r="FP44" t="n">
+        <v>6.93718143413444</v>
+      </c>
+      <c r="FQ44" t="n">
+        <v>8.297019802476489</v>
+      </c>
+      <c r="FR44" t="n">
+        <v>10.81503693256692</v>
+      </c>
+      <c r="FS44" t="n">
+        <v>7.143742382220795</v>
+      </c>
+      <c r="FT44" t="n">
+        <v>6.830229539278107</v>
+      </c>
+      <c r="FU44" t="n">
+        <v>9.883576821311445</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16494,6 +17982,42 @@
       <c r="FI45" t="n">
         <v>1.319617012942293</v>
       </c>
+      <c r="FJ45" t="n">
+        <v>11.8315012674621</v>
+      </c>
+      <c r="FK45" t="n">
+        <v>0.3741808920810551</v>
+      </c>
+      <c r="FL45" t="n">
+        <v>11.83741667687489</v>
+      </c>
+      <c r="FM45" t="n">
+        <v>1.182074125880672</v>
+      </c>
+      <c r="FN45" t="n">
+        <v>0.1536802418580728</v>
+      </c>
+      <c r="FO45" t="n">
+        <v>1.19202217085678</v>
+      </c>
+      <c r="FP45" t="n">
+        <v>5.514574650178908</v>
+      </c>
+      <c r="FQ45" t="n">
+        <v>0.1411543523052208</v>
+      </c>
+      <c r="FR45" t="n">
+        <v>5.516380890001209</v>
+      </c>
+      <c r="FS45" t="n">
+        <v>12.59109170630936</v>
+      </c>
+      <c r="FT45" t="n">
+        <v>0.2937212090607966</v>
+      </c>
+      <c r="FU45" t="n">
+        <v>12.59451716046886</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16853,6 +18377,42 @@
       <c r="FI46" t="n">
         <v>1.192409823995364</v>
       </c>
+      <c r="FJ46" t="n">
+        <v>1.431515040949967</v>
+      </c>
+      <c r="FK46" t="n">
+        <v>0.2628454201233674</v>
+      </c>
+      <c r="FL46" t="n">
+        <v>1.455445989154464</v>
+      </c>
+      <c r="FM46" t="n">
+        <v>0.816283362564573</v>
+      </c>
+      <c r="FN46" t="n">
+        <v>0.1959072656871132</v>
+      </c>
+      <c r="FO46" t="n">
+        <v>0.8394630335808285</v>
+      </c>
+      <c r="FP46" t="n">
+        <v>3.091992622913172</v>
+      </c>
+      <c r="FQ46" t="n">
+        <v>0.1402729188749104</v>
+      </c>
+      <c r="FR46" t="n">
+        <v>3.095172833933375</v>
+      </c>
+      <c r="FS46" t="n">
+        <v>2.12925440617476</v>
+      </c>
+      <c r="FT46" t="n">
+        <v>0.2019979098409767</v>
+      </c>
+      <c r="FU46" t="n">
+        <v>2.138814503830276</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -17212,6 +18772,42 @@
       <c r="FI47" t="n">
         <v>1.53641619085053</v>
       </c>
+      <c r="FJ47" t="n">
+        <v>15.37941786195785</v>
+      </c>
+      <c r="FK47" t="n">
+        <v>0.5115044811396212</v>
+      </c>
+      <c r="FL47" t="n">
+        <v>15.38792158177751</v>
+      </c>
+      <c r="FM47" t="n">
+        <v>11.43515488671587</v>
+      </c>
+      <c r="FN47" t="n">
+        <v>0.3817861748691163</v>
+      </c>
+      <c r="FO47" t="n">
+        <v>11.44152647012203</v>
+      </c>
+      <c r="FP47" t="n">
+        <v>15.20467878278714</v>
+      </c>
+      <c r="FQ47" t="n">
+        <v>0.4687279530202096</v>
+      </c>
+      <c r="FR47" t="n">
+        <v>15.21190201065205</v>
+      </c>
+      <c r="FS47" t="n">
+        <v>16.19757077025162</v>
+      </c>
+      <c r="FT47" t="n">
+        <v>0.2793391397791822</v>
+      </c>
+      <c r="FU47" t="n">
+        <v>16.19997929666339</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -17571,6 +19167,42 @@
       <c r="FI48" t="n">
         <v>1.188551314689845</v>
       </c>
+      <c r="FJ48" t="n">
+        <v>2.532847315748743</v>
+      </c>
+      <c r="FK48" t="n">
+        <v>9.882774676337146</v>
+      </c>
+      <c r="FL48" t="n">
+        <v>10.20218363038749</v>
+      </c>
+      <c r="FM48" t="n">
+        <v>0.5262412671987187</v>
+      </c>
+      <c r="FN48" t="n">
+        <v>0.3564804293969701</v>
+      </c>
+      <c r="FO48" t="n">
+        <v>0.6356163684534574</v>
+      </c>
+      <c r="FP48" t="n">
+        <v>2.717391133849206</v>
+      </c>
+      <c r="FQ48" t="n">
+        <v>9.941404662937604</v>
+      </c>
+      <c r="FR48" t="n">
+        <v>10.30610213643353</v>
+      </c>
+      <c r="FS48" t="n">
+        <v>2.791484726323181</v>
+      </c>
+      <c r="FT48" t="n">
+        <v>8.779295943066611</v>
+      </c>
+      <c r="FU48" t="n">
+        <v>9.212405995897134</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -17930,6 +19562,42 @@
       <c r="FI49" t="n">
         <v>1.192666986633151</v>
       </c>
+      <c r="FJ49" t="n">
+        <v>1.358141815172933</v>
+      </c>
+      <c r="FK49" t="n">
+        <v>0.2759773995864318</v>
+      </c>
+      <c r="FL49" t="n">
+        <v>1.38589780113965</v>
+      </c>
+      <c r="FM49" t="n">
+        <v>0.4430507320025405</v>
+      </c>
+      <c r="FN49" t="n">
+        <v>0.1429933850424038</v>
+      </c>
+      <c r="FO49" t="n">
+        <v>0.4655545717677704</v>
+      </c>
+      <c r="FP49" t="n">
+        <v>2.713100895462373</v>
+      </c>
+      <c r="FQ49" t="n">
+        <v>0.1510069043262609</v>
+      </c>
+      <c r="FR49" t="n">
+        <v>2.717300048598413</v>
+      </c>
+      <c r="FS49" t="n">
+        <v>2.067535107593898</v>
+      </c>
+      <c r="FT49" t="n">
+        <v>0.2837617042885123</v>
+      </c>
+      <c r="FU49" t="n">
+        <v>2.086916894836503</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -18289,6 +19957,42 @@
       <c r="FI50" t="n">
         <v>1.190866659666432</v>
       </c>
+      <c r="FJ50" t="n">
+        <v>1.441917118208714</v>
+      </c>
+      <c r="FK50" t="n">
+        <v>0.2731599171688306</v>
+      </c>
+      <c r="FL50" t="n">
+        <v>1.467563053545231</v>
+      </c>
+      <c r="FM50" t="n">
+        <v>0.5217903856239713</v>
+      </c>
+      <c r="FN50" t="n">
+        <v>0.1679017561564508</v>
+      </c>
+      <c r="FO50" t="n">
+        <v>0.5481388567233971</v>
+      </c>
+      <c r="FP50" t="n">
+        <v>3.279089523637096</v>
+      </c>
+      <c r="FQ50" t="n">
+        <v>0.1444446704835581</v>
+      </c>
+      <c r="FR50" t="n">
+        <v>3.282269392791771</v>
+      </c>
+      <c r="FS50" t="n">
+        <v>2.057704666295349</v>
+      </c>
+      <c r="FT50" t="n">
+        <v>0.233489200568482</v>
+      </c>
+      <c r="FU50" t="n">
+        <v>2.070909389730937</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -18647,6 +20351,42 @@
       </c>
       <c r="FI51" t="n">
         <v>1.223766255785051</v>
+      </c>
+      <c r="FJ51" t="n">
+        <v>2.426026652190076</v>
+      </c>
+      <c r="FK51" t="n">
+        <v>7.321318287626557</v>
+      </c>
+      <c r="FL51" t="n">
+        <v>7.712801487518763</v>
+      </c>
+      <c r="FM51" t="n">
+        <v>0.4889848175203712</v>
+      </c>
+      <c r="FN51" t="n">
+        <v>0.3194585633013968</v>
+      </c>
+      <c r="FO51" t="n">
+        <v>0.5840889704762651</v>
+      </c>
+      <c r="FP51" t="n">
+        <v>2.343493614520334</v>
+      </c>
+      <c r="FQ51" t="n">
+        <v>8.041699578500666</v>
+      </c>
+      <c r="FR51" t="n">
+        <v>8.376210027939567</v>
+      </c>
+      <c r="FS51" t="n">
+        <v>2.697096243186959</v>
+      </c>
+      <c r="FT51" t="n">
+        <v>6.042340625102693</v>
+      </c>
+      <c r="FU51" t="n">
+        <v>6.616963682443754</v>
       </c>
     </row>
     <row r="52">
@@ -18897,6 +20637,18 @@
       <c r="FG52" t="inlineStr"/>
       <c r="FH52" t="inlineStr"/>
       <c r="FI52" t="inlineStr"/>
+      <c r="FJ52" t="inlineStr"/>
+      <c r="FK52" t="inlineStr"/>
+      <c r="FL52" t="inlineStr"/>
+      <c r="FM52" t="inlineStr"/>
+      <c r="FN52" t="inlineStr"/>
+      <c r="FO52" t="inlineStr"/>
+      <c r="FP52" t="inlineStr"/>
+      <c r="FQ52" t="inlineStr"/>
+      <c r="FR52" t="inlineStr"/>
+      <c r="FS52" t="inlineStr"/>
+      <c r="FT52" t="inlineStr"/>
+      <c r="FU52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -19256,6 +21008,42 @@
       <c r="FI53" t="n">
         <v>1.534683882793128</v>
       </c>
+      <c r="FJ53" t="n">
+        <v>14.79314580316297</v>
+      </c>
+      <c r="FK53" t="n">
+        <v>8.168992854269355</v>
+      </c>
+      <c r="FL53" t="n">
+        <v>16.89880489877145</v>
+      </c>
+      <c r="FM53" t="n">
+        <v>11.57542493806857</v>
+      </c>
+      <c r="FN53" t="n">
+        <v>0.6980283239900179</v>
+      </c>
+      <c r="FO53" t="n">
+        <v>11.59645230395711</v>
+      </c>
+      <c r="FP53" t="n">
+        <v>15.54915596528659</v>
+      </c>
+      <c r="FQ53" t="n">
+        <v>6.403506688402647</v>
+      </c>
+      <c r="FR53" t="n">
+        <v>16.81609791661624</v>
+      </c>
+      <c r="FS53" t="n">
+        <v>16.36092117188419</v>
+      </c>
+      <c r="FT53" t="n">
+        <v>6.404674085036127</v>
+      </c>
+      <c r="FU53" t="n">
+        <v>17.56984893868305</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -19615,6 +21403,42 @@
       <c r="FI54" t="n">
         <v>1.226969671812089</v>
       </c>
+      <c r="FJ54" t="n">
+        <v>3.747528981618872</v>
+      </c>
+      <c r="FK54" t="n">
+        <v>8.334125534999961</v>
+      </c>
+      <c r="FL54" t="n">
+        <v>9.137922187303399</v>
+      </c>
+      <c r="FM54" t="n">
+        <v>0.9116242547436735</v>
+      </c>
+      <c r="FN54" t="n">
+        <v>0.4356547600113409</v>
+      </c>
+      <c r="FO54" t="n">
+        <v>1.010373125017435</v>
+      </c>
+      <c r="FP54" t="n">
+        <v>3.738709640130689</v>
+      </c>
+      <c r="FQ54" t="n">
+        <v>8.141313812396728</v>
+      </c>
+      <c r="FR54" t="n">
+        <v>8.958735422208196</v>
+      </c>
+      <c r="FS54" t="n">
+        <v>5.331566307910149</v>
+      </c>
+      <c r="FT54" t="n">
+        <v>7.322079052083258</v>
+      </c>
+      <c r="FU54" t="n">
+        <v>9.057507435304656</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -19974,6 +21798,42 @@
       <c r="FI55" t="n">
         <v>1.197294349469238</v>
       </c>
+      <c r="FJ55" t="n">
+        <v>1.449418017012981</v>
+      </c>
+      <c r="FK55" t="n">
+        <v>0.280301552359907</v>
+      </c>
+      <c r="FL55" t="n">
+        <v>1.476272856993996</v>
+      </c>
+      <c r="FM55" t="n">
+        <v>1.281187739748811</v>
+      </c>
+      <c r="FN55" t="n">
+        <v>0.1788931822695058</v>
+      </c>
+      <c r="FO55" t="n">
+        <v>1.293616942972369</v>
+      </c>
+      <c r="FP55" t="n">
+        <v>1.111132178802135</v>
+      </c>
+      <c r="FQ55" t="n">
+        <v>0.1496293620156138</v>
+      </c>
+      <c r="FR55" t="n">
+        <v>1.121161747807505</v>
+      </c>
+      <c r="FS55" t="n">
+        <v>1.969324962777373</v>
+      </c>
+      <c r="FT55" t="n">
+        <v>0.2657787494603426</v>
+      </c>
+      <c r="FU55" t="n">
+        <v>1.987178691683967</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
videre arbeid med ensure-stillwater
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
+++ b/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
@@ -1368,7 +1368,7 @@
         <v>170</v>
       </c>
       <c r="R2" t="n">
-        <v>271.97</v>
+        <v>272.5280651625832</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
@@ -1394,7 +1394,7 @@
         <v>250</v>
       </c>
       <c r="AL2" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9536072144288</v>
       </c>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
@@ -1420,7 +1420,7 @@
         <v>340</v>
       </c>
       <c r="BF2" t="n">
-        <v>271.75</v>
+        <v>272.6194530997479</v>
       </c>
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
@@ -1446,7 +1446,7 @@
         <v>250</v>
       </c>
       <c r="BZ2" t="n">
-        <v>271.98</v>
+        <v>272.8078828624992</v>
       </c>
       <c r="CA2" t="inlineStr"/>
       <c r="CB2" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
         <v>0.6462706246618998</v>
       </c>
       <c r="DY2" t="n">
-        <v>0.7436363950959103</v>
+        <v>0.7436363950959101</v>
       </c>
       <c r="DZ2" t="n">
         <v>0.4210196248262004</v>
@@ -1572,7 +1572,7 @@
         <v>0.7173913043478261</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.3902921326715521</v>
+        <v>0.390292132671552</v>
       </c>
       <c r="EG2" t="n">
         <v>1.321752265861027</v>
@@ -1677,7 +1677,7 @@
         <v>0.366768399617689</v>
       </c>
       <c r="FO2" t="n">
-        <v>0.6512079829558821</v>
+        <v>0.651207982955882</v>
       </c>
       <c r="FP2" t="n">
         <v>1.545508909730039</v>
@@ -1763,7 +1763,7 @@
         <v>170</v>
       </c>
       <c r="R3" t="n">
-        <v>271.97</v>
+        <v>271.8626608054819</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
@@ -1789,7 +1789,7 @@
         <v>250</v>
       </c>
       <c r="AL3" t="n">
-        <v>272.1199999999999</v>
+        <v>272.2772945891784</v>
       </c>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
@@ -1815,7 +1815,7 @@
         <v>340</v>
       </c>
       <c r="BF3" t="n">
-        <v>271.75</v>
+        <v>272.1776682397052</v>
       </c>
       <c r="BG3" t="inlineStr"/>
       <c r="BH3" t="inlineStr"/>
@@ -1841,7 +1841,7 @@
         <v>250</v>
       </c>
       <c r="BZ3" t="n">
-        <v>271.98</v>
+        <v>271.9952168853836</v>
       </c>
       <c r="CA3" t="inlineStr"/>
       <c r="CB3" t="inlineStr"/>
@@ -1893,7 +1893,7 @@
       <c r="DF3" t="inlineStr"/>
       <c r="DG3" t="inlineStr"/>
       <c r="DH3" t="n">
-        <v>0.4076436929804917</v>
+        <v>0.4076436929804916</v>
       </c>
       <c r="DI3" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         <v>0.06324751182594683</v>
       </c>
       <c r="DZ3" t="n">
-        <v>0.0494608246068068</v>
+        <v>0.04946082460680681</v>
       </c>
       <c r="EA3" t="n">
         <v>1.812688821752266</v>
@@ -2057,7 +2057,7 @@
         <v>1.136597562556303</v>
       </c>
       <c r="FJ3" t="n">
-        <v>0.2571986493406551</v>
+        <v>0.257198649340655</v>
       </c>
       <c r="FK3" t="n">
         <v>0.2345041529064142</v>
@@ -2066,13 +2066,13 @@
         <v>0.3480565226410965</v>
       </c>
       <c r="FM3" t="n">
-        <v>0.01437080539401557</v>
+        <v>0.01437080539401558</v>
       </c>
       <c r="FN3" t="n">
         <v>0.01954343965078708</v>
       </c>
       <c r="FO3" t="n">
-        <v>0.02425831983169122</v>
+        <v>0.02425831983169123</v>
       </c>
       <c r="FP3" t="n">
         <v>0.4127929659477516</v>
@@ -2158,7 +2158,7 @@
         <v>170</v>
       </c>
       <c r="R4" t="n">
-        <v>271.97</v>
+        <v>272.6997595190381</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
@@ -2184,7 +2184,7 @@
         <v>250</v>
       </c>
       <c r="AL4" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1281162324649</v>
       </c>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
@@ -2210,7 +2210,7 @@
         <v>340</v>
       </c>
       <c r="BF4" t="n">
-        <v>271.75</v>
+        <v>272.7334468937876</v>
       </c>
       <c r="BG4" t="inlineStr"/>
       <c r="BH4" t="inlineStr"/>
@@ -2236,7 +2236,7 @@
         <v>250</v>
       </c>
       <c r="BZ4" t="n">
-        <v>271.98</v>
+        <v>273.0175751503006</v>
       </c>
       <c r="CA4" t="inlineStr"/>
       <c r="CB4" t="inlineStr"/>
@@ -2288,7 +2288,7 @@
       <c r="DF4" t="inlineStr"/>
       <c r="DG4" t="inlineStr"/>
       <c r="DH4" t="n">
-        <v>0.9975922507294624</v>
+        <v>0.9975922507294627</v>
       </c>
       <c r="DI4" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
         <v>1.412666666666667</v>
       </c>
       <c r="EC4" t="n">
-        <v>7.972966629562706</v>
+        <v>7.972966629562708</v>
       </c>
       <c r="ED4" t="n">
         <v>0.7049700387733521</v>
@@ -2464,7 +2464,7 @@
         <v>12.9571523721344</v>
       </c>
       <c r="FN4" t="n">
-        <v>0.6795468404788301</v>
+        <v>0.6795468404788302</v>
       </c>
       <c r="FO4" t="n">
         <v>12.9749597881116</v>
@@ -2473,7 +2473,7 @@
         <v>13.97812676542665</v>
       </c>
       <c r="FQ4" t="n">
-        <v>7.108740060065507</v>
+        <v>7.108740060065506</v>
       </c>
       <c r="FR4" t="n">
         <v>15.68190718987703</v>
@@ -2553,7 +2553,7 @@
         <v>170</v>
       </c>
       <c r="R5" t="n">
-        <v>271.97</v>
+        <v>272.6462085461245</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
@@ -2579,7 +2579,7 @@
         <v>250</v>
       </c>
       <c r="AL5" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0736873747495</v>
       </c>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
@@ -2605,7 +2605,7 @@
         <v>340</v>
       </c>
       <c r="BF5" t="n">
-        <v>271.75</v>
+        <v>272.6978925593122</v>
       </c>
       <c r="BG5" t="inlineStr"/>
       <c r="BH5" t="inlineStr"/>
@@ -2631,7 +2631,7 @@
         <v>250</v>
       </c>
       <c r="BZ5" t="n">
-        <v>271.98</v>
+        <v>272.9521727325619</v>
       </c>
       <c r="CA5" t="inlineStr"/>
       <c r="CB5" t="inlineStr"/>
@@ -2948,7 +2948,7 @@
         <v>170</v>
       </c>
       <c r="R6" t="n">
-        <v>271.97</v>
+        <v>272.0379041954877</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
         <v>250</v>
       </c>
       <c r="AL6" t="n">
-        <v>272.1199999999999</v>
+        <v>272.4554108216433</v>
       </c>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
@@ -3000,7 +3000,7 @@
         <v>340</v>
       </c>
       <c r="BF6" t="n">
-        <v>271.75</v>
+        <v>272.2940183592992</v>
       </c>
       <c r="BG6" t="inlineStr"/>
       <c r="BH6" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
         <v>250</v>
       </c>
       <c r="BZ6" t="n">
-        <v>271.98</v>
+        <v>272.2092436485875</v>
       </c>
       <c r="CA6" t="inlineStr"/>
       <c r="CB6" t="inlineStr"/>
@@ -3128,7 +3128,7 @@
         <v>0.08753377739745957</v>
       </c>
       <c r="DX6" t="n">
-        <v>0.08668146181368427</v>
+        <v>0.08668146181368426</v>
       </c>
       <c r="DY6" t="n">
         <v>0.105239216428749</v>
@@ -3152,7 +3152,7 @@
         <v>0.8943529411764706</v>
       </c>
       <c r="EF6" t="n">
-        <v>0.3191122499893997</v>
+        <v>0.3191122499893998</v>
       </c>
       <c r="EG6" t="n">
         <v>1.128518321826872</v>
@@ -3254,13 +3254,13 @@
         <v>0.2248298780424435</v>
       </c>
       <c r="FN6" t="n">
-        <v>0.08287363708341197</v>
+        <v>0.08287363708341199</v>
       </c>
       <c r="FO6" t="n">
         <v>0.2396174321371738</v>
       </c>
       <c r="FP6" t="n">
-        <v>0.4971315775308695</v>
+        <v>0.4971315775308694</v>
       </c>
       <c r="FQ6" t="n">
         <v>0.12296873720625</v>
@@ -3343,7 +3343,7 @@
         <v>170</v>
       </c>
       <c r="R7" t="n">
-        <v>271.97</v>
+        <v>272.713955653242</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -3369,7 +3369,7 @@
         <v>250</v>
       </c>
       <c r="AL7" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1425450901803</v>
       </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
@@ -3395,7 +3395,7 @@
         <v>340</v>
       </c>
       <c r="BF7" t="n">
-        <v>271.75</v>
+        <v>272.7428721960049</v>
       </c>
       <c r="BG7" t="inlineStr"/>
       <c r="BH7" t="inlineStr"/>
@@ -3421,7 +3421,7 @@
         <v>250</v>
       </c>
       <c r="BZ7" t="n">
-        <v>271.98</v>
+        <v>273.0349130519103</v>
       </c>
       <c r="CA7" t="inlineStr"/>
       <c r="CB7" t="inlineStr"/>
@@ -3473,7 +3473,7 @@
       <c r="DF7" t="inlineStr"/>
       <c r="DG7" t="inlineStr"/>
       <c r="DH7" t="n">
-        <v>0.8877865747975324</v>
+        <v>0.8877865747975322</v>
       </c>
       <c r="DI7" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
         <v>1.437166666666666</v>
       </c>
       <c r="EC7" t="n">
-        <v>7.883788504415101</v>
+        <v>7.883788504415099</v>
       </c>
       <c r="ED7" t="n">
         <v>0.7059654076950228</v>
@@ -3556,7 +3556,7 @@
         <v>1.4175</v>
       </c>
       <c r="EI7" t="n">
-        <v>7.306551124468012</v>
+        <v>7.306551124468013</v>
       </c>
       <c r="EJ7" t="n">
         <v>0.6894174422612892</v>
@@ -3649,7 +3649,7 @@
         <v>13.08821814370633</v>
       </c>
       <c r="FN7" t="n">
-        <v>0.7235402384326545</v>
+        <v>0.7235402384326546</v>
       </c>
       <c r="FO7" t="n">
         <v>13.10820218999825</v>
@@ -3738,7 +3738,7 @@
         <v>170</v>
       </c>
       <c r="R8" t="n">
-        <v>271.97</v>
+        <v>272.5489650268278</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
@@ -3764,7 +3764,7 @@
         <v>250</v>
       </c>
       <c r="AL8" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9748496993988</v>
       </c>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
@@ -3790,7 +3790,7 @@
         <v>340</v>
       </c>
       <c r="BF8" t="n">
-        <v>271.75</v>
+        <v>272.6333292391234</v>
       </c>
       <c r="BG8" t="inlineStr"/>
       <c r="BH8" t="inlineStr"/>
@@ -3816,7 +3816,7 @@
         <v>250</v>
       </c>
       <c r="BZ8" t="n">
-        <v>271.98</v>
+        <v>272.8334081065356</v>
       </c>
       <c r="CA8" t="inlineStr"/>
       <c r="CB8" t="inlineStr"/>
@@ -3933,7 +3933,7 @@
         <v>0.4957037037037037</v>
       </c>
       <c r="EC8" t="n">
-        <v>0.07256315515673269</v>
+        <v>0.0725631551567327</v>
       </c>
       <c r="ED8" t="n">
         <v>1.439830251591391</v>
@@ -3942,7 +3942,7 @@
         <v>0.6945263157894737</v>
       </c>
       <c r="EF8" t="n">
-        <v>0.3906928232548914</v>
+        <v>0.3906928232548912</v>
       </c>
       <c r="EG8" t="n">
         <v>2.163533273649657</v>
@@ -4056,7 +4056,7 @@
         <v>7.773588806713883</v>
       </c>
       <c r="FR8" t="n">
-        <v>7.864143157876013</v>
+        <v>7.864143157876012</v>
       </c>
       <c r="FS8" t="n">
         <v>1.148490601477886</v>
@@ -4133,7 +4133,7 @@
         <v>170</v>
       </c>
       <c r="R9" t="n">
-        <v>271.97</v>
+        <v>271.794440493891</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
@@ -4159,7 +4159,7 @@
         <v>250</v>
       </c>
       <c r="AL9" t="n">
-        <v>272.1199999999999</v>
+        <v>272.2079559118237</v>
       </c>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
@@ -4185,7 +4185,7 @@
         <v>340</v>
       </c>
       <c r="BF9" t="n">
-        <v>271.75</v>
+        <v>272.1323744262719</v>
       </c>
       <c r="BG9" t="inlineStr"/>
       <c r="BH9" t="inlineStr"/>
@@ -4211,7 +4211,7 @@
         <v>250</v>
       </c>
       <c r="BZ9" t="n">
-        <v>271.98</v>
+        <v>271.9118986359816</v>
       </c>
       <c r="CA9" t="inlineStr"/>
       <c r="CB9" t="inlineStr"/>
@@ -4263,7 +4263,7 @@
       <c r="DF9" t="inlineStr"/>
       <c r="DG9" t="inlineStr"/>
       <c r="DH9" t="n">
-        <v>0.2581230964072965</v>
+        <v>0.2581230964072966</v>
       </c>
       <c r="DI9" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         <v>0.2062287858177964</v>
       </c>
       <c r="DZ9" t="n">
-        <v>0.2778815319883882</v>
+        <v>0.2778815319883881</v>
       </c>
       <c r="EA9" t="n">
         <v>1.201619023526435</v>
@@ -4346,7 +4346,7 @@
         <v>0.8766666666666668</v>
       </c>
       <c r="EI9" t="n">
-        <v>0.4075370927484007</v>
+        <v>0.4075370927484006</v>
       </c>
       <c r="EJ9" t="n">
         <v>1.251564455569462</v>
@@ -4528,7 +4528,7 @@
         <v>170</v>
       </c>
       <c r="R10" t="n">
-        <v>271.97</v>
+        <v>271.8403413278169</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
@@ -4554,7 +4554,7 @@
         <v>250</v>
       </c>
       <c r="AL10" t="n">
-        <v>272.1199999999999</v>
+        <v>272.2546092184369</v>
       </c>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
@@ -4580,7 +4580,7 @@
         <v>340</v>
       </c>
       <c r="BF10" t="n">
-        <v>271.75</v>
+        <v>272.162849570108</v>
       </c>
       <c r="BG10" t="inlineStr"/>
       <c r="BH10" t="inlineStr"/>
@@ -4606,7 +4606,7 @@
         <v>250</v>
       </c>
       <c r="BZ10" t="n">
-        <v>271.98</v>
+        <v>271.9679578511862</v>
       </c>
       <c r="CA10" t="inlineStr"/>
       <c r="CB10" t="inlineStr"/>
@@ -4741,7 +4741,7 @@
         <v>0.7503157894736843</v>
       </c>
       <c r="EI10" t="n">
-        <v>0.08742216227879442</v>
+        <v>0.0874221622787944</v>
       </c>
       <c r="EJ10" t="n">
         <v>1.232598607888631</v>
@@ -4837,7 +4837,7 @@
         <v>0.02862339444644768</v>
       </c>
       <c r="FO10" t="n">
-        <v>0.03641826059280504</v>
+        <v>0.03641826059280503</v>
       </c>
       <c r="FP10" t="n">
         <v>0.3448536940719071</v>
@@ -4846,7 +4846,7 @@
         <v>0.1176040477019546</v>
       </c>
       <c r="FR10" t="n">
-        <v>0.3643552968613523</v>
+        <v>0.3643552968613522</v>
       </c>
       <c r="FS10" t="n">
         <v>0.1925436650309388</v>
@@ -4923,7 +4923,7 @@
         <v>170</v>
       </c>
       <c r="R11" t="n">
-        <v>271.97</v>
+        <v>271.9920822289741</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
@@ -4949,7 +4949,7 @@
         <v>250</v>
       </c>
       <c r="AL11" t="n">
-        <v>272.1199999999999</v>
+        <v>272.4088376753507</v>
       </c>
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
@@ -4975,7 +4975,7 @@
         <v>340</v>
       </c>
       <c r="BF11" t="n">
-        <v>271.75</v>
+        <v>272.2635955782533</v>
       </c>
       <c r="BG11" t="inlineStr"/>
       <c r="BH11" t="inlineStr"/>
@@ -5001,7 +5001,7 @@
         <v>250</v>
       </c>
       <c r="BZ11" t="n">
-        <v>271.98</v>
+        <v>272.1532807550585</v>
       </c>
       <c r="CA11" t="inlineStr"/>
       <c r="CB11" t="inlineStr"/>
@@ -5318,7 +5318,7 @@
         <v>170</v>
       </c>
       <c r="R12" t="n">
-        <v>271.97</v>
+        <v>272.671288383218</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
@@ -5344,7 +5344,7 @@
         <v>250</v>
       </c>
       <c r="AL12" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0991783567134</v>
       </c>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
@@ -5370,7 +5370,7 @@
         <v>340</v>
       </c>
       <c r="BF12" t="n">
-        <v>271.75</v>
+        <v>272.7145439265628</v>
       </c>
       <c r="BG12" t="inlineStr"/>
       <c r="BH12" t="inlineStr"/>
@@ -5396,7 +5396,7 @@
         <v>250</v>
       </c>
       <c r="BZ12" t="n">
-        <v>271.98</v>
+        <v>272.9828030254056</v>
       </c>
       <c r="CA12" t="inlineStr"/>
       <c r="CB12" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
         <v>0.5707272727272727</v>
       </c>
       <c r="EI12" t="n">
-        <v>0.5996599989341055</v>
+        <v>0.5996599989341057</v>
       </c>
       <c r="EJ12" t="n">
         <v>1.729016032694121</v>
@@ -5699,7 +5699,7 @@
         <v>170</v>
       </c>
       <c r="R13" t="n">
-        <v>271.97</v>
+        <v>272.7638787251923</v>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
@@ -5725,7 +5725,7 @@
         <v>250</v>
       </c>
       <c r="AL13" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1932865731463</v>
       </c>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         <v>340</v>
       </c>
       <c r="BF13" t="n">
-        <v>271.75</v>
+        <v>272.7760178421359</v>
       </c>
       <c r="BG13" t="inlineStr"/>
       <c r="BH13" t="inlineStr"/>
@@ -5777,7 +5777,7 @@
         <v>250</v>
       </c>
       <c r="BZ13" t="n">
-        <v>271.98</v>
+        <v>273.0958846725709</v>
       </c>
       <c r="CA13" t="inlineStr"/>
       <c r="CB13" t="inlineStr"/>
@@ -5970,7 +5970,7 @@
         <v>170</v>
       </c>
       <c r="R14" t="n">
-        <v>271.97</v>
+        <v>272.7287827267438</v>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
@@ -5996,7 +5996,7 @@
         <v>250</v>
       </c>
       <c r="AL14" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1576152304609</v>
       </c>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
@@ -6022,7 +6022,7 @@
         <v>340</v>
       </c>
       <c r="BF14" t="n">
-        <v>271.75</v>
+        <v>272.752716400543</v>
       </c>
       <c r="BG14" t="inlineStr"/>
       <c r="BH14" t="inlineStr"/>
@@ -6048,7 +6048,7 @@
         <v>250</v>
       </c>
       <c r="BZ14" t="n">
-        <v>271.98</v>
+        <v>273.0530215269248</v>
       </c>
       <c r="CA14" t="inlineStr"/>
       <c r="CB14" t="inlineStr"/>
@@ -6100,7 +6100,7 @@
       <c r="DF14" t="inlineStr"/>
       <c r="DG14" t="inlineStr"/>
       <c r="DH14" t="n">
-        <v>0.8461845720990009</v>
+        <v>0.846184572099001</v>
       </c>
       <c r="DI14" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v>11.09538118464997</v>
       </c>
       <c r="DZ14" t="n">
-        <v>9.171023925447864</v>
+        <v>9.171023925447862</v>
       </c>
       <c r="EA14" t="n">
         <v>0.7987220447284344</v>
@@ -6351,7 +6351,7 @@
         <v>170</v>
       </c>
       <c r="R15" t="n">
-        <v>271.97</v>
+        <v>272.8</v>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
@@ -6377,7 +6377,7 @@
         <v>250</v>
       </c>
       <c r="AL15" t="n">
-        <v>272.1199999999999</v>
+        <v>273.23</v>
       </c>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
@@ -6403,7 +6403,7 @@
         <v>340</v>
       </c>
       <c r="BF15" t="n">
-        <v>271.75</v>
+        <v>272.8</v>
       </c>
       <c r="BG15" t="inlineStr"/>
       <c r="BH15" t="inlineStr"/>
@@ -6429,7 +6429,7 @@
         <v>250</v>
       </c>
       <c r="BZ15" t="n">
-        <v>271.98</v>
+        <v>273.14</v>
       </c>
       <c r="CA15" t="inlineStr"/>
       <c r="CB15" t="inlineStr"/>
@@ -6626,7 +6626,7 @@
         <v>170</v>
       </c>
       <c r="R16" t="n">
-        <v>271.97</v>
+        <v>272.6335108927532</v>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
@@ -6652,7 +6652,7 @@
         <v>250</v>
       </c>
       <c r="AL16" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0607815631262</v>
       </c>
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
@@ -6678,7 +6678,7 @@
         <v>340</v>
       </c>
       <c r="BF16" t="n">
-        <v>271.75</v>
+        <v>272.6894621501067</v>
       </c>
       <c r="BG16" t="inlineStr"/>
       <c r="BH16" t="inlineStr"/>
@@ -6704,7 +6704,7 @@
         <v>250</v>
       </c>
       <c r="BZ16" t="n">
-        <v>271.98</v>
+        <v>272.9366649427888</v>
       </c>
       <c r="CA16" t="inlineStr"/>
       <c r="CB16" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
         <v>9.820872512715903</v>
       </c>
       <c r="FM16" t="n">
-        <v>0.7758551428006574</v>
+        <v>0.7758551428006575</v>
       </c>
       <c r="FN16" t="n">
         <v>0.4614623654134864</v>
@@ -7021,7 +7021,7 @@
         <v>170</v>
       </c>
       <c r="R17" t="n">
-        <v>271.97</v>
+        <v>272.5431288383218</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
@@ -7047,7 +7047,7 @@
         <v>250</v>
       </c>
       <c r="AL17" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9689178356713</v>
       </c>
       <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
@@ -7073,7 +7073,7 @@
         <v>340</v>
       </c>
       <c r="BF17" t="n">
-        <v>271.75</v>
+        <v>272.6294543926563</v>
       </c>
       <c r="BG17" t="inlineStr"/>
       <c r="BH17" t="inlineStr"/>
@@ -7099,7 +7099,7 @@
         <v>250</v>
       </c>
       <c r="BZ17" t="n">
-        <v>271.98</v>
+        <v>272.8262803025406</v>
       </c>
       <c r="CA17" t="inlineStr"/>
       <c r="CB17" t="inlineStr"/>
@@ -7327,7 +7327,7 @@
         <v>0.4509662203506125</v>
       </c>
       <c r="FN17" t="n">
-        <v>0.3286466067181548</v>
+        <v>0.3286466067181547</v>
       </c>
       <c r="FO17" t="n">
         <v>0.5580135518109526</v>
@@ -7416,7 +7416,7 @@
         <v>170</v>
       </c>
       <c r="R18" t="n">
-        <v>271.97</v>
+        <v>272.5205727584201</v>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
@@ -7442,7 +7442,7 @@
         <v>250</v>
       </c>
       <c r="AL18" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9459919839679</v>
       </c>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
@@ -7468,7 +7468,7 @@
         <v>340</v>
       </c>
       <c r="BF18" t="n">
-        <v>271.75</v>
+        <v>272.6144786346887</v>
       </c>
       <c r="BG18" t="inlineStr"/>
       <c r="BH18" t="inlineStr"/>
@@ -7494,7 +7494,7 @@
         <v>250</v>
       </c>
       <c r="BZ18" t="n">
-        <v>271.98</v>
+        <v>272.7987323033163</v>
       </c>
       <c r="CA18" t="inlineStr"/>
       <c r="CB18" t="inlineStr"/>
@@ -7546,7 +7546,7 @@
       <c r="DF18" t="inlineStr"/>
       <c r="DG18" t="inlineStr"/>
       <c r="DH18" t="n">
-        <v>0.1861584400726204</v>
+        <v>0.1861584400726205</v>
       </c>
       <c r="DI18" t="inlineStr">
         <is>
@@ -7629,7 +7629,7 @@
         <v>0.78</v>
       </c>
       <c r="EI18" t="n">
-        <v>1.29766739358821</v>
+        <v>1.297667393588211</v>
       </c>
       <c r="EJ18" t="n">
         <v>1.38568129330254</v>
@@ -7811,7 +7811,7 @@
         <v>170</v>
       </c>
       <c r="R19" t="n">
-        <v>271.97</v>
+        <v>272.6570133816019</v>
       </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
@@ -7837,7 +7837,7 @@
         <v>250</v>
       </c>
       <c r="AL19" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0846693386773</v>
       </c>
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
@@ -7863,7 +7863,7 @@
         <v>340</v>
       </c>
       <c r="BF19" t="n">
-        <v>271.75</v>
+        <v>272.7050662615554</v>
       </c>
       <c r="BG19" t="inlineStr"/>
       <c r="BH19" t="inlineStr"/>
@@ -7889,7 +7889,7 @@
         <v>250</v>
       </c>
       <c r="BZ19" t="n">
-        <v>271.98</v>
+        <v>272.9653688021203</v>
       </c>
       <c r="CA19" t="inlineStr"/>
       <c r="CB19" t="inlineStr"/>
@@ -7941,7 +7941,7 @@
       <c r="DF19" t="inlineStr"/>
       <c r="DG19" t="inlineStr"/>
       <c r="DH19" t="n">
-        <v>0.4791387731280216</v>
+        <v>0.4791387731280217</v>
       </c>
       <c r="DI19" t="inlineStr">
         <is>
@@ -8114,7 +8114,7 @@
         <v>7.776043143028404</v>
       </c>
       <c r="FM19" t="n">
-        <v>0.5822810218316877</v>
+        <v>0.5822810218316878</v>
       </c>
       <c r="FN19" t="n">
         <v>0.3779381368831495</v>
@@ -8126,7 +8126,7 @@
         <v>1.388163955848753</v>
       </c>
       <c r="FQ19" t="n">
-        <v>8.783250441101025</v>
+        <v>8.783250441101027</v>
       </c>
       <c r="FR19" t="n">
         <v>8.892271221651926</v>
@@ -8135,10 +8135,10 @@
         <v>1.424737970534595</v>
       </c>
       <c r="FT19" t="n">
-        <v>6.51183192928177</v>
+        <v>6.511831929281769</v>
       </c>
       <c r="FU19" t="n">
-        <v>6.66587078781884</v>
+        <v>6.665870787818839</v>
       </c>
     </row>
     <row r="20">
@@ -8206,7 +8206,7 @@
         <v>170</v>
       </c>
       <c r="R20" t="n">
-        <v>271.97</v>
+        <v>272.6905320318056</v>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
@@ -8232,7 +8232,7 @@
         <v>250</v>
       </c>
       <c r="AL20" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1187374749499</v>
       </c>
       <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="inlineStr"/>
@@ -8258,7 +8258,7 @@
         <v>340</v>
       </c>
       <c r="BF20" t="n">
-        <v>271.75</v>
+        <v>272.7273204473463</v>
       </c>
       <c r="BG20" t="inlineStr"/>
       <c r="BH20" t="inlineStr"/>
@@ -8284,7 +8284,7 @@
         <v>250</v>
       </c>
       <c r="BZ20" t="n">
-        <v>271.98</v>
+        <v>273.0063055142543</v>
       </c>
       <c r="CA20" t="inlineStr"/>
       <c r="CB20" t="inlineStr"/>
@@ -8601,7 +8601,7 @@
         <v>170</v>
       </c>
       <c r="R21" t="n">
-        <v>271.97</v>
+        <v>272.5129226194324</v>
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
@@ -8627,7 +8627,7 @@
         <v>250</v>
       </c>
       <c r="AL21" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9382164328657</v>
       </c>
       <c r="AM21" t="inlineStr"/>
       <c r="AN21" t="inlineStr"/>
@@ -8653,7 +8653,7 @@
         <v>340</v>
       </c>
       <c r="BF21" t="n">
-        <v>271.75</v>
+        <v>272.6093994440494</v>
       </c>
       <c r="BG21" t="inlineStr"/>
       <c r="BH21" t="inlineStr"/>
@@ -8679,7 +8679,7 @@
         <v>250</v>
       </c>
       <c r="BZ21" t="n">
-        <v>271.98</v>
+        <v>272.7893891007822</v>
       </c>
       <c r="CA21" t="inlineStr"/>
       <c r="CB21" t="inlineStr"/>
@@ -8731,7 +8731,7 @@
       <c r="DF21" t="inlineStr"/>
       <c r="DG21" t="inlineStr"/>
       <c r="DH21" t="n">
-        <v>0.1174224535824063</v>
+        <v>0.1174224535824064</v>
       </c>
       <c r="DI21" t="inlineStr">
         <is>
@@ -8796,7 +8796,7 @@
         <v>0.7377391304347826</v>
       </c>
       <c r="EC21" t="n">
-        <v>0.1709798984572658</v>
+        <v>0.1709798984572659</v>
       </c>
       <c r="ED21" t="n">
         <v>0.9840240796480667</v>
@@ -8805,7 +8805,7 @@
         <v>1.016235294117647</v>
       </c>
       <c r="EF21" t="n">
-        <v>0.8506673545535686</v>
+        <v>0.8506673545535687</v>
       </c>
       <c r="EG21" t="n">
         <v>1.390820584144645</v>
@@ -8996,7 +8996,7 @@
         <v>170</v>
       </c>
       <c r="R22" t="n">
-        <v>271.97</v>
+        <v>271.7751968453035</v>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
@@ -9022,7 +9022,7 @@
         <v>250</v>
       </c>
       <c r="AL22" t="n">
-        <v>272.1199999999999</v>
+        <v>272.1883967935872</v>
       </c>
       <c r="AM22" t="inlineStr"/>
       <c r="AN22" t="inlineStr"/>
@@ -9048,7 +9048,7 @@
         <v>340</v>
       </c>
       <c r="BF22" t="n">
-        <v>271.75</v>
+        <v>272.1195979054884</v>
       </c>
       <c r="BG22" t="inlineStr"/>
       <c r="BH22" t="inlineStr"/>
@@ -9074,7 +9074,7 @@
         <v>250</v>
       </c>
       <c r="BZ22" t="n">
-        <v>271.98</v>
+        <v>271.8883961471329</v>
       </c>
       <c r="CA22" t="inlineStr"/>
       <c r="CB22" t="inlineStr"/>
@@ -9126,7 +9126,7 @@
       <c r="DF22" t="inlineStr"/>
       <c r="DG22" t="inlineStr"/>
       <c r="DH22" t="n">
-        <v>0.193491096809835</v>
+        <v>0.1934910968098349</v>
       </c>
       <c r="DI22" t="inlineStr">
         <is>
@@ -9182,7 +9182,7 @@
         <v>0.8322659710624521</v>
       </c>
       <c r="DZ22" t="n">
-        <v>0.723296779035464</v>
+        <v>0.7232967790354641</v>
       </c>
       <c r="EA22" t="n">
         <v>1.279664960446719</v>
@@ -9308,7 +9308,7 @@
         <v>0.370049482717691</v>
       </c>
       <c r="FP22" t="n">
-        <v>0.9115630591000866</v>
+        <v>0.9115630591000865</v>
       </c>
       <c r="FQ22" t="n">
         <v>0.1307104290022208</v>
@@ -9391,7 +9391,7 @@
         <v>170</v>
       </c>
       <c r="R23" t="n">
-        <v>271.97</v>
+        <v>271.8154192255479</v>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
@@ -9417,7 +9417,7 @@
         <v>250</v>
       </c>
       <c r="AL23" t="n">
-        <v>272.1199999999999</v>
+        <v>272.2292785571142</v>
       </c>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
@@ -9443,7 +9443,7 @@
         <v>340</v>
       </c>
       <c r="BF23" t="n">
-        <v>271.75</v>
+        <v>272.1463029284375</v>
       </c>
       <c r="BG23" t="inlineStr"/>
       <c r="BH23" t="inlineStr"/>
@@ -9469,7 +9469,7 @@
         <v>250</v>
       </c>
       <c r="BZ23" t="n">
-        <v>271.98</v>
+        <v>271.9375202016937</v>
       </c>
       <c r="CA23" t="inlineStr"/>
       <c r="CB23" t="inlineStr"/>
@@ -9521,7 +9521,7 @@
       <c r="DF23" t="inlineStr"/>
       <c r="DG23" t="inlineStr"/>
       <c r="DH23" t="n">
-        <v>0.2052480797297535</v>
+        <v>0.2052480797297534</v>
       </c>
       <c r="DI23" t="inlineStr">
         <is>
@@ -9571,7 +9571,7 @@
         <v>0.008906733277153822</v>
       </c>
       <c r="DX23" t="n">
-        <v>0.06561264662205639</v>
+        <v>0.0656126466220564</v>
       </c>
       <c r="DY23" t="n">
         <v>0.09534992150607427</v>
@@ -9586,7 +9586,7 @@
         <v>0.884235294117647</v>
       </c>
       <c r="EC23" t="n">
-        <v>0.03639511948224063</v>
+        <v>0.03639511948224062</v>
       </c>
       <c r="ED23" t="n">
         <v>1.915455746367239</v>
@@ -9694,13 +9694,13 @@
         <v>0.3680676948724736</v>
       </c>
       <c r="FM23" t="n">
-        <v>0.02073298622780809</v>
+        <v>0.02073298622780808</v>
       </c>
       <c r="FN23" t="n">
         <v>0.04019064708389952</v>
       </c>
       <c r="FO23" t="n">
-        <v>0.04522327753430794</v>
+        <v>0.04522327753430793</v>
       </c>
       <c r="FP23" t="n">
         <v>0.3942193329484346</v>
@@ -9786,7 +9786,7 @@
         <v>170</v>
       </c>
       <c r="R24" t="n">
-        <v>271.97</v>
+        <v>272.7416381149396</v>
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
@@ -9812,7 +9812,7 @@
         <v>250</v>
       </c>
       <c r="AL24" t="n">
-        <v>272.1199999999999</v>
+        <v>273.1706813627254</v>
       </c>
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr"/>
@@ -9838,7 +9838,7 @@
         <v>340</v>
       </c>
       <c r="BF24" t="n">
-        <v>271.75</v>
+        <v>272.7612515353287</v>
       </c>
       <c r="BG24" t="inlineStr"/>
       <c r="BH24" t="inlineStr"/>
@@ -9864,7 +9864,7 @@
         <v>250</v>
       </c>
       <c r="BZ24" t="n">
-        <v>271.98</v>
+        <v>273.0687219600491</v>
       </c>
       <c r="CA24" t="inlineStr"/>
       <c r="CB24" t="inlineStr"/>
@@ -9963,16 +9963,16 @@
         <v>10.97804000426573</v>
       </c>
       <c r="DW24" t="n">
-        <v>8.80273576061456</v>
+        <v>8.802735760614562</v>
       </c>
       <c r="DX24" t="n">
         <v>11.0432990424374</v>
       </c>
       <c r="DY24" t="n">
-        <v>11.29938977520158</v>
+        <v>11.29938977520157</v>
       </c>
       <c r="DZ24" t="n">
-        <v>8.101973941045543</v>
+        <v>8.101973941045541</v>
       </c>
       <c r="EA24" t="n">
         <v>0.885216878135143</v>
@@ -9981,7 +9981,7 @@
         <v>1.129666666666667</v>
       </c>
       <c r="EC24" t="n">
-        <v>7.010079803575977</v>
+        <v>7.010079803575975</v>
       </c>
       <c r="ED24" t="n">
         <v>0.9019843656043295</v>
@@ -10181,7 +10181,7 @@
         <v>170</v>
       </c>
       <c r="R25" t="n">
-        <v>271.97</v>
+        <v>272.6627707026957</v>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
@@ -10207,7 +10207,7 @@
         <v>250</v>
       </c>
       <c r="AL25" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0905210420842</v>
       </c>
       <c r="AM25" t="inlineStr"/>
       <c r="AN25" t="inlineStr"/>
@@ -10233,7 +10233,7 @@
         <v>340</v>
       </c>
       <c r="BF25" t="n">
-        <v>271.75</v>
+        <v>272.7088887452324</v>
       </c>
       <c r="BG25" t="inlineStr"/>
       <c r="BH25" t="inlineStr"/>
@@ -10259,7 +10259,7 @@
         <v>250</v>
       </c>
       <c r="BZ25" t="n">
-        <v>271.98</v>
+        <v>272.9724002844399</v>
       </c>
       <c r="CA25" t="inlineStr"/>
       <c r="CB25" t="inlineStr"/>
@@ -10385,7 +10385,7 @@
         <v>0.7386666666666667</v>
       </c>
       <c r="EF25" t="n">
-        <v>0.8117143924798389</v>
+        <v>0.8117143924798388</v>
       </c>
       <c r="EG25" t="n">
         <v>2.120569524386549</v>
@@ -10576,7 +10576,7 @@
         <v>170</v>
       </c>
       <c r="R26" t="n">
-        <v>271.97</v>
+        <v>272.0193703536104</v>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
@@ -10602,7 +10602,7 @@
         <v>250</v>
       </c>
       <c r="AL26" t="n">
-        <v>272.1199999999999</v>
+        <v>272.4365731462926</v>
       </c>
       <c r="AM26" t="inlineStr"/>
       <c r="AN26" t="inlineStr"/>
@@ -10628,7 +10628,7 @@
         <v>340</v>
       </c>
       <c r="BF26" t="n">
-        <v>271.75</v>
+        <v>272.2817131036266</v>
       </c>
       <c r="BG26" t="inlineStr"/>
       <c r="BH26" t="inlineStr"/>
@@ -10654,7 +10654,7 @@
         <v>250</v>
       </c>
       <c r="BZ26" t="n">
-        <v>271.98</v>
+        <v>272.1866080548193</v>
       </c>
       <c r="CA26" t="inlineStr"/>
       <c r="CB26" t="inlineStr"/>
@@ -10780,7 +10780,7 @@
         <v>0.9522352941176468</v>
       </c>
       <c r="EF26" t="n">
-        <v>0.4952680952007097</v>
+        <v>0.4952680952007099</v>
       </c>
       <c r="EG26" t="n">
         <v>1.207115628970775</v>
@@ -10789,7 +10789,7 @@
         <v>0.8284210526315788</v>
       </c>
       <c r="EI26" t="n">
-        <v>0.7346269887990021</v>
+        <v>0.7346269887990026</v>
       </c>
       <c r="EJ26" t="n">
         <v>1.316119328152419</v>
@@ -10971,7 +10971,7 @@
         <v>170</v>
       </c>
       <c r="R27" t="n">
-        <v>271.97</v>
+        <v>272.640845562092</v>
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
@@ -10997,7 +10997,7 @@
         <v>250</v>
       </c>
       <c r="AL27" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0682364729458</v>
       </c>
       <c r="AM27" t="inlineStr"/>
       <c r="AN27" t="inlineStr"/>
@@ -11023,7 +11023,7 @@
         <v>340</v>
       </c>
       <c r="BF27" t="n">
-        <v>271.75</v>
+        <v>272.6943318895856</v>
       </c>
       <c r="BG27" t="inlineStr"/>
       <c r="BH27" t="inlineStr"/>
@@ -11049,7 +11049,7 @@
         <v>250</v>
       </c>
       <c r="BZ27" t="n">
-        <v>271.98</v>
+        <v>272.9456228586204</v>
       </c>
       <c r="CA27" t="inlineStr"/>
       <c r="CB27" t="inlineStr"/>
@@ -11175,7 +11175,7 @@
         <v>0.99475</v>
       </c>
       <c r="EF27" t="n">
-        <v>0.8358240368578193</v>
+        <v>0.8358240368578195</v>
       </c>
       <c r="EG27" t="n">
         <v>1.297257227575982</v>
@@ -11268,7 +11268,7 @@
         <v>1.982634154341693</v>
       </c>
       <c r="FK27" t="n">
-        <v>7.556855011428787</v>
+        <v>7.556855011428788</v>
       </c>
       <c r="FL27" t="n">
         <v>7.812611333844695</v>
@@ -11280,7 +11280,7 @@
         <v>0.4229918877081993</v>
       </c>
       <c r="FO27" t="n">
-        <v>0.5993310939233347</v>
+        <v>0.5993310939233348</v>
       </c>
       <c r="FP27" t="n">
         <v>2.051048136397865</v>
@@ -11366,7 +11366,7 @@
         <v>170</v>
       </c>
       <c r="R28" t="n">
-        <v>271.97</v>
+        <v>272.5335858814403</v>
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
@@ -11392,7 +11392,7 @@
         <v>250</v>
       </c>
       <c r="AL28" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9592184368737</v>
       </c>
       <c r="AM28" t="inlineStr"/>
       <c r="AN28" t="inlineStr"/>
@@ -11418,7 +11418,7 @@
         <v>340</v>
       </c>
       <c r="BF28" t="n">
-        <v>271.75</v>
+        <v>272.6231184950547</v>
       </c>
       <c r="BG28" t="inlineStr"/>
       <c r="BH28" t="inlineStr"/>
@@ -11444,7 +11444,7 @@
         <v>250</v>
       </c>
       <c r="BZ28" t="n">
-        <v>271.98</v>
+        <v>272.8146253797918</v>
       </c>
       <c r="CA28" t="inlineStr"/>
       <c r="CB28" t="inlineStr"/>
@@ -11496,7 +11496,7 @@
       <c r="DF28" t="inlineStr"/>
       <c r="DG28" t="inlineStr"/>
       <c r="DH28" t="n">
-        <v>0.4954165952357098</v>
+        <v>0.4954165952357096</v>
       </c>
       <c r="DI28" t="inlineStr">
         <is>
@@ -11552,7 +11552,7 @@
         <v>0.5267586644570371</v>
       </c>
       <c r="DZ28" t="n">
-        <v>0.2156852645063936</v>
+        <v>0.2156852645063937</v>
       </c>
       <c r="EA28" t="n">
         <v>1.74496644295302</v>
@@ -11755,7 +11755,7 @@
         <v>170</v>
       </c>
       <c r="R29" t="n">
-        <v>271.97</v>
+        <v>271.8848225483225</v>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
@@ -11781,7 +11781,7 @@
         <v>250</v>
       </c>
       <c r="AL29" t="n">
-        <v>272.1199999999999</v>
+        <v>272.2998196392786</v>
       </c>
       <c r="AM29" t="inlineStr"/>
       <c r="AN29" t="inlineStr"/>
@@ -11807,7 +11807,7 @@
         <v>340</v>
       </c>
       <c r="BF29" t="n">
-        <v>271.75</v>
+        <v>272.1923821837223</v>
       </c>
       <c r="BG29" t="inlineStr"/>
       <c r="BH29" t="inlineStr"/>
@@ -11833,7 +11833,7 @@
         <v>250</v>
       </c>
       <c r="BZ29" t="n">
-        <v>271.98</v>
+        <v>272.0222832762299</v>
       </c>
       <c r="CA29" t="inlineStr"/>
       <c r="CB29" t="inlineStr"/>
@@ -12018,7 +12018,7 @@
         <v>170</v>
       </c>
       <c r="R30" t="n">
-        <v>271.97</v>
+        <v>272.4326355937682</v>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
@@ -12044,7 +12044,7 @@
         <v>250</v>
       </c>
       <c r="AL30" t="n">
-        <v>272.1199999999999</v>
+        <v>272.8566132264529</v>
       </c>
       <c r="AM30" t="inlineStr"/>
       <c r="AN30" t="inlineStr"/>
@@ -12070,7 +12070,7 @@
         <v>340</v>
       </c>
       <c r="BF30" t="n">
-        <v>271.75</v>
+        <v>272.5560941237313</v>
       </c>
       <c r="BG30" t="inlineStr"/>
       <c r="BH30" t="inlineStr"/>
@@ -12096,7 +12096,7 @@
         <v>250</v>
       </c>
       <c r="BZ30" t="n">
-        <v>271.98</v>
+        <v>272.6913336350119</v>
       </c>
       <c r="CA30" t="inlineStr"/>
       <c r="CB30" t="inlineStr"/>
@@ -12285,7 +12285,7 @@
         <v>170</v>
       </c>
       <c r="R31" t="n">
-        <v>271.97</v>
+        <v>272.4659176417351</v>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
@@ -12311,7 +12311,7 @@
         <v>250</v>
       </c>
       <c r="AL31" t="n">
-        <v>272.1199999999999</v>
+        <v>272.8904408817635</v>
       </c>
       <c r="AM31" t="inlineStr"/>
       <c r="AN31" t="inlineStr"/>
@@ -12337,7 +12337,7 @@
         <v>340</v>
       </c>
       <c r="BF31" t="n">
-        <v>271.75</v>
+        <v>272.578191221152</v>
       </c>
       <c r="BG31" t="inlineStr"/>
       <c r="BH31" t="inlineStr"/>
@@ -12363,7 +12363,7 @@
         <v>250</v>
       </c>
       <c r="BZ31" t="n">
-        <v>271.98</v>
+        <v>272.731981382119</v>
       </c>
       <c r="CA31" t="inlineStr"/>
       <c r="CB31" t="inlineStr"/>
@@ -12415,7 +12415,7 @@
       <c r="DF31" t="inlineStr"/>
       <c r="DG31" t="inlineStr"/>
       <c r="DH31" t="n">
-        <v>0.6259114331506873</v>
+        <v>0.6259114331506874</v>
       </c>
       <c r="DI31" t="inlineStr">
         <is>
@@ -12489,7 +12489,7 @@
         <v>1.018</v>
       </c>
       <c r="EF31" t="n">
-        <v>4.435904015016542</v>
+        <v>4.435904015016543</v>
       </c>
       <c r="EG31" t="n">
         <v>0.9985022466300549</v>
@@ -12674,7 +12674,7 @@
         <v>170</v>
       </c>
       <c r="R32" t="n">
-        <v>271.97</v>
+        <v>272.1737138793716</v>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
@@ -12700,7 +12700,7 @@
         <v>250</v>
       </c>
       <c r="AL32" t="n">
-        <v>272.1199999999999</v>
+        <v>272.5934468937876</v>
       </c>
       <c r="AM32" t="inlineStr"/>
       <c r="AN32" t="inlineStr"/>
@@ -12726,7 +12726,7 @@
         <v>340</v>
       </c>
       <c r="BF32" t="n">
-        <v>271.75</v>
+        <v>272.3841870838451</v>
       </c>
       <c r="BG32" t="inlineStr"/>
       <c r="BH32" t="inlineStr"/>
@@ -12752,7 +12752,7 @@
         <v>250</v>
       </c>
       <c r="BZ32" t="n">
-        <v>271.98</v>
+        <v>272.3751095739867</v>
       </c>
       <c r="CA32" t="inlineStr"/>
       <c r="CB32" t="inlineStr"/>
@@ -12949,7 +12949,7 @@
         <v>170</v>
       </c>
       <c r="R33" t="n">
-        <v>271.97</v>
+        <v>271.6874962828883</v>
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
@@ -12975,7 +12975,7 @@
         <v>250</v>
       </c>
       <c r="AL33" t="n">
-        <v>272.1199999999999</v>
+        <v>272.0992585170341</v>
       </c>
       <c r="AM33" t="inlineStr"/>
       <c r="AN33" t="inlineStr"/>
@@ -13001,7 +13001,7 @@
         <v>340</v>
       </c>
       <c r="BF33" t="n">
-        <v>271.75</v>
+        <v>272.0613704829013</v>
       </c>
       <c r="BG33" t="inlineStr"/>
       <c r="BH33" t="inlineStr"/>
@@ -13027,7 +13027,7 @@
         <v>250</v>
       </c>
       <c r="BZ33" t="n">
-        <v>271.98</v>
+        <v>271.7812864438554</v>
       </c>
       <c r="CA33" t="inlineStr"/>
       <c r="CB33" t="inlineStr"/>
@@ -13162,7 +13162,7 @@
         <v>1.019666666666667</v>
       </c>
       <c r="EI33" t="n">
-        <v>4.433238197348763</v>
+        <v>4.433238197348764</v>
       </c>
       <c r="EJ33" t="n">
         <v>0.9998333611064821</v>
@@ -13344,7 +13344,7 @@
         <v>170</v>
       </c>
       <c r="R34" t="n">
-        <v>271.97</v>
+        <v>272.5656849182236</v>
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
@@ -13370,7 +13370,7 @@
         <v>250</v>
       </c>
       <c r="AL34" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9918436873747</v>
       </c>
       <c r="AM34" t="inlineStr"/>
       <c r="AN34" t="inlineStr"/>
@@ -13396,7 +13396,7 @@
         <v>340</v>
       </c>
       <c r="BF34" t="n">
-        <v>271.75</v>
+        <v>272.6444301506239</v>
       </c>
       <c r="BG34" t="inlineStr"/>
       <c r="BH34" t="inlineStr"/>
@@ -13422,7 +13422,7 @@
         <v>250</v>
       </c>
       <c r="BZ34" t="n">
-        <v>271.98</v>
+        <v>272.8538283017648</v>
       </c>
       <c r="CA34" t="inlineStr"/>
       <c r="CB34" t="inlineStr"/>
@@ -13521,7 +13521,7 @@
         <v>1.126706548840547</v>
       </c>
       <c r="DW34" t="n">
-        <v>0.3364290486630284</v>
+        <v>0.3364290486630283</v>
       </c>
       <c r="DX34" t="n">
         <v>1.405209777908067</v>
@@ -13739,7 +13739,7 @@
         <v>170</v>
       </c>
       <c r="R35" t="n">
-        <v>271.97</v>
+        <v>271.970078220958</v>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
@@ -13765,7 +13765,7 @@
         <v>250</v>
       </c>
       <c r="AL35" t="n">
-        <v>272.1199999999999</v>
+        <v>272.3864729458918</v>
       </c>
       <c r="AM35" t="inlineStr"/>
       <c r="AN35" t="inlineStr"/>
@@ -13791,7 +13791,7 @@
         <v>340</v>
       </c>
       <c r="BF35" t="n">
-        <v>271.75</v>
+        <v>272.2489863598164</v>
       </c>
       <c r="BG35" t="inlineStr"/>
       <c r="BH35" t="inlineStr"/>
@@ -13817,7 +13817,7 @@
         <v>250</v>
       </c>
       <c r="BZ35" t="n">
-        <v>271.98</v>
+        <v>272.1264070075635</v>
       </c>
       <c r="CA35" t="inlineStr"/>
       <c r="CB35" t="inlineStr"/>
@@ -14134,7 +14134,7 @@
         <v>170</v>
       </c>
       <c r="R36" t="n">
-        <v>271.97</v>
+        <v>271.9323007304932</v>
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
@@ -14160,7 +14160,7 @@
         <v>250</v>
       </c>
       <c r="AL36" t="n">
-        <v>272.1199999999999</v>
+        <v>272.3480761523046</v>
       </c>
       <c r="AM36" t="inlineStr"/>
       <c r="AN36" t="inlineStr"/>
@@ -14186,7 +14186,7 @@
         <v>340</v>
       </c>
       <c r="BF36" t="n">
-        <v>271.75</v>
+        <v>272.2239045833603</v>
       </c>
       <c r="BG36" t="inlineStr"/>
       <c r="BH36" t="inlineStr"/>
@@ -14212,7 +14212,7 @@
         <v>250</v>
       </c>
       <c r="BZ36" t="n">
-        <v>271.98</v>
+        <v>272.0802689249467</v>
       </c>
       <c r="CA36" t="inlineStr"/>
       <c r="CB36" t="inlineStr"/>
@@ -14311,7 +14311,7 @@
         <v>9.166790938934399</v>
       </c>
       <c r="DW36" t="n">
-        <v>3.937398401852224</v>
+        <v>3.937398401852225</v>
       </c>
       <c r="DX36" t="n">
         <v>9.169906179949747</v>
@@ -14347,7 +14347,7 @@
         <v>0.8946666666666666</v>
       </c>
       <c r="EI36" t="n">
-        <v>7.598374036343248</v>
+        <v>7.598374036343251</v>
       </c>
       <c r="EJ36" t="n">
         <v>1.092299290005462</v>
@@ -14437,13 +14437,13 @@
         <v>13.00217164285054</v>
       </c>
       <c r="FM36" t="n">
-        <v>5.583599023167512</v>
+        <v>5.583599023167513</v>
       </c>
       <c r="FN36" t="n">
         <v>0.2170766497360541</v>
       </c>
       <c r="FO36" t="n">
-        <v>5.587817134031662</v>
+        <v>5.587817134031663</v>
       </c>
       <c r="FP36" t="n">
         <v>12.98676786739762</v>
@@ -14529,7 +14529,7 @@
         <v>170</v>
       </c>
       <c r="R37" t="n">
-        <v>271.97</v>
+        <v>271.7256681104143</v>
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
@@ -14555,7 +14555,7 @@
         <v>250</v>
       </c>
       <c r="AL37" t="n">
-        <v>272.1199999999999</v>
+        <v>272.1380561122244</v>
       </c>
       <c r="AM37" t="inlineStr"/>
       <c r="AN37" t="inlineStr"/>
@@ -14581,7 +14581,7 @@
         <v>340</v>
       </c>
       <c r="BF37" t="n">
-        <v>271.75</v>
+        <v>272.0867140733079</v>
       </c>
       <c r="BG37" t="inlineStr"/>
       <c r="BH37" t="inlineStr"/>
@@ -14607,7 +14607,7 @@
         <v>250</v>
       </c>
       <c r="BZ37" t="n">
-        <v>271.98</v>
+        <v>271.8279061348503</v>
       </c>
       <c r="CA37" t="inlineStr"/>
       <c r="CB37" t="inlineStr"/>
@@ -14742,7 +14742,7 @@
         <v>0.8220000000000001</v>
       </c>
       <c r="EI37" t="n">
-        <v>2.747164891153741</v>
+        <v>2.747164891153742</v>
       </c>
       <c r="EJ37" t="n">
         <v>1.176109633871957</v>
@@ -14832,7 +14832,7 @@
         <v>5.889124694069777</v>
       </c>
       <c r="FM37" t="n">
-        <v>0.6151270194977739</v>
+        <v>0.6151270194977738</v>
       </c>
       <c r="FN37" t="n">
         <v>0.1694613089260373</v>
@@ -14924,7 +14924,7 @@
         <v>170</v>
       </c>
       <c r="R38" t="n">
-        <v>271.97</v>
+        <v>272.4976223414571</v>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
@@ -14950,7 +14950,7 @@
         <v>250</v>
       </c>
       <c r="AL38" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9226653306613</v>
       </c>
       <c r="AM38" t="inlineStr"/>
       <c r="AN38" t="inlineStr"/>
@@ -14976,7 +14976,7 @@
         <v>340</v>
       </c>
       <c r="BF38" t="n">
-        <v>271.75</v>
+        <v>272.5992410627707</v>
       </c>
       <c r="BG38" t="inlineStr"/>
       <c r="BH38" t="inlineStr"/>
@@ -15002,7 +15002,7 @@
         <v>250</v>
       </c>
       <c r="BZ38" t="n">
-        <v>271.98</v>
+        <v>272.770702695714</v>
       </c>
       <c r="CA38" t="inlineStr"/>
       <c r="CB38" t="inlineStr"/>
@@ -15119,7 +15119,7 @@
         <v>0.831</v>
       </c>
       <c r="EC38" t="n">
-        <v>0.8066488475872474</v>
+        <v>0.8066488475872475</v>
       </c>
       <c r="ED38" t="n">
         <v>1.109542061730886</v>
@@ -15319,7 +15319,7 @@
         <v>170</v>
       </c>
       <c r="R39" t="n">
-        <v>271.97</v>
+        <v>272.5846919645743</v>
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
@@ -15345,7 +15345,7 @@
         <v>250</v>
       </c>
       <c r="AL39" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0111623246493</v>
       </c>
       <c r="AM39" t="inlineStr"/>
       <c r="AN39" t="inlineStr"/>
@@ -15371,7 +15371,7 @@
         <v>340</v>
       </c>
       <c r="BF39" t="n">
-        <v>271.75</v>
+        <v>272.6570495830371</v>
       </c>
       <c r="BG39" t="inlineStr"/>
       <c r="BH39" t="inlineStr"/>
@@ -15397,7 +15397,7 @@
         <v>250</v>
       </c>
       <c r="BZ39" t="n">
-        <v>271.98</v>
+        <v>272.8770418255866</v>
       </c>
       <c r="CA39" t="inlineStr"/>
       <c r="CB39" t="inlineStr"/>
@@ -15449,7 +15449,7 @@
       <c r="DF39" t="inlineStr"/>
       <c r="DG39" t="inlineStr"/>
       <c r="DH39" t="n">
-        <v>0.5416943107967015</v>
+        <v>0.5416943107967014</v>
       </c>
       <c r="DI39" t="inlineStr">
         <is>
@@ -15514,7 +15514,7 @@
         <v>0.8938333333333335</v>
       </c>
       <c r="EC39" t="n">
-        <v>3.518900338963616</v>
+        <v>3.518900338963615</v>
       </c>
       <c r="ED39" t="n">
         <v>1.107011070110701</v>
@@ -15714,7 +15714,7 @@
         <v>170</v>
       </c>
       <c r="R40" t="n">
-        <v>271.97</v>
+        <v>272.5969164134721</v>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
@@ -15740,7 +15740,7 @@
         <v>250</v>
       </c>
       <c r="AL40" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0235871743487</v>
       </c>
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" t="inlineStr"/>
@@ -15766,7 +15766,7 @@
         <v>340</v>
       </c>
       <c r="BF40" t="n">
-        <v>271.75</v>
+        <v>272.665165815502</v>
       </c>
       <c r="BG40" t="inlineStr"/>
       <c r="BH40" t="inlineStr"/>
@@ -15792,7 +15792,7 @@
         <v>250</v>
       </c>
       <c r="BZ40" t="n">
-        <v>271.98</v>
+        <v>272.8919716853061</v>
       </c>
       <c r="CA40" t="inlineStr"/>
       <c r="CB40" t="inlineStr"/>
@@ -15844,7 +15844,7 @@
       <c r="DF40" t="inlineStr"/>
       <c r="DG40" t="inlineStr"/>
       <c r="DH40" t="n">
-        <v>0.2967343972161288</v>
+        <v>0.2967343972161287</v>
       </c>
       <c r="DI40" t="inlineStr">
         <is>
@@ -15900,7 +15900,7 @@
         <v>8.916003516550758</v>
       </c>
       <c r="DZ40" t="n">
-        <v>5.378123272938971</v>
+        <v>5.378123272938972</v>
       </c>
       <c r="EA40" t="n">
         <v>1.211387038158692</v>
@@ -15918,7 +15918,7 @@
         <v>0.8983636363636365</v>
       </c>
       <c r="EF40" t="n">
-        <v>5.260393748791476</v>
+        <v>5.260393748791475</v>
       </c>
       <c r="EG40" t="n">
         <v>1.217779581895677</v>
@@ -16023,7 +16023,7 @@
         <v>0.4122503996461332</v>
       </c>
       <c r="FO40" t="n">
-        <v>1.472014525229466</v>
+        <v>1.472014525229467</v>
       </c>
       <c r="FP40" t="n">
         <v>6.340710204283535</v>
@@ -16109,7 +16109,7 @@
         <v>170</v>
       </c>
       <c r="R41" t="n">
-        <v>271.97</v>
+        <v>272.4792462344043</v>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
@@ -16135,7 +16135,7 @@
         <v>250</v>
       </c>
       <c r="AL41" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9039879759518</v>
       </c>
       <c r="AM41" t="inlineStr"/>
       <c r="AN41" t="inlineStr"/>
@@ -16161,7 +16161,7 @@
         <v>340</v>
       </c>
       <c r="BF41" t="n">
-        <v>271.75</v>
+        <v>272.5870405326783</v>
       </c>
       <c r="BG41" t="inlineStr"/>
       <c r="BH41" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
         <v>250</v>
       </c>
       <c r="BZ41" t="n">
-        <v>271.98</v>
+        <v>272.748259745297</v>
       </c>
       <c r="CA41" t="inlineStr"/>
       <c r="CB41" t="inlineStr"/>
@@ -16239,7 +16239,7 @@
       <c r="DF41" t="inlineStr"/>
       <c r="DG41" t="inlineStr"/>
       <c r="DH41" t="n">
-        <v>0.5291126160983808</v>
+        <v>0.5291126160983809</v>
       </c>
       <c r="DI41" t="inlineStr">
         <is>
@@ -16406,7 +16406,7 @@
         <v>6.922230949607161</v>
       </c>
       <c r="FK41" t="n">
-        <v>9.767271637381242</v>
+        <v>9.76727163738124</v>
       </c>
       <c r="FL41" t="n">
         <v>11.97150268588248</v>
@@ -16424,7 +16424,7 @@
         <v>6.667747990662222</v>
       </c>
       <c r="FQ41" t="n">
-        <v>7.231325106161351</v>
+        <v>7.23132510616135</v>
       </c>
       <c r="FR41" t="n">
         <v>9.836204860512998</v>
@@ -16504,7 +16504,7 @@
         <v>170</v>
       </c>
       <c r="R42" t="n">
-        <v>271.97</v>
+        <v>272.2353881957463</v>
       </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
@@ -16530,7 +16530,7 @@
         <v>250</v>
       </c>
       <c r="AL42" t="n">
-        <v>272.1199999999999</v>
+        <v>272.656132264529</v>
       </c>
       <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
@@ -16556,7 +16556,7 @@
         <v>340</v>
       </c>
       <c r="BF42" t="n">
-        <v>271.75</v>
+        <v>272.4251347857004</v>
       </c>
       <c r="BG42" t="inlineStr"/>
       <c r="BH42" t="inlineStr"/>
@@ -16582,7 +16582,7 @@
         <v>250</v>
       </c>
       <c r="BZ42" t="n">
-        <v>271.98</v>
+        <v>272.4504331243131</v>
       </c>
       <c r="CA42" t="inlineStr"/>
       <c r="CB42" t="inlineStr"/>
@@ -16899,7 +16899,7 @@
         <v>170</v>
       </c>
       <c r="R43" t="n">
-        <v>271.97</v>
+        <v>271.7081595448962</v>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
@@ -16925,7 +16925,7 @@
         <v>250</v>
       </c>
       <c r="AL43" t="n">
-        <v>272.1199999999999</v>
+        <v>272.1202605210421</v>
       </c>
       <c r="AM43" t="inlineStr"/>
       <c r="AN43" t="inlineStr"/>
@@ -16951,7 +16951,7 @@
         <v>340</v>
       </c>
       <c r="BF43" t="n">
-        <v>271.75</v>
+        <v>272.0750895339065</v>
       </c>
       <c r="BG43" t="inlineStr"/>
       <c r="BH43" t="inlineStr"/>
@@ -16977,7 +16977,7 @@
         <v>250</v>
       </c>
       <c r="BZ43" t="n">
-        <v>271.98</v>
+        <v>271.8065227228651</v>
       </c>
       <c r="CA43" t="inlineStr"/>
       <c r="CB43" t="inlineStr"/>
@@ -17029,7 +17029,7 @@
       <c r="DF43" t="inlineStr"/>
       <c r="DG43" t="inlineStr"/>
       <c r="DH43" t="n">
-        <v>0.5131387234291755</v>
+        <v>0.5131387234291754</v>
       </c>
       <c r="DI43" t="inlineStr">
         <is>
@@ -17082,10 +17082,10 @@
         <v>4.585159998814004</v>
       </c>
       <c r="DY43" t="n">
-        <v>4.981553392314504</v>
+        <v>4.981553392314505</v>
       </c>
       <c r="DZ43" t="n">
-        <v>3.290170790476471</v>
+        <v>3.290170790476472</v>
       </c>
       <c r="EA43" t="n">
         <v>1.112966054535337</v>
@@ -17193,7 +17193,7 @@
         <v>1.418016365693152</v>
       </c>
       <c r="FJ43" t="n">
-        <v>6.487510310209787</v>
+        <v>6.487510310209788</v>
       </c>
       <c r="FK43" t="n">
         <v>0.2439363214032747</v>
@@ -17294,7 +17294,7 @@
         <v>170</v>
       </c>
       <c r="R44" t="n">
-        <v>271.97</v>
+        <v>272.4865809037429</v>
       </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
@@ -17320,7 +17320,7 @@
         <v>250</v>
       </c>
       <c r="AL44" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9114428857715</v>
       </c>
       <c r="AM44" t="inlineStr"/>
       <c r="AN44" t="inlineStr"/>
@@ -17346,7 +17346,7 @@
         <v>340</v>
       </c>
       <c r="BF44" t="n">
-        <v>271.75</v>
+        <v>272.5919102721572</v>
       </c>
       <c r="BG44" t="inlineStr"/>
       <c r="BH44" t="inlineStr"/>
@@ -17372,7 +17372,7 @@
         <v>250</v>
       </c>
       <c r="BZ44" t="n">
-        <v>271.98</v>
+        <v>272.7572176611287</v>
       </c>
       <c r="CA44" t="inlineStr"/>
       <c r="CB44" t="inlineStr"/>
@@ -17424,7 +17424,7 @@
       <c r="DF44" t="inlineStr"/>
       <c r="DG44" t="inlineStr"/>
       <c r="DH44" t="n">
-        <v>0.5101775793707777</v>
+        <v>0.5101775793707778</v>
       </c>
       <c r="DI44" t="inlineStr">
         <is>
@@ -17498,7 +17498,7 @@
         <v>0.9389565217391305</v>
       </c>
       <c r="EF44" t="n">
-        <v>3.301170235629682</v>
+        <v>3.301170235629681</v>
       </c>
       <c r="EG44" t="n">
         <v>1.075168287210172</v>
@@ -17507,7 +17507,7 @@
         <v>0.9300869565217391</v>
       </c>
       <c r="EI44" t="n">
-        <v>3.649290058400059</v>
+        <v>3.649290058400058</v>
       </c>
       <c r="EJ44" t="n">
         <v>1.110494169905608</v>
@@ -17597,7 +17597,7 @@
         <v>9.407223934465888</v>
       </c>
       <c r="FM44" t="n">
-        <v>3.056175912376234</v>
+        <v>3.056175912376233</v>
       </c>
       <c r="FN44" t="n">
         <v>0.3749609915580815</v>
@@ -17689,7 +17689,7 @@
         <v>170</v>
       </c>
       <c r="R45" t="n">
-        <v>271.97</v>
+        <v>271.9541470036848</v>
       </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr"/>
@@ -17715,7 +17715,7 @@
         <v>250</v>
       </c>
       <c r="AL45" t="n">
-        <v>272.1199999999999</v>
+        <v>272.3702805611222</v>
       </c>
       <c r="AM45" t="inlineStr"/>
       <c r="AN45" t="inlineStr"/>
@@ -17741,7 +17741,7 @@
         <v>340</v>
       </c>
       <c r="BF45" t="n">
-        <v>271.75</v>
+        <v>272.238409076217</v>
       </c>
       <c r="BG45" t="inlineStr"/>
       <c r="BH45" t="inlineStr"/>
@@ -17767,7 +17767,7 @@
         <v>250</v>
       </c>
       <c r="BZ45" t="n">
-        <v>271.98</v>
+        <v>272.1069500290904</v>
       </c>
       <c r="CA45" t="inlineStr"/>
       <c r="CB45" t="inlineStr"/>
@@ -18084,7 +18084,7 @@
         <v>170</v>
       </c>
       <c r="R46" t="n">
-        <v>271.97</v>
+        <v>272.1841243777878</v>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr"/>
@@ -18110,7 +18110,7 @@
         <v>250</v>
       </c>
       <c r="AL46" t="n">
-        <v>272.1199999999999</v>
+        <v>272.6040280561122</v>
       </c>
       <c r="AM46" t="inlineStr"/>
       <c r="AN46" t="inlineStr"/>
@@ -18136,7 +18136,7 @@
         <v>340</v>
       </c>
       <c r="BF46" t="n">
-        <v>271.75</v>
+        <v>272.3910989721379</v>
       </c>
       <c r="BG46" t="inlineStr"/>
       <c r="BH46" t="inlineStr"/>
@@ -18162,7 +18162,7 @@
         <v>250</v>
       </c>
       <c r="BZ46" t="n">
-        <v>271.98</v>
+        <v>272.3878240351671</v>
       </c>
       <c r="CA46" t="inlineStr"/>
       <c r="CB46" t="inlineStr"/>
@@ -18402,7 +18402,7 @@
         <v>0.1418289068710316</v>
       </c>
       <c r="FR46" t="n">
-        <v>1.469652975444205</v>
+        <v>1.469652975444206</v>
       </c>
       <c r="FS46" t="n">
         <v>2.136300397810691</v>
@@ -18479,7 +18479,7 @@
         <v>170</v>
       </c>
       <c r="R47" t="n">
-        <v>271.97</v>
+        <v>271.9106121921262</v>
       </c>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
@@ -18505,7 +18505,7 @@
         <v>250</v>
       </c>
       <c r="AL47" t="n">
-        <v>272.1199999999999</v>
+        <v>272.3260320641282</v>
       </c>
       <c r="AM47" t="inlineStr"/>
       <c r="AN47" t="inlineStr"/>
@@ -18531,7 +18531,7 @@
         <v>340</v>
       </c>
       <c r="BF47" t="n">
-        <v>271.75</v>
+        <v>272.2095048160838</v>
       </c>
       <c r="BG47" t="inlineStr"/>
       <c r="BH47" t="inlineStr"/>
@@ -18557,7 +18557,7 @@
         <v>250</v>
       </c>
       <c r="BZ47" t="n">
-        <v>271.98</v>
+        <v>272.0537804641541</v>
       </c>
       <c r="CA47" t="inlineStr"/>
       <c r="CB47" t="inlineStr"/>
@@ -18665,7 +18665,7 @@
         <v>11.4342895343131</v>
       </c>
       <c r="DZ47" t="n">
-        <v>7.495630639989661</v>
+        <v>7.495630639989662</v>
       </c>
       <c r="EA47" t="n">
         <v>0.981675392670157</v>
@@ -18776,7 +18776,7 @@
         <v>15.37291571150778</v>
       </c>
       <c r="FK47" t="n">
-        <v>0.5112749152302906</v>
+        <v>0.5112749152302904</v>
       </c>
       <c r="FL47" t="n">
         <v>15.38141539365173</v>
@@ -18803,7 +18803,7 @@
         <v>16.18599694658085</v>
       </c>
       <c r="FT47" t="n">
-        <v>0.2793154711966758</v>
+        <v>0.2793154711966759</v>
       </c>
       <c r="FU47" t="n">
         <v>16.188406786561</v>
@@ -18874,7 +18874,7 @@
         <v>170</v>
       </c>
       <c r="R48" t="n">
-        <v>271.97</v>
+        <v>272.5043260714978</v>
       </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
@@ -18900,7 +18900,7 @@
         <v>250</v>
       </c>
       <c r="AL48" t="n">
-        <v>272.1199999999999</v>
+        <v>272.9294789579158</v>
       </c>
       <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
@@ -18926,7 +18926,7 @@
         <v>340</v>
       </c>
       <c r="BF48" t="n">
-        <v>271.75</v>
+        <v>272.6036918999289</v>
       </c>
       <c r="BG48" t="inlineStr"/>
       <c r="BH48" t="inlineStr"/>
@@ -18952,7 +18952,7 @@
         <v>250</v>
       </c>
       <c r="BZ48" t="n">
-        <v>271.98</v>
+        <v>272.7788900381408</v>
       </c>
       <c r="CA48" t="inlineStr"/>
       <c r="CB48" t="inlineStr"/>
@@ -19004,7 +19004,7 @@
       <c r="DF48" t="inlineStr"/>
       <c r="DG48" t="inlineStr"/>
       <c r="DH48" t="n">
-        <v>0.174444538861642</v>
+        <v>0.1744445388616421</v>
       </c>
       <c r="DI48" t="inlineStr">
         <is>
@@ -19051,7 +19051,7 @@
         <v>1.305487673084401</v>
       </c>
       <c r="DW48" t="n">
-        <v>0.2936795412862166</v>
+        <v>0.2936795412862165</v>
       </c>
       <c r="DX48" t="n">
         <v>1.566092310818048</v>
@@ -19177,7 +19177,7 @@
         <v>10.20262775502309</v>
       </c>
       <c r="FM48" t="n">
-        <v>0.5230325975711334</v>
+        <v>0.5230325975711333</v>
       </c>
       <c r="FN48" t="n">
         <v>0.3562622527893183</v>
@@ -19269,7 +19269,7 @@
         <v>170</v>
       </c>
       <c r="R49" t="n">
-        <v>271.97</v>
+        <v>271.6520848147908</v>
       </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
@@ -19295,7 +19295,7 @@
         <v>250</v>
       </c>
       <c r="AL49" t="n">
-        <v>272.1199999999999</v>
+        <v>272.0632665330662</v>
       </c>
       <c r="AM49" t="inlineStr"/>
       <c r="AN49" t="inlineStr"/>
@@ -19321,7 +19321,7 @@
         <v>340</v>
       </c>
       <c r="BF49" t="n">
-        <v>271.75</v>
+        <v>272.0378595901481</v>
       </c>
       <c r="BG49" t="inlineStr"/>
       <c r="BH49" t="inlineStr"/>
@@ -19347,7 +19347,7 @@
         <v>250</v>
       </c>
       <c r="BZ49" t="n">
-        <v>271.98</v>
+        <v>271.7380380115069</v>
       </c>
       <c r="CA49" t="inlineStr"/>
       <c r="CB49" t="inlineStr"/>
@@ -19399,7 +19399,7 @@
       <c r="DF49" t="inlineStr"/>
       <c r="DG49" t="inlineStr"/>
       <c r="DH49" t="n">
-        <v>0.1677555410992942</v>
+        <v>0.1677555410992941</v>
       </c>
       <c r="DI49" t="inlineStr">
         <is>
@@ -19664,7 +19664,7 @@
         <v>170</v>
       </c>
       <c r="R50" t="n">
-        <v>271.97</v>
+        <v>271.7479875880794</v>
       </c>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
@@ -19690,7 +19690,7 @@
         <v>250</v>
       </c>
       <c r="AL50" t="n">
-        <v>272.1199999999999</v>
+        <v>272.1607414829659</v>
       </c>
       <c r="AM50" t="inlineStr"/>
       <c r="AN50" t="inlineStr"/>
@@ -19716,7 +19716,7 @@
         <v>340</v>
       </c>
       <c r="BF50" t="n">
-        <v>271.75</v>
+        <v>272.1015327429052</v>
       </c>
       <c r="BG50" t="inlineStr"/>
       <c r="BH50" t="inlineStr"/>
@@ -19742,7 +19742,7 @@
         <v>250</v>
       </c>
       <c r="BZ50" t="n">
-        <v>271.98</v>
+        <v>271.8551651690478</v>
       </c>
       <c r="CA50" t="inlineStr"/>
       <c r="CB50" t="inlineStr"/>
@@ -19961,7 +19961,7 @@
         <v>1.441917118208714</v>
       </c>
       <c r="FK50" t="n">
-        <v>0.2731599171688306</v>
+        <v>0.2731599171688305</v>
       </c>
       <c r="FL50" t="n">
         <v>1.467563053545231</v>
@@ -20059,7 +20059,7 @@
         <v>170</v>
       </c>
       <c r="R51" t="n">
-        <v>271.97</v>
+        <v>272.4473837998578</v>
       </c>
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr"/>
@@ -20085,7 +20085,7 @@
         <v>250</v>
       </c>
       <c r="AL51" t="n">
-        <v>272.1199999999999</v>
+        <v>272.8716032064128</v>
       </c>
       <c r="AM51" t="inlineStr"/>
       <c r="AN51" t="inlineStr"/>
@@ -20111,7 +20111,7 @@
         <v>340</v>
       </c>
       <c r="BF51" t="n">
-        <v>271.75</v>
+        <v>272.5658859654794</v>
       </c>
       <c r="BG51" t="inlineStr"/>
       <c r="BH51" t="inlineStr"/>
@@ -20137,7 +20137,7 @@
         <v>250</v>
       </c>
       <c r="BZ51" t="n">
-        <v>271.98</v>
+        <v>272.7093457883509</v>
       </c>
       <c r="CA51" t="inlineStr"/>
       <c r="CB51" t="inlineStr"/>
@@ -20440,7 +20440,7 @@
         <v>170</v>
       </c>
       <c r="R52" t="n">
-        <v>271.97</v>
+        <v>271.58</v>
       </c>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
@@ -20466,7 +20466,7 @@
         <v>250</v>
       </c>
       <c r="AL52" t="n">
-        <v>272.1199999999999</v>
+        <v>271.99</v>
       </c>
       <c r="AM52" t="inlineStr"/>
       <c r="AN52" t="inlineStr"/>
@@ -20492,7 +20492,7 @@
         <v>340</v>
       </c>
       <c r="BF52" t="n">
-        <v>271.75</v>
+        <v>271.99</v>
       </c>
       <c r="BG52" t="inlineStr"/>
       <c r="BH52" t="inlineStr"/>
@@ -20518,7 +20518,7 @@
         <v>250</v>
       </c>
       <c r="BZ52" t="n">
-        <v>271.98</v>
+        <v>271.65</v>
       </c>
       <c r="CA52" t="inlineStr"/>
       <c r="CB52" t="inlineStr"/>
@@ -20715,7 +20715,7 @@
         <v>170</v>
       </c>
       <c r="R53" t="n">
-        <v>271.97</v>
+        <v>272.575227875105</v>
       </c>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr"/>
@@ -20741,7 +20741,7 @@
         <v>250</v>
       </c>
       <c r="AL53" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0015430861723</v>
       </c>
       <c r="AM53" t="inlineStr"/>
       <c r="AN53" t="inlineStr"/>
@@ -20767,7 +20767,7 @@
         <v>340</v>
       </c>
       <c r="BF53" t="n">
-        <v>271.75</v>
+        <v>272.6507660482255</v>
       </c>
       <c r="BG53" t="inlineStr"/>
       <c r="BH53" t="inlineStr"/>
@@ -20793,7 +20793,7 @@
         <v>250</v>
       </c>
       <c r="BZ53" t="n">
-        <v>271.98</v>
+        <v>272.8654832245135</v>
       </c>
       <c r="CA53" t="inlineStr"/>
       <c r="CB53" t="inlineStr"/>
@@ -21110,7 +21110,7 @@
         <v>170</v>
       </c>
       <c r="R54" t="n">
-        <v>271.97</v>
+        <v>272.611428017325</v>
       </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr"/>
@@ -21136,7 +21136,7 @@
         <v>250</v>
       </c>
       <c r="AL54" t="n">
-        <v>272.1199999999999</v>
+        <v>273.0383366733466</v>
       </c>
       <c r="AM54" t="inlineStr"/>
       <c r="AN54" t="inlineStr"/>
@@ -21162,7 +21162,7 @@
         <v>340</v>
       </c>
       <c r="BF54" t="n">
-        <v>271.75</v>
+        <v>272.6748005688797</v>
       </c>
       <c r="BG54" t="inlineStr"/>
       <c r="BH54" t="inlineStr"/>
@@ -21188,7 +21188,7 @@
         <v>250</v>
       </c>
       <c r="BZ54" t="n">
-        <v>271.98</v>
+        <v>272.9096948736182</v>
       </c>
       <c r="CA54" t="inlineStr"/>
       <c r="CB54" t="inlineStr"/>
@@ -21287,7 +21287,7 @@
         <v>2.413316474631636</v>
       </c>
       <c r="DW54" t="n">
-        <v>0.5050356543704714</v>
+        <v>0.5050356543704715</v>
       </c>
       <c r="DX54" t="n">
         <v>2.435212839205118</v>
@@ -21314,7 +21314,7 @@
         <v>0.9616842105263159</v>
       </c>
       <c r="EF54" t="n">
-        <v>4.056410637229751</v>
+        <v>4.05641063722975</v>
       </c>
       <c r="EG54" t="n">
         <v>1.293382194438456</v>
@@ -21505,7 +21505,7 @@
         <v>170</v>
       </c>
       <c r="R55" t="n">
-        <v>271.97</v>
+        <v>271.6622587109703</v>
       </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr"/>
@@ -21531,7 +21531,7 @@
         <v>250</v>
       </c>
       <c r="AL55" t="n">
-        <v>272.1199999999999</v>
+        <v>272.0736072144289</v>
       </c>
       <c r="AM55" t="inlineStr"/>
       <c r="AN55" t="inlineStr"/>
@@ -21557,7 +21557,7 @@
         <v>340</v>
       </c>
       <c r="BF55" t="n">
-        <v>271.75</v>
+        <v>272.0446143900705</v>
       </c>
       <c r="BG55" t="inlineStr"/>
       <c r="BH55" t="inlineStr"/>
@@ -21583,7 +21583,7 @@
         <v>250</v>
       </c>
       <c r="BZ55" t="n">
-        <v>271.98</v>
+        <v>271.7504635076605</v>
       </c>
       <c r="CA55" t="inlineStr"/>
       <c r="CB55" t="inlineStr"/>

</xml_diff>

<commit_message>
restarter - claude fikset qt browser
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
+++ b/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
@@ -2113,7 +2113,7 @@
         <v>0.2</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7000000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="J4" t="n">
         <v>40</v>
@@ -3274,7 +3274,7 @@
         <v>0.2</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7000000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="J7" t="n">
         <v>40</v>

</xml_diff>

<commit_message>
claude lagrer fft todelt i parquet tror æ
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
+++ b/waveprocessed/PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof/meta.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FU55"/>
+  <dimension ref="A1:FW55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1244,60 +1244,70 @@
       </c>
       <c r="FJ1" t="inlineStr">
         <is>
+          <t>in_position</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>out_position</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
           <t>Probe 9373/170 Swell Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="FM1" t="inlineStr">
         <is>
           <t>Probe 9373/170 Wind Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="FN1" t="inlineStr">
         <is>
           <t>Probe 9373/170 Total Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FM1" t="inlineStr">
+      <c r="FO1" t="inlineStr">
         <is>
           <t>Probe 12545 Swell Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FN1" t="inlineStr">
+      <c r="FP1" t="inlineStr">
         <is>
           <t>Probe 12545 Wind Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FO1" t="inlineStr">
+      <c r="FQ1" t="inlineStr">
         <is>
           <t>Probe 12545 Total Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FP1" t="inlineStr">
+      <c r="FR1" t="inlineStr">
         <is>
           <t>Probe 9373/340 Swell Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FQ1" t="inlineStr">
+      <c r="FS1" t="inlineStr">
         <is>
           <t>Probe 9373/340 Wind Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FR1" t="inlineStr">
+      <c r="FT1" t="inlineStr">
         <is>
           <t>Probe 9373/340 Total Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FS1" t="inlineStr">
+      <c r="FU1" t="inlineStr">
         <is>
           <t>Probe 8804 Swell Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FT1" t="inlineStr">
+      <c r="FV1" t="inlineStr">
         <is>
           <t>Probe 8804 Wind Amplitude (PSD)</t>
         </is>
       </c>
-      <c r="FU1" t="inlineStr">
+      <c r="FW1" t="inlineStr">
         <is>
           <t>Probe 8804 Total Amplitude (PSD)</t>
         </is>
@@ -1653,40 +1663,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ2" t="n">
+      <c r="FJ2" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK2" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL2" t="n">
         <v>11.23363225321726</v>
       </c>
-      <c r="FK2" t="n">
+      <c r="FM2" t="n">
         <v>6.602376612422562</v>
       </c>
-      <c r="FL2" t="n">
+      <c r="FN2" t="n">
         <v>13.03019073278621</v>
       </c>
-      <c r="FM2" t="n">
+      <c r="FO2" t="n">
         <v>6.660844822240905</v>
       </c>
-      <c r="FN2" t="n">
+      <c r="FP2" t="n">
         <v>0.760486478236138</v>
       </c>
-      <c r="FO2" t="n">
+      <c r="FQ2" t="n">
         <v>6.704117647353266</v>
       </c>
-      <c r="FP2" t="n">
+      <c r="FR2" t="n">
         <v>11.33901449187054</v>
       </c>
-      <c r="FQ2" t="n">
+      <c r="FS2" t="n">
         <v>3.991196236955225</v>
       </c>
-      <c r="FR2" t="n">
+      <c r="FT2" t="n">
         <v>12.02093578090889</v>
       </c>
-      <c r="FS2" t="n">
+      <c r="FU2" t="n">
         <v>12.0786619722239</v>
       </c>
-      <c r="FT2" t="n">
+      <c r="FV2" t="n">
         <v>5.477700305372392</v>
       </c>
-      <c r="FU2" t="n">
+      <c r="FW2" t="n">
         <v>13.26270242728549</v>
       </c>
     </row>
@@ -2040,40 +2060,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ3" t="n">
+      <c r="FJ3" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK3" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL3" t="n">
         <v>8.812854164768082</v>
       </c>
-      <c r="FK3" t="n">
+      <c r="FM3" t="n">
         <v>0.5147407490389215</v>
       </c>
-      <c r="FL3" t="n">
+      <c r="FN3" t="n">
         <v>8.827873841882386</v>
       </c>
-      <c r="FM3" t="n">
+      <c r="FO3" t="n">
         <v>1.820938041695341</v>
       </c>
-      <c r="FN3" t="n">
+      <c r="FP3" t="n">
         <v>0.1394616286025474</v>
       </c>
-      <c r="FO3" t="n">
+      <c r="FQ3" t="n">
         <v>1.826270762385945</v>
       </c>
-      <c r="FP3" t="n">
+      <c r="FR3" t="n">
         <v>8.631720343374155</v>
       </c>
-      <c r="FQ3" t="n">
+      <c r="FS3" t="n">
         <v>0.3809557776537063</v>
       </c>
-      <c r="FR3" t="n">
+      <c r="FT3" t="n">
         <v>8.640122880535149</v>
       </c>
-      <c r="FS3" t="n">
+      <c r="FU3" t="n">
         <v>9.568842686593078</v>
       </c>
-      <c r="FT3" t="n">
+      <c r="FV3" t="n">
         <v>0.3077838821085279</v>
       </c>
-      <c r="FU3" t="n">
+      <c r="FW3" t="n">
         <v>9.573791374312039</v>
       </c>
     </row>
@@ -2427,40 +2457,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ4" t="n">
+      <c r="FJ4" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK4" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL4" t="n">
         <v>15.40526648232108</v>
       </c>
-      <c r="FK4" t="n">
+      <c r="FM4" t="n">
         <v>7.56573904009105</v>
       </c>
-      <c r="FL4" t="n">
+      <c r="FN4" t="n">
         <v>17.16282734907285</v>
       </c>
-      <c r="FM4" t="n">
+      <c r="FO4" t="n">
         <v>16.0028101298167</v>
       </c>
-      <c r="FN4" t="n">
+      <c r="FP4" t="n">
         <v>0.7712911061118694</v>
       </c>
-      <c r="FO4" t="n">
+      <c r="FQ4" t="n">
         <v>16.02138639510737</v>
       </c>
-      <c r="FP4" t="n">
+      <c r="FR4" t="n">
         <v>15.14392296276992</v>
       </c>
-      <c r="FQ4" t="n">
+      <c r="FS4" t="n">
         <v>7.675061877116122</v>
       </c>
-      <c r="FR4" t="n">
+      <c r="FT4" t="n">
         <v>16.97777893364945</v>
       </c>
-      <c r="FS4" t="n">
+      <c r="FU4" t="n">
         <v>14.66626605375265</v>
       </c>
-      <c r="FT4" t="n">
+      <c r="FV4" t="n">
         <v>6.940171393216092</v>
       </c>
-      <c r="FU4" t="n">
+      <c r="FW4" t="n">
         <v>16.22545342745997</v>
       </c>
     </row>
@@ -2814,40 +2854,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ5" t="n">
+      <c r="FJ5" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK5" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL5" t="n">
         <v>22.07778301145052</v>
       </c>
-      <c r="FK5" t="n">
+      <c r="FM5" t="n">
         <v>3.637750961324596</v>
       </c>
-      <c r="FL5" t="n">
+      <c r="FN5" t="n">
         <v>22.37547172144782</v>
       </c>
-      <c r="FM5" t="n">
+      <c r="FO5" t="n">
         <v>12.80778392836232</v>
       </c>
-      <c r="FN5" t="n">
+      <c r="FP5" t="n">
         <v>1.062393025105198</v>
       </c>
-      <c r="FO5" t="n">
+      <c r="FQ5" t="n">
         <v>12.85177062102371</v>
       </c>
-      <c r="FP5" t="n">
+      <c r="FR5" t="n">
         <v>25.17885982210843</v>
       </c>
-      <c r="FQ5" t="n">
+      <c r="FS5" t="n">
         <v>4.795083012295237</v>
       </c>
-      <c r="FR5" t="n">
+      <c r="FT5" t="n">
         <v>25.63138316666091</v>
       </c>
-      <c r="FS5" t="n">
+      <c r="FU5" t="n">
         <v>22.25574612064434</v>
       </c>
-      <c r="FT5" t="n">
+      <c r="FV5" t="n">
         <v>3.996504243710195</v>
       </c>
-      <c r="FU5" t="n">
+      <c r="FW5" t="n">
         <v>22.61172884935093</v>
       </c>
     </row>
@@ -3201,40 +3251,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ6" t="n">
+      <c r="FJ6" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK6" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL6" t="n">
         <v>22.36396170184736</v>
       </c>
-      <c r="FK6" t="n">
+      <c r="FM6" t="n">
         <v>7.514890774556765</v>
       </c>
-      <c r="FL6" t="n">
+      <c r="FN6" t="n">
         <v>23.59280327462622</v>
       </c>
-      <c r="FM6" t="n">
+      <c r="FO6" t="n">
         <v>9.671228600928028</v>
       </c>
-      <c r="FN6" t="n">
+      <c r="FP6" t="n">
         <v>0.2441693113478326</v>
       </c>
-      <c r="FO6" t="n">
+      <c r="FQ6" t="n">
         <v>9.674310378730484</v>
       </c>
-      <c r="FP6" t="n">
+      <c r="FR6" t="n">
         <v>22.01893119233196</v>
       </c>
-      <c r="FQ6" t="n">
+      <c r="FS6" t="n">
         <v>7.019581723394649</v>
       </c>
-      <c r="FR6" t="n">
+      <c r="FT6" t="n">
         <v>23.11077364399698</v>
       </c>
-      <c r="FS6" t="n">
+      <c r="FU6" t="n">
         <v>21.02924185336531</v>
       </c>
-      <c r="FT6" t="n">
+      <c r="FV6" t="n">
         <v>3.478381969525225</v>
       </c>
-      <c r="FU6" t="n">
+      <c r="FW6" t="n">
         <v>21.31497487808159</v>
       </c>
     </row>
@@ -3588,40 +3648,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ7" t="n">
+      <c r="FJ7" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK7" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL7" t="n">
         <v>15.23192847140227</v>
       </c>
-      <c r="FK7" t="n">
+      <c r="FM7" t="n">
         <v>8.382883472730272</v>
       </c>
-      <c r="FL7" t="n">
+      <c r="FN7" t="n">
         <v>17.38632739468832</v>
       </c>
-      <c r="FM7" t="n">
+      <c r="FO7" t="n">
         <v>16.10950471702693</v>
       </c>
-      <c r="FN7" t="n">
+      <c r="FP7" t="n">
         <v>0.7764805258033659</v>
       </c>
-      <c r="FO7" t="n">
+      <c r="FQ7" t="n">
         <v>16.12820709920556</v>
       </c>
-      <c r="FP7" t="n">
+      <c r="FR7" t="n">
         <v>15.23959245760613</v>
       </c>
-      <c r="FQ7" t="n">
+      <c r="FS7" t="n">
         <v>7.695635569705036</v>
       </c>
-      <c r="FR7" t="n">
+      <c r="FT7" t="n">
         <v>17.07243348487951</v>
       </c>
-      <c r="FS7" t="n">
+      <c r="FU7" t="n">
         <v>14.81117825687589</v>
       </c>
-      <c r="FT7" t="n">
+      <c r="FV7" t="n">
         <v>6.145605603191213</v>
       </c>
-      <c r="FU7" t="n">
+      <c r="FW7" t="n">
         <v>16.03556888878372</v>
       </c>
     </row>
@@ -3975,40 +4045,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ8" t="n">
+      <c r="FJ8" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK8" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL8" t="n">
         <v>12.45638042715818</v>
       </c>
-      <c r="FK8" t="n">
+      <c r="FM8" t="n">
         <v>6.90006871848267</v>
       </c>
-      <c r="FL8" t="n">
+      <c r="FN8" t="n">
         <v>14.23981606854079</v>
       </c>
-      <c r="FM8" t="n">
+      <c r="FO8" t="n">
         <v>5.583833832753895</v>
       </c>
-      <c r="FN8" t="n">
+      <c r="FP8" t="n">
         <v>0.7646816354685342</v>
       </c>
-      <c r="FO8" t="n">
+      <c r="FQ8" t="n">
         <v>5.635950521023928</v>
       </c>
-      <c r="FP8" t="n">
+      <c r="FR8" t="n">
         <v>10.79513817043517</v>
       </c>
-      <c r="FQ8" t="n">
+      <c r="FS8" t="n">
         <v>5.341392781511947</v>
       </c>
-      <c r="FR8" t="n">
+      <c r="FT8" t="n">
         <v>12.04431338703765</v>
       </c>
-      <c r="FS8" t="n">
+      <c r="FU8" t="n">
         <v>13.41746074539884</v>
       </c>
-      <c r="FT8" t="n">
+      <c r="FV8" t="n">
         <v>4.483850607786716</v>
       </c>
-      <c r="FU8" t="n">
+      <c r="FW8" t="n">
         <v>14.14684307989836</v>
       </c>
     </row>
@@ -4362,40 +4442,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ9" t="n">
+      <c r="FJ9" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK9" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL9" t="n">
         <v>10.95958129695609</v>
       </c>
-      <c r="FK9" t="n">
+      <c r="FM9" t="n">
         <v>0.5840093204502427</v>
       </c>
-      <c r="FL9" t="n">
+      <c r="FN9" t="n">
         <v>10.97513048172834</v>
       </c>
-      <c r="FM9" t="n">
+      <c r="FO9" t="n">
         <v>4.22942194412723</v>
       </c>
-      <c r="FN9" t="n">
+      <c r="FP9" t="n">
         <v>0.3009834817800837</v>
       </c>
-      <c r="FO9" t="n">
+      <c r="FQ9" t="n">
         <v>4.24011804526353</v>
       </c>
-      <c r="FP9" t="n">
+      <c r="FR9" t="n">
         <v>10.64256091615308</v>
       </c>
-      <c r="FQ9" t="n">
+      <c r="FS9" t="n">
         <v>0.4935887688192945</v>
       </c>
-      <c r="FR9" t="n">
+      <c r="FT9" t="n">
         <v>10.65400078499779</v>
       </c>
-      <c r="FS9" t="n">
+      <c r="FU9" t="n">
         <v>10.23955393254601</v>
       </c>
-      <c r="FT9" t="n">
+      <c r="FV9" t="n">
         <v>0.3068515970832132</v>
       </c>
-      <c r="FU9" t="n">
+      <c r="FW9" t="n">
         <v>10.24415065489331</v>
       </c>
     </row>
@@ -4749,40 +4839,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ10" t="n">
+      <c r="FJ10" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK10" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL10" t="n">
         <v>9.547429219288917</v>
       </c>
-      <c r="FK10" t="n">
+      <c r="FM10" t="n">
         <v>0.58793546548715</v>
       </c>
-      <c r="FL10" t="n">
+      <c r="FN10" t="n">
         <v>9.565514769677028</v>
       </c>
-      <c r="FM10" t="n">
+      <c r="FO10" t="n">
         <v>2.059288174256375</v>
       </c>
-      <c r="FN10" t="n">
+      <c r="FP10" t="n">
         <v>0.2508833855479254</v>
       </c>
-      <c r="FO10" t="n">
+      <c r="FQ10" t="n">
         <v>2.074514463139783</v>
       </c>
-      <c r="FP10" t="n">
+      <c r="FR10" t="n">
         <v>9.508344465197851</v>
       </c>
-      <c r="FQ10" t="n">
+      <c r="FS10" t="n">
         <v>0.652409344294311</v>
       </c>
-      <c r="FR10" t="n">
+      <c r="FT10" t="n">
         <v>9.530700521020536</v>
       </c>
-      <c r="FS10" t="n">
+      <c r="FU10" t="n">
         <v>9.879857771699022</v>
       </c>
-      <c r="FT10" t="n">
+      <c r="FV10" t="n">
         <v>0.3504062490519649</v>
       </c>
-      <c r="FU10" t="n">
+      <c r="FW10" t="n">
         <v>9.886069700764621</v>
       </c>
     </row>
@@ -5136,40 +5236,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ11" t="n">
+      <c r="FJ11" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK11" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL11" t="n">
         <v>19.72477729067073</v>
       </c>
-      <c r="FK11" t="n">
+      <c r="FM11" t="n">
         <v>1.278327177070766</v>
       </c>
-      <c r="FL11" t="n">
+      <c r="FN11" t="n">
         <v>19.76615692384834</v>
       </c>
-      <c r="FM11" t="n">
+      <c r="FO11" t="n">
         <v>14.44505627073458</v>
       </c>
-      <c r="FN11" t="n">
+      <c r="FP11" t="n">
         <v>0.3532913823210957</v>
       </c>
-      <c r="FO11" t="n">
+      <c r="FQ11" t="n">
         <v>14.44937595418953</v>
       </c>
-      <c r="FP11" t="n">
+      <c r="FR11" t="n">
         <v>19.832793099581</v>
       </c>
-      <c r="FQ11" t="n">
+      <c r="FS11" t="n">
         <v>2.515140141474394</v>
       </c>
-      <c r="FR11" t="n">
+      <c r="FT11" t="n">
         <v>19.99163855370648</v>
       </c>
-      <c r="FS11" t="n">
+      <c r="FU11" t="n">
         <v>22.60595046716871</v>
       </c>
-      <c r="FT11" t="n">
+      <c r="FV11" t="n">
         <v>1.520678008839956</v>
       </c>
-      <c r="FU11" t="n">
+      <c r="FW11" t="n">
         <v>22.65703992428522</v>
       </c>
     </row>
@@ -5523,40 +5633,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ12" t="n">
+      <c r="FJ12" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK12" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL12" t="n">
         <v>23.77856371414163</v>
       </c>
-      <c r="FK12" t="n">
+      <c r="FM12" t="n">
         <v>13.21382033136575</v>
       </c>
-      <c r="FL12" t="n">
+      <c r="FN12" t="n">
         <v>27.20340309698601</v>
       </c>
-      <c r="FM12" t="n">
+      <c r="FO12" t="n">
         <v>10.76315098157229</v>
       </c>
-      <c r="FN12" t="n">
+      <c r="FP12" t="n">
         <v>1.687338211223412</v>
       </c>
-      <c r="FO12" t="n">
+      <c r="FQ12" t="n">
         <v>10.89461010276068</v>
       </c>
-      <c r="FP12" t="n">
+      <c r="FR12" t="n">
         <v>23.04153037374169</v>
       </c>
-      <c r="FQ12" t="n">
+      <c r="FS12" t="n">
         <v>11.58352636185127</v>
       </c>
-      <c r="FR12" t="n">
+      <c r="FT12" t="n">
         <v>25.7893428559117</v>
       </c>
-      <c r="FS12" t="n">
+      <c r="FU12" t="n">
         <v>23.52761270409876</v>
       </c>
-      <c r="FT12" t="n">
+      <c r="FV12" t="n">
         <v>8.737207161136141</v>
       </c>
-      <c r="FU12" t="n">
+      <c r="FW12" t="n">
         <v>25.09755662471305</v>
       </c>
     </row>
@@ -5796,8 +5916,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ13" t="inlineStr"/>
-      <c r="FK13" t="inlineStr"/>
+      <c r="FJ13" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK13" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL13" t="inlineStr"/>
       <c r="FM13" t="inlineStr"/>
       <c r="FN13" t="inlineStr"/>
@@ -5808,6 +5936,8 @@
       <c r="FS13" t="inlineStr"/>
       <c r="FT13" t="inlineStr"/>
       <c r="FU13" t="inlineStr"/>
+      <c r="FV13" t="inlineStr"/>
+      <c r="FW13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6159,40 +6289,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ14" t="n">
+      <c r="FJ14" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK14" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL14" t="n">
         <v>16.66246873798455</v>
       </c>
-      <c r="FK14" t="n">
+      <c r="FM14" t="n">
         <v>7.362064840878699</v>
       </c>
-      <c r="FL14" t="n">
+      <c r="FN14" t="n">
         <v>18.21641740753694</v>
       </c>
-      <c r="FM14" t="n">
+      <c r="FO14" t="n">
         <v>16.65351050049835</v>
       </c>
-      <c r="FN14" t="n">
+      <c r="FP14" t="n">
         <v>0.807905887560127</v>
       </c>
-      <c r="FO14" t="n">
+      <c r="FQ14" t="n">
         <v>16.67309581071743</v>
       </c>
-      <c r="FP14" t="n">
+      <c r="FR14" t="n">
         <v>16.66159768962547</v>
       </c>
-      <c r="FQ14" t="n">
+      <c r="FS14" t="n">
         <v>6.957004530662539</v>
       </c>
-      <c r="FR14" t="n">
+      <c r="FT14" t="n">
         <v>18.05571238169771</v>
       </c>
-      <c r="FS14" t="n">
+      <c r="FU14" t="n">
         <v>17.79071713148385</v>
       </c>
-      <c r="FT14" t="n">
+      <c r="FV14" t="n">
         <v>6.712327562233456</v>
       </c>
-      <c r="FU14" t="n">
+      <c r="FW14" t="n">
         <v>19.01486148661599</v>
       </c>
     </row>
@@ -6436,8 +6576,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ15" t="inlineStr"/>
-      <c r="FK15" t="inlineStr"/>
+      <c r="FJ15" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK15" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL15" t="inlineStr"/>
       <c r="FM15" t="inlineStr"/>
       <c r="FN15" t="inlineStr"/>
@@ -6448,6 +6596,8 @@
       <c r="FS15" t="inlineStr"/>
       <c r="FT15" t="inlineStr"/>
       <c r="FU15" t="inlineStr"/>
+      <c r="FV15" t="inlineStr"/>
+      <c r="FW15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6799,40 +6949,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ16" t="n">
+      <c r="FJ16" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK16" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL16" t="n">
         <v>23.57276408876551</v>
       </c>
-      <c r="FK16" t="n">
+      <c r="FM16" t="n">
         <v>5.709354013668034</v>
       </c>
-      <c r="FL16" t="n">
+      <c r="FN16" t="n">
         <v>24.25431776072006</v>
       </c>
-      <c r="FM16" t="n">
+      <c r="FO16" t="n">
         <v>14.68648906551087</v>
       </c>
-      <c r="FN16" t="n">
+      <c r="FP16" t="n">
         <v>0.881189918642043</v>
       </c>
-      <c r="FO16" t="n">
+      <c r="FQ16" t="n">
         <v>14.71290103086698</v>
       </c>
-      <c r="FP16" t="n">
+      <c r="FR16" t="n">
         <v>21.74020505221871</v>
       </c>
-      <c r="FQ16" t="n">
+      <c r="FS16" t="n">
         <v>4.60958940486415</v>
       </c>
-      <c r="FR16" t="n">
+      <c r="FT16" t="n">
         <v>22.22351975259436</v>
       </c>
-      <c r="FS16" t="n">
+      <c r="FU16" t="n">
         <v>23.68335049599564</v>
       </c>
-      <c r="FT16" t="n">
+      <c r="FV16" t="n">
         <v>4.704470142815306</v>
       </c>
-      <c r="FU16" t="n">
+      <c r="FW16" t="n">
         <v>24.1460789786006</v>
       </c>
     </row>
@@ -7186,40 +7346,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ17" t="n">
+      <c r="FJ17" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK17" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL17" t="n">
         <v>12.56801063805021</v>
       </c>
-      <c r="FK17" t="n">
+      <c r="FM17" t="n">
         <v>5.53541792481932</v>
       </c>
-      <c r="FL17" t="n">
+      <c r="FN17" t="n">
         <v>13.73301652953765</v>
       </c>
-      <c r="FM17" t="n">
+      <c r="FO17" t="n">
         <v>5.351786492515732</v>
       </c>
-      <c r="FN17" t="n">
+      <c r="FP17" t="n">
         <v>0.7215897876706209</v>
       </c>
-      <c r="FO17" t="n">
+      <c r="FQ17" t="n">
         <v>5.400213929386906</v>
       </c>
-      <c r="FP17" t="n">
+      <c r="FR17" t="n">
         <v>12.36354420780947</v>
       </c>
-      <c r="FQ17" t="n">
+      <c r="FS17" t="n">
         <v>5.086243260570073</v>
       </c>
-      <c r="FR17" t="n">
+      <c r="FT17" t="n">
         <v>13.36888536431342</v>
       </c>
-      <c r="FS17" t="n">
+      <c r="FU17" t="n">
         <v>12.12553494858496</v>
       </c>
-      <c r="FT17" t="n">
+      <c r="FV17" t="n">
         <v>3.995092736407302</v>
       </c>
-      <c r="FU17" t="n">
+      <c r="FW17" t="n">
         <v>12.76672878077426</v>
       </c>
     </row>
@@ -7573,40 +7743,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ18" t="n">
+      <c r="FJ18" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK18" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL18" t="n">
         <v>11.6988405708822</v>
       </c>
-      <c r="FK18" t="n">
+      <c r="FM18" t="n">
         <v>5.782371542129826</v>
       </c>
-      <c r="FL18" t="n">
+      <c r="FN18" t="n">
         <v>13.04985407405585</v>
       </c>
-      <c r="FM18" t="n">
+      <c r="FO18" t="n">
         <v>6.730102175627211</v>
       </c>
-      <c r="FN18" t="n">
+      <c r="FP18" t="n">
         <v>0.8110639820229936</v>
       </c>
-      <c r="FO18" t="n">
+      <c r="FQ18" t="n">
         <v>6.778797834226738</v>
       </c>
-      <c r="FP18" t="n">
+      <c r="FR18" t="n">
         <v>11.91048785758825</v>
       </c>
-      <c r="FQ18" t="n">
+      <c r="FS18" t="n">
         <v>5.467895107114291</v>
       </c>
-      <c r="FR18" t="n">
+      <c r="FT18" t="n">
         <v>13.10563229715231</v>
       </c>
-      <c r="FS18" t="n">
+      <c r="FU18" t="n">
         <v>11.95705446294246</v>
       </c>
-      <c r="FT18" t="n">
+      <c r="FV18" t="n">
         <v>5.610233010060628</v>
       </c>
-      <c r="FU18" t="n">
+      <c r="FW18" t="n">
         <v>13.20779564715271</v>
       </c>
     </row>
@@ -7960,40 +8140,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ19" t="n">
+      <c r="FJ19" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK19" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL19" t="n">
         <v>23.90851187632177</v>
       </c>
-      <c r="FK19" t="n">
+      <c r="FM19" t="n">
         <v>5.387925382861173</v>
       </c>
-      <c r="FL19" t="n">
+      <c r="FN19" t="n">
         <v>24.5080941746089</v>
       </c>
-      <c r="FM19" t="n">
+      <c r="FO19" t="n">
         <v>12.05031803699369</v>
       </c>
-      <c r="FN19" t="n">
+      <c r="FP19" t="n">
         <v>1.389631225244185</v>
       </c>
-      <c r="FO19" t="n">
+      <c r="FQ19" t="n">
         <v>12.13017888305317</v>
       </c>
-      <c r="FP19" t="n">
+      <c r="FR19" t="n">
         <v>21.61207922022084</v>
       </c>
-      <c r="FQ19" t="n">
+      <c r="FS19" t="n">
         <v>4.162783118962383</v>
       </c>
-      <c r="FR19" t="n">
+      <c r="FT19" t="n">
         <v>22.00933282761246</v>
       </c>
-      <c r="FS19" t="n">
+      <c r="FU19" t="n">
         <v>23.62231570091741</v>
       </c>
-      <c r="FT19" t="n">
+      <c r="FV19" t="n">
         <v>5.35846391554769</v>
       </c>
-      <c r="FU19" t="n">
+      <c r="FW19" t="n">
         <v>24.22244691619812</v>
       </c>
     </row>
@@ -8347,40 +8537,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ20" t="n">
+      <c r="FJ20" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK20" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL20" t="n">
         <v>12.76517375884876</v>
       </c>
-      <c r="FK20" t="n">
+      <c r="FM20" t="n">
         <v>8.257539699358256</v>
       </c>
-      <c r="FL20" t="n">
+      <c r="FN20" t="n">
         <v>15.20317805526458</v>
       </c>
-      <c r="FM20" t="n">
+      <c r="FO20" t="n">
         <v>10.20110982423881</v>
       </c>
-      <c r="FN20" t="n">
+      <c r="FP20" t="n">
         <v>0.5817313594809707</v>
       </c>
-      <c r="FO20" t="n">
+      <c r="FQ20" t="n">
         <v>10.21768334901729</v>
       </c>
-      <c r="FP20" t="n">
+      <c r="FR20" t="n">
         <v>12.80516910761891</v>
       </c>
-      <c r="FQ20" t="n">
+      <c r="FS20" t="n">
         <v>8.044958506649209</v>
       </c>
-      <c r="FR20" t="n">
+      <c r="FT20" t="n">
         <v>15.12262256516459</v>
       </c>
-      <c r="FS20" t="n">
+      <c r="FU20" t="n">
         <v>10.25841789421533</v>
       </c>
-      <c r="FT20" t="n">
+      <c r="FV20" t="n">
         <v>7.820518618012822</v>
       </c>
-      <c r="FU20" t="n">
+      <c r="FW20" t="n">
         <v>12.8994437533966</v>
       </c>
     </row>
@@ -8734,40 +8934,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ21" t="n">
+      <c r="FJ21" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK21" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL21" t="n">
         <v>11.59968727863275</v>
       </c>
-      <c r="FK21" t="n">
+      <c r="FM21" t="n">
         <v>5.584553624576874</v>
       </c>
-      <c r="FL21" t="n">
+      <c r="FN21" t="n">
         <v>12.87400420024202</v>
       </c>
-      <c r="FM21" t="n">
+      <c r="FO21" t="n">
         <v>6.921901605813077</v>
       </c>
-      <c r="FN21" t="n">
+      <c r="FP21" t="n">
         <v>0.8239892824827922</v>
       </c>
-      <c r="FO21" t="n">
+      <c r="FQ21" t="n">
         <v>6.970773284091527</v>
       </c>
-      <c r="FP21" t="n">
+      <c r="FR21" t="n">
         <v>11.30051154896729</v>
       </c>
-      <c r="FQ21" t="n">
+      <c r="FS21" t="n">
         <v>6.20848018655163</v>
       </c>
-      <c r="FR21" t="n">
+      <c r="FT21" t="n">
         <v>12.89367238203094</v>
       </c>
-      <c r="FS21" t="n">
+      <c r="FU21" t="n">
         <v>12.06887867323049</v>
       </c>
-      <c r="FT21" t="n">
+      <c r="FV21" t="n">
         <v>5.185372393935745</v>
       </c>
-      <c r="FU21" t="n">
+      <c r="FW21" t="n">
         <v>13.13567353784908</v>
       </c>
     </row>
@@ -9121,40 +9331,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ22" t="n">
+      <c r="FJ22" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK22" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL22" t="n">
         <v>10.06838070765761</v>
       </c>
-      <c r="FK22" t="n">
+      <c r="FM22" t="n">
         <v>0.4782476570339776</v>
       </c>
-      <c r="FL22" t="n">
+      <c r="FN22" t="n">
         <v>10.07973267977829</v>
       </c>
-      <c r="FM22" t="n">
+      <c r="FO22" t="n">
         <v>5.689733683844232</v>
       </c>
-      <c r="FN22" t="n">
+      <c r="FP22" t="n">
         <v>0.2954621404044286</v>
       </c>
-      <c r="FO22" t="n">
+      <c r="FQ22" t="n">
         <v>5.697400044711975</v>
       </c>
-      <c r="FP22" t="n">
+      <c r="FR22" t="n">
         <v>10.15749265398484</v>
       </c>
-      <c r="FQ22" t="n">
+      <c r="FS22" t="n">
         <v>0.3881044704227118</v>
       </c>
-      <c r="FR22" t="n">
+      <c r="FT22" t="n">
         <v>10.1649044312142</v>
       </c>
-      <c r="FS22" t="n">
+      <c r="FU22" t="n">
         <v>11.15650869544317</v>
       </c>
-      <c r="FT22" t="n">
+      <c r="FV22" t="n">
         <v>0.5774027828550554</v>
       </c>
-      <c r="FU22" t="n">
+      <c r="FW22" t="n">
         <v>11.17144038363666</v>
       </c>
     </row>
@@ -9508,40 +9728,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ23" t="n">
+      <c r="FJ23" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK23" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL23" t="n">
         <v>10.82152258911765</v>
       </c>
-      <c r="FK23" t="n">
+      <c r="FM23" t="n">
         <v>0.5394836242535124</v>
       </c>
-      <c r="FL23" t="n">
+      <c r="FN23" t="n">
         <v>10.83496163941623</v>
       </c>
-      <c r="FM23" t="n">
+      <c r="FO23" t="n">
         <v>3.075035786166461</v>
       </c>
-      <c r="FN23" t="n">
+      <c r="FP23" t="n">
         <v>0.2780699176236071</v>
       </c>
-      <c r="FO23" t="n">
+      <c r="FQ23" t="n">
         <v>3.087582867761055</v>
       </c>
-      <c r="FP23" t="n">
+      <c r="FR23" t="n">
         <v>10.74183435454661</v>
       </c>
-      <c r="FQ23" t="n">
+      <c r="FS23" t="n">
         <v>0.5201634266724104</v>
       </c>
-      <c r="FR23" t="n">
+      <c r="FT23" t="n">
         <v>10.75442119739437</v>
       </c>
-      <c r="FS23" t="n">
+      <c r="FU23" t="n">
         <v>10.88433533316919</v>
       </c>
-      <c r="FT23" t="n">
+      <c r="FV23" t="n">
         <v>0.2660956421395523</v>
       </c>
-      <c r="FU23" t="n">
+      <c r="FW23" t="n">
         <v>10.88758754433878</v>
       </c>
     </row>
@@ -9895,40 +10125,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ24" t="n">
+      <c r="FJ24" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK24" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL24" t="n">
         <v>18.52607742075992</v>
       </c>
-      <c r="FK24" t="n">
+      <c r="FM24" t="n">
         <v>7.154468255719379</v>
       </c>
-      <c r="FL24" t="n">
+      <c r="FN24" t="n">
         <v>19.85955590193514</v>
       </c>
-      <c r="FM24" t="n">
+      <c r="FO24" t="n">
         <v>16.95525357163482</v>
       </c>
-      <c r="FN24" t="n">
+      <c r="FP24" t="n">
         <v>0.8100464240684657</v>
       </c>
-      <c r="FO24" t="n">
+      <c r="FQ24" t="n">
         <v>16.97459274585347</v>
       </c>
-      <c r="FP24" t="n">
+      <c r="FR24" t="n">
         <v>18.72315257610699</v>
       </c>
-      <c r="FQ24" t="n">
+      <c r="FS24" t="n">
         <v>6.42915633578095</v>
       </c>
-      <c r="FR24" t="n">
+      <c r="FT24" t="n">
         <v>19.79622422529342</v>
       </c>
-      <c r="FS24" t="n">
+      <c r="FU24" t="n">
         <v>18.64106344333563</v>
       </c>
-      <c r="FT24" t="n">
+      <c r="FV24" t="n">
         <v>5.836097498076973</v>
       </c>
-      <c r="FU24" t="n">
+      <c r="FW24" t="n">
         <v>19.53328646965288</v>
       </c>
     </row>
@@ -10282,40 +10522,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ25" t="n">
+      <c r="FJ25" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK25" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL25" t="n">
         <v>23.45683531976787</v>
       </c>
-      <c r="FK25" t="n">
+      <c r="FM25" t="n">
         <v>4.599494412844084</v>
       </c>
-      <c r="FL25" t="n">
+      <c r="FN25" t="n">
         <v>23.90352426050379</v>
       </c>
-      <c r="FM25" t="n">
+      <c r="FO25" t="n">
         <v>11.7930955359003</v>
       </c>
-      <c r="FN25" t="n">
+      <c r="FP25" t="n">
         <v>1.246961800547395</v>
       </c>
-      <c r="FO25" t="n">
+      <c r="FQ25" t="n">
         <v>11.85883704462187</v>
       </c>
-      <c r="FP25" t="n">
+      <c r="FR25" t="n">
         <v>23.12033664226451</v>
       </c>
-      <c r="FQ25" t="n">
+      <c r="FS25" t="n">
         <v>4.881616368837643</v>
       </c>
-      <c r="FR25" t="n">
+      <c r="FT25" t="n">
         <v>23.63006865889607</v>
       </c>
-      <c r="FS25" t="n">
+      <c r="FU25" t="n">
         <v>25.46407310004149</v>
       </c>
-      <c r="FT25" t="n">
+      <c r="FV25" t="n">
         <v>7.738547036375929</v>
       </c>
-      <c r="FU25" t="n">
+      <c r="FW25" t="n">
         <v>26.61398371304941</v>
       </c>
     </row>
@@ -10669,40 +10919,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ26" t="n">
+      <c r="FJ26" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK26" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL26" t="n">
         <v>20.64917345827275</v>
       </c>
-      <c r="FK26" t="n">
+      <c r="FM26" t="n">
         <v>1.528327080046198</v>
       </c>
-      <c r="FL26" t="n">
+      <c r="FN26" t="n">
         <v>20.70565498054669</v>
       </c>
-      <c r="FM26" t="n">
+      <c r="FO26" t="n">
         <v>12.13061983076333</v>
       </c>
-      <c r="FN26" t="n">
+      <c r="FP26" t="n">
         <v>0.2269115447275628</v>
       </c>
-      <c r="FO26" t="n">
+      <c r="FQ26" t="n">
         <v>12.1327419130071</v>
       </c>
-      <c r="FP26" t="n">
+      <c r="FR26" t="n">
         <v>20.96251919755805</v>
       </c>
-      <c r="FQ26" t="n">
+      <c r="FS26" t="n">
         <v>3.127084127826677</v>
       </c>
-      <c r="FR26" t="n">
+      <c r="FT26" t="n">
         <v>21.19447725825044</v>
       </c>
-      <c r="FS26" t="n">
+      <c r="FU26" t="n">
         <v>20.67400847566489</v>
       </c>
-      <c r="FT26" t="n">
+      <c r="FV26" t="n">
         <v>2.206021715848991</v>
       </c>
-      <c r="FU26" t="n">
+      <c r="FW26" t="n">
         <v>20.79137220730419</v>
       </c>
     </row>
@@ -11056,40 +11316,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ27" t="n">
+      <c r="FJ27" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK27" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL27" t="n">
         <v>22.70808457043826</v>
       </c>
-      <c r="FK27" t="n">
+      <c r="FM27" t="n">
         <v>5.441318300519193</v>
       </c>
-      <c r="FL27" t="n">
+      <c r="FN27" t="n">
         <v>23.35091111082694</v>
       </c>
-      <c r="FM27" t="n">
+      <c r="FO27" t="n">
         <v>14.23096538904335</v>
       </c>
-      <c r="FN27" t="n">
+      <c r="FP27" t="n">
         <v>1.027937769485584</v>
       </c>
-      <c r="FO27" t="n">
+      <c r="FQ27" t="n">
         <v>14.26804233110081</v>
       </c>
-      <c r="FP27" t="n">
+      <c r="FR27" t="n">
         <v>22.42313373559066</v>
       </c>
-      <c r="FQ27" t="n">
+      <c r="FS27" t="n">
         <v>4.124460057881371</v>
       </c>
-      <c r="FR27" t="n">
+      <c r="FT27" t="n">
         <v>22.79930036850348</v>
       </c>
-      <c r="FS27" t="n">
+      <c r="FU27" t="n">
         <v>23.05309100598607</v>
       </c>
-      <c r="FT27" t="n">
+      <c r="FV27" t="n">
         <v>4.662477879391781</v>
       </c>
-      <c r="FU27" t="n">
+      <c r="FW27" t="n">
         <v>23.51985767189278</v>
       </c>
     </row>
@@ -11443,40 +11713,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ28" t="n">
+      <c r="FJ28" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK28" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL28" t="n">
         <v>12.74256316009895</v>
       </c>
-      <c r="FK28" t="n">
+      <c r="FM28" t="n">
         <v>7.11070035069484</v>
       </c>
-      <c r="FL28" t="n">
+      <c r="FN28" t="n">
         <v>14.59229164204453</v>
       </c>
-      <c r="FM28" t="n">
+      <c r="FO28" t="n">
         <v>6.250665059623991</v>
       </c>
-      <c r="FN28" t="n">
+      <c r="FP28" t="n">
         <v>0.6963419413388723</v>
       </c>
-      <c r="FO28" t="n">
+      <c r="FQ28" t="n">
         <v>6.289332698058814</v>
       </c>
-      <c r="FP28" t="n">
+      <c r="FR28" t="n">
         <v>12.46459684720019</v>
       </c>
-      <c r="FQ28" t="n">
+      <c r="FS28" t="n">
         <v>5.364199129595028</v>
       </c>
-      <c r="FR28" t="n">
+      <c r="FT28" t="n">
         <v>13.56984918358273</v>
       </c>
-      <c r="FS28" t="n">
+      <c r="FU28" t="n">
         <v>12.0184447842989</v>
       </c>
-      <c r="FT28" t="n">
+      <c r="FV28" t="n">
         <v>4.863137494607851</v>
       </c>
-      <c r="FU28" t="n">
+      <c r="FW28" t="n">
         <v>12.96507313225429</v>
       </c>
     </row>
@@ -11728,8 +12008,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ29" t="inlineStr"/>
-      <c r="FK29" t="inlineStr"/>
+      <c r="FJ29" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK29" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL29" t="inlineStr"/>
       <c r="FM29" t="inlineStr"/>
       <c r="FN29" t="inlineStr"/>
@@ -11740,6 +12028,8 @@
       <c r="FS29" t="inlineStr"/>
       <c r="FT29" t="inlineStr"/>
       <c r="FU29" t="inlineStr"/>
+      <c r="FV29" t="inlineStr"/>
+      <c r="FW29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -11975,8 +12265,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ30" t="inlineStr"/>
-      <c r="FK30" t="inlineStr"/>
+      <c r="FJ30" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK30" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL30" t="inlineStr"/>
       <c r="FM30" t="inlineStr"/>
       <c r="FN30" t="inlineStr"/>
@@ -11987,6 +12285,8 @@
       <c r="FS30" t="inlineStr"/>
       <c r="FT30" t="inlineStr"/>
       <c r="FU30" t="inlineStr"/>
+      <c r="FV30" t="inlineStr"/>
+      <c r="FW30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12338,40 +12638,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ31" t="n">
+      <c r="FJ31" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK31" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL31" t="n">
         <v>10.27508223365736</v>
       </c>
-      <c r="FK31" t="n">
+      <c r="FM31" t="n">
         <v>8.006156663369223</v>
       </c>
-      <c r="FL31" t="n">
+      <c r="FN31" t="n">
         <v>13.02596865598995</v>
       </c>
-      <c r="FM31" t="n">
+      <c r="FO31" t="n">
         <v>8.553102682453693</v>
       </c>
-      <c r="FN31" t="n">
+      <c r="FP31" t="n">
         <v>0.680313884081196</v>
       </c>
-      <c r="FO31" t="n">
+      <c r="FQ31" t="n">
         <v>8.580116110955037</v>
       </c>
-      <c r="FP31" t="n">
+      <c r="FR31" t="n">
         <v>10.35935518299652</v>
       </c>
-      <c r="FQ31" t="n">
+      <c r="FS31" t="n">
         <v>8.315947152816483</v>
       </c>
-      <c r="FR31" t="n">
+      <c r="FT31" t="n">
         <v>13.28424694350091</v>
       </c>
-      <c r="FS31" t="n">
+      <c r="FU31" t="n">
         <v>10.04058048505608</v>
       </c>
-      <c r="FT31" t="n">
+      <c r="FV31" t="n">
         <v>8.090359733318055</v>
       </c>
-      <c r="FU31" t="n">
+      <c r="FW31" t="n">
         <v>12.8944630400565</v>
       </c>
     </row>
@@ -12623,8 +12933,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ32" t="inlineStr"/>
-      <c r="FK32" t="inlineStr"/>
+      <c r="FJ32" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK32" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL32" t="inlineStr"/>
       <c r="FM32" t="inlineStr"/>
       <c r="FN32" t="inlineStr"/>
@@ -12635,6 +12953,8 @@
       <c r="FS32" t="inlineStr"/>
       <c r="FT32" t="inlineStr"/>
       <c r="FU32" t="inlineStr"/>
+      <c r="FV32" t="inlineStr"/>
+      <c r="FW32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -12986,40 +13306,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ33" t="n">
+      <c r="FJ33" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK33" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL33" t="n">
         <v>10.13926251462559</v>
       </c>
-      <c r="FK33" t="n">
+      <c r="FM33" t="n">
         <v>0.3711899805154612</v>
       </c>
-      <c r="FL33" t="n">
+      <c r="FN33" t="n">
         <v>10.14605471807277</v>
       </c>
-      <c r="FM33" t="n">
+      <c r="FO33" t="n">
         <v>9.195925087990119</v>
       </c>
-      <c r="FN33" t="n">
+      <c r="FP33" t="n">
         <v>0.3451720912671527</v>
       </c>
-      <c r="FO33" t="n">
+      <c r="FQ33" t="n">
         <v>9.202400882189162</v>
       </c>
-      <c r="FP33" t="n">
+      <c r="FR33" t="n">
         <v>10.06315709072355</v>
       </c>
-      <c r="FQ33" t="n">
+      <c r="FS33" t="n">
         <v>0.2455054519345234</v>
       </c>
-      <c r="FR33" t="n">
+      <c r="FT33" t="n">
         <v>10.06615137773664</v>
       </c>
-      <c r="FS33" t="n">
+      <c r="FU33" t="n">
         <v>10.09805406138959</v>
       </c>
-      <c r="FT33" t="n">
+      <c r="FV33" t="n">
         <v>0.2481430806857248</v>
       </c>
-      <c r="FU33" t="n">
+      <c r="FW33" t="n">
         <v>10.10110245543718</v>
       </c>
     </row>
@@ -13373,40 +13703,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ34" t="n">
+      <c r="FJ34" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK34" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL34" t="n">
         <v>11.58574047457262</v>
       </c>
-      <c r="FK34" t="n">
+      <c r="FM34" t="n">
         <v>7.396085523071864</v>
       </c>
-      <c r="FL34" t="n">
+      <c r="FN34" t="n">
         <v>13.74523420712588</v>
       </c>
-      <c r="FM34" t="n">
+      <c r="FO34" t="n">
         <v>7.133364993411141</v>
       </c>
-      <c r="FN34" t="n">
+      <c r="FP34" t="n">
         <v>0.8195481453703527</v>
       </c>
-      <c r="FO34" t="n">
+      <c r="FQ34" t="n">
         <v>7.180289359893758</v>
       </c>
-      <c r="FP34" t="n">
+      <c r="FR34" t="n">
         <v>11.84501363463948</v>
       </c>
-      <c r="FQ34" t="n">
+      <c r="FS34" t="n">
         <v>6.8827394388336</v>
       </c>
-      <c r="FR34" t="n">
+      <c r="FT34" t="n">
         <v>13.69950547237639</v>
       </c>
-      <c r="FS34" t="n">
+      <c r="FU34" t="n">
         <v>11.01677675789685</v>
       </c>
-      <c r="FT34" t="n">
+      <c r="FV34" t="n">
         <v>6.463199257582217</v>
       </c>
-      <c r="FU34" t="n">
+      <c r="FW34" t="n">
         <v>12.77271759558425</v>
       </c>
     </row>
@@ -13760,40 +14100,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ35" t="n">
+      <c r="FJ35" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK35" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL35" t="n">
         <v>21.06994802101308</v>
       </c>
-      <c r="FK35" t="n">
+      <c r="FM35" t="n">
         <v>0.9995498263668281</v>
       </c>
-      <c r="FL35" t="n">
+      <c r="FN35" t="n">
         <v>21.0936438166473</v>
       </c>
-      <c r="FM35" t="n">
+      <c r="FO35" t="n">
         <v>15.51228274144422</v>
       </c>
-      <c r="FN35" t="n">
+      <c r="FP35" t="n">
         <v>0.2857348404096482</v>
       </c>
-      <c r="FO35" t="n">
+      <c r="FQ35" t="n">
         <v>15.51491412317619</v>
       </c>
-      <c r="FP35" t="n">
+      <c r="FR35" t="n">
         <v>21.89135143780826</v>
       </c>
-      <c r="FQ35" t="n">
+      <c r="FS35" t="n">
         <v>1.006362884444798</v>
       </c>
-      <c r="FR35" t="n">
+      <c r="FT35" t="n">
         <v>21.91447088178992</v>
       </c>
-      <c r="FS35" t="n">
+      <c r="FU35" t="n">
         <v>19.99335081361543</v>
       </c>
-      <c r="FT35" t="n">
+      <c r="FV35" t="n">
         <v>0.5255208051462807</v>
       </c>
-      <c r="FU35" t="n">
+      <c r="FW35" t="n">
         <v>20.00025622018223</v>
       </c>
     </row>
@@ -14147,40 +14497,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ36" t="n">
+      <c r="FJ36" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK36" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL36" t="n">
         <v>21.01912485110731</v>
       </c>
-      <c r="FK36" t="n">
+      <c r="FM36" t="n">
         <v>0.5154703101026169</v>
       </c>
-      <c r="FL36" t="n">
+      <c r="FN36" t="n">
         <v>21.02544456478946</v>
       </c>
-      <c r="FM36" t="n">
+      <c r="FO36" t="n">
         <v>18.45264952542191</v>
       </c>
-      <c r="FN36" t="n">
+      <c r="FP36" t="n">
         <v>0.2949945261609049</v>
       </c>
-      <c r="FO36" t="n">
+      <c r="FQ36" t="n">
         <v>18.45500734972811</v>
       </c>
-      <c r="FP36" t="n">
+      <c r="FR36" t="n">
         <v>21.00665899337289</v>
       </c>
-      <c r="FQ36" t="n">
+      <c r="FS36" t="n">
         <v>0.4916754235820499</v>
       </c>
-      <c r="FR36" t="n">
+      <c r="FT36" t="n">
         <v>21.01241220769307</v>
       </c>
-      <c r="FS36" t="n">
+      <c r="FU36" t="n">
         <v>21.05502212777985</v>
       </c>
-      <c r="FT36" t="n">
+      <c r="FV36" t="n">
         <v>0.4006527245731421</v>
       </c>
-      <c r="FU36" t="n">
+      <c r="FW36" t="n">
         <v>21.05883376179714</v>
       </c>
     </row>
@@ -14534,40 +14894,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ37" t="n">
+      <c r="FJ37" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK37" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL37" t="n">
         <v>10.96947277744752</v>
       </c>
-      <c r="FK37" t="n">
+      <c r="FM37" t="n">
         <v>0.3011961489087248</v>
       </c>
-      <c r="FL37" t="n">
+      <c r="FN37" t="n">
         <v>10.97360707038846</v>
       </c>
-      <c r="FM37" t="n">
+      <c r="FO37" t="n">
         <v>8.363642685084212</v>
       </c>
-      <c r="FN37" t="n">
+      <c r="FP37" t="n">
         <v>0.3134737698162107</v>
       </c>
-      <c r="FO37" t="n">
+      <c r="FQ37" t="n">
         <v>8.369515205083594</v>
       </c>
-      <c r="FP37" t="n">
+      <c r="FR37" t="n">
         <v>10.89474094983856</v>
       </c>
-      <c r="FQ37" t="n">
+      <c r="FS37" t="n">
         <v>0.3590079961185646</v>
       </c>
-      <c r="FR37" t="n">
+      <c r="FT37" t="n">
         <v>10.90065443472851</v>
       </c>
-      <c r="FS37" t="n">
+      <c r="FU37" t="n">
         <v>10.85711927153742</v>
       </c>
-      <c r="FT37" t="n">
+      <c r="FV37" t="n">
         <v>0.2816921770068496</v>
       </c>
-      <c r="FU37" t="n">
+      <c r="FW37" t="n">
         <v>10.86077296323683</v>
       </c>
     </row>
@@ -14921,40 +15291,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ38" t="n">
+      <c r="FJ38" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK38" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL38" t="n">
         <v>11.35284150308764</v>
       </c>
-      <c r="FK38" t="n">
+      <c r="FM38" t="n">
         <v>7.27976447298062</v>
       </c>
-      <c r="FL38" t="n">
+      <c r="FN38" t="n">
         <v>13.48636277786936</v>
       </c>
-      <c r="FM38" t="n">
+      <c r="FO38" t="n">
         <v>7.715136773351234</v>
       </c>
-      <c r="FN38" t="n">
+      <c r="FP38" t="n">
         <v>0.7656970862355915</v>
       </c>
-      <c r="FO38" t="n">
+      <c r="FQ38" t="n">
         <v>7.753039885063545</v>
       </c>
-      <c r="FP38" t="n">
+      <c r="FR38" t="n">
         <v>10.67652178954796</v>
       </c>
-      <c r="FQ38" t="n">
+      <c r="FS38" t="n">
         <v>7.604543779682491</v>
       </c>
-      <c r="FR38" t="n">
+      <c r="FT38" t="n">
         <v>13.10790614933598</v>
       </c>
-      <c r="FS38" t="n">
+      <c r="FU38" t="n">
         <v>10.82337996347081</v>
       </c>
-      <c r="FT38" t="n">
+      <c r="FV38" t="n">
         <v>5.650153138749794</v>
       </c>
-      <c r="FU38" t="n">
+      <c r="FW38" t="n">
         <v>12.20941375844826</v>
       </c>
     </row>
@@ -15308,40 +15688,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ39" t="n">
+      <c r="FJ39" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK39" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL39" t="n">
         <v>20.98914564037201</v>
       </c>
-      <c r="FK39" t="n">
+      <c r="FM39" t="n">
         <v>5.814635058140599</v>
       </c>
-      <c r="FL39" t="n">
+      <c r="FN39" t="n">
         <v>21.77967436790791</v>
       </c>
-      <c r="FM39" t="n">
+      <c r="FO39" t="n">
         <v>17.61812485635178</v>
       </c>
-      <c r="FN39" t="n">
+      <c r="FP39" t="n">
         <v>0.8888563137253359</v>
       </c>
-      <c r="FO39" t="n">
+      <c r="FQ39" t="n">
         <v>17.64053256000084</v>
       </c>
-      <c r="FP39" t="n">
+      <c r="FR39" t="n">
         <v>20.5725082764983</v>
       </c>
-      <c r="FQ39" t="n">
+      <c r="FS39" t="n">
         <v>6.336799374574555</v>
       </c>
-      <c r="FR39" t="n">
+      <c r="FT39" t="n">
         <v>21.52633557064925</v>
       </c>
-      <c r="FS39" t="n">
+      <c r="FU39" t="n">
         <v>20.57923674859626</v>
       </c>
-      <c r="FT39" t="n">
+      <c r="FV39" t="n">
         <v>5.505089344234035</v>
       </c>
-      <c r="FU39" t="n">
+      <c r="FW39" t="n">
         <v>21.30284004171213</v>
       </c>
     </row>
@@ -15695,40 +16085,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ40" t="n">
+      <c r="FJ40" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK40" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL40" t="n">
         <v>22.03910048877085</v>
       </c>
-      <c r="FK40" t="n">
+      <c r="FM40" t="n">
         <v>5.500870797997629</v>
       </c>
-      <c r="FL40" t="n">
+      <c r="FN40" t="n">
         <v>22.71522682894455</v>
       </c>
-      <c r="FM40" t="n">
+      <c r="FO40" t="n">
         <v>17.11934350990678</v>
       </c>
-      <c r="FN40" t="n">
+      <c r="FP40" t="n">
         <v>0.9111607266161953</v>
       </c>
-      <c r="FO40" t="n">
+      <c r="FQ40" t="n">
         <v>17.14357419209644</v>
       </c>
-      <c r="FP40" t="n">
+      <c r="FR40" t="n">
         <v>21.44582942244931</v>
       </c>
-      <c r="FQ40" t="n">
+      <c r="FS40" t="n">
         <v>5.622424262031559</v>
       </c>
-      <c r="FR40" t="n">
+      <c r="FT40" t="n">
         <v>22.17059435827271</v>
       </c>
-      <c r="FS40" t="n">
+      <c r="FU40" t="n">
         <v>22.43384222760642</v>
       </c>
-      <c r="FT40" t="n">
+      <c r="FV40" t="n">
         <v>5.013190136527002</v>
       </c>
-      <c r="FU40" t="n">
+      <c r="FW40" t="n">
         <v>22.9871562494822</v>
       </c>
     </row>
@@ -16082,40 +16482,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ41" t="n">
+      <c r="FJ41" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK41" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL41" t="n">
         <v>10.46117497570881</v>
       </c>
-      <c r="FK41" t="n">
+      <c r="FM41" t="n">
         <v>6.127439729074627</v>
       </c>
-      <c r="FL41" t="n">
+      <c r="FN41" t="n">
         <v>12.12360092983262</v>
       </c>
-      <c r="FM41" t="n">
+      <c r="FO41" t="n">
         <v>8.253105166243735</v>
       </c>
-      <c r="FN41" t="n">
+      <c r="FP41" t="n">
         <v>0.7169558774105811</v>
       </c>
-      <c r="FO41" t="n">
+      <c r="FQ41" t="n">
         <v>8.284187987680664</v>
       </c>
-      <c r="FP41" t="n">
+      <c r="FR41" t="n">
         <v>10.06248866419739</v>
       </c>
-      <c r="FQ41" t="n">
+      <c r="FS41" t="n">
         <v>6.825084800805658</v>
       </c>
-      <c r="FR41" t="n">
+      <c r="FT41" t="n">
         <v>12.15876065457698</v>
       </c>
-      <c r="FS41" t="n">
+      <c r="FU41" t="n">
         <v>10.56043475277702</v>
       </c>
-      <c r="FT41" t="n">
+      <c r="FV41" t="n">
         <v>6.817349882231063</v>
       </c>
-      <c r="FU41" t="n">
+      <c r="FW41" t="n">
         <v>12.56976696619378</v>
       </c>
     </row>
@@ -16469,40 +16879,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ42" t="n">
+      <c r="FJ42" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK42" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL42" t="n">
         <v>10.79047342816301</v>
       </c>
-      <c r="FK42" t="n">
+      <c r="FM42" t="n">
         <v>0.4230529732758205</v>
       </c>
-      <c r="FL42" t="n">
+      <c r="FN42" t="n">
         <v>10.79876338392918</v>
       </c>
-      <c r="FM42" t="n">
+      <c r="FO42" t="n">
         <v>7.441255061391746</v>
       </c>
-      <c r="FN42" t="n">
+      <c r="FP42" t="n">
         <v>0.3192883302831512</v>
       </c>
-      <c r="FO42" t="n">
+      <c r="FQ42" t="n">
         <v>7.448101900923702</v>
       </c>
-      <c r="FP42" t="n">
+      <c r="FR42" t="n">
         <v>11.17082488685008</v>
       </c>
-      <c r="FQ42" t="n">
+      <c r="FS42" t="n">
         <v>0.4613121512953902</v>
       </c>
-      <c r="FR42" t="n">
+      <c r="FT42" t="n">
         <v>11.18034603908134</v>
       </c>
-      <c r="FS42" t="n">
+      <c r="FU42" t="n">
         <v>10.74577314268967</v>
       </c>
-      <c r="FT42" t="n">
+      <c r="FV42" t="n">
         <v>0.5106737623768642</v>
       </c>
-      <c r="FU42" t="n">
+      <c r="FW42" t="n">
         <v>10.75790073042742</v>
       </c>
     </row>
@@ -16856,40 +17276,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ43" t="n">
+      <c r="FJ43" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK43" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL43" t="n">
         <v>10.38527128428521</v>
       </c>
-      <c r="FK43" t="n">
+      <c r="FM43" t="n">
         <v>0.2886676670102404</v>
       </c>
-      <c r="FL43" t="n">
+      <c r="FN43" t="n">
         <v>10.38928239438009</v>
       </c>
-      <c r="FM43" t="n">
+      <c r="FO43" t="n">
         <v>8.974444776383145</v>
       </c>
-      <c r="FN43" t="n">
+      <c r="FP43" t="n">
         <v>0.3850587685763026</v>
       </c>
-      <c r="FO43" t="n">
+      <c r="FQ43" t="n">
         <v>8.982701670411204</v>
       </c>
-      <c r="FP43" t="n">
+      <c r="FR43" t="n">
         <v>10.34718403643685</v>
       </c>
-      <c r="FQ43" t="n">
+      <c r="FS43" t="n">
         <v>0.2848296797765695</v>
       </c>
-      <c r="FR43" t="n">
+      <c r="FT43" t="n">
         <v>10.35110358514372</v>
       </c>
-      <c r="FS43" t="n">
+      <c r="FU43" t="n">
         <v>10.55515648413704</v>
       </c>
-      <c r="FT43" t="n">
+      <c r="FV43" t="n">
         <v>0.2365137125803344</v>
       </c>
-      <c r="FU43" t="n">
+      <c r="FW43" t="n">
         <v>10.55780598139873</v>
       </c>
     </row>
@@ -17243,40 +17673,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ44" t="n">
+      <c r="FJ44" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK44" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL44" t="n">
         <v>11.88044494731319</v>
       </c>
-      <c r="FK44" t="n">
+      <c r="FM44" t="n">
         <v>8.660961691921244</v>
       </c>
-      <c r="FL44" t="n">
+      <c r="FN44" t="n">
         <v>14.70228654240784</v>
       </c>
-      <c r="FM44" t="n">
+      <c r="FO44" t="n">
         <v>8.180075024423862</v>
       </c>
-      <c r="FN44" t="n">
+      <c r="FP44" t="n">
         <v>0.7438797872583195</v>
       </c>
-      <c r="FO44" t="n">
+      <c r="FQ44" t="n">
         <v>8.213828860105044</v>
       </c>
-      <c r="FP44" t="n">
+      <c r="FR44" t="n">
         <v>10.13634144286843</v>
       </c>
-      <c r="FQ44" t="n">
+      <c r="FS44" t="n">
         <v>8.260924739217774</v>
       </c>
-      <c r="FR44" t="n">
+      <c r="FT44" t="n">
         <v>13.07624928614594</v>
       </c>
-      <c r="FS44" t="n">
+      <c r="FU44" t="n">
         <v>10.50693258013568</v>
       </c>
-      <c r="FT44" t="n">
+      <c r="FV44" t="n">
         <v>6.976419236690684</v>
       </c>
-      <c r="FU44" t="n">
+      <c r="FW44" t="n">
         <v>12.61213929551939</v>
       </c>
     </row>
@@ -17630,40 +18070,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ45" t="n">
+      <c r="FJ45" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK45" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL45" t="n">
         <v>22.1077045392002</v>
       </c>
-      <c r="FK45" t="n">
+      <c r="FM45" t="n">
         <v>0.8128534359202585</v>
       </c>
-      <c r="FL45" t="n">
+      <c r="FN45" t="n">
         <v>22.12264294113297</v>
       </c>
-      <c r="FM45" t="n">
+      <c r="FO45" t="n">
         <v>17.66376467168595</v>
       </c>
-      <c r="FN45" t="n">
+      <c r="FP45" t="n">
         <v>0.2927971303862626</v>
       </c>
-      <c r="FO45" t="n">
+      <c r="FQ45" t="n">
         <v>17.66619122890565</v>
       </c>
-      <c r="FP45" t="n">
+      <c r="FR45" t="n">
         <v>22.1495997354</v>
       </c>
-      <c r="FQ45" t="n">
+      <c r="FS45" t="n">
         <v>0.7917744789960137</v>
       </c>
-      <c r="FR45" t="n">
+      <c r="FT45" t="n">
         <v>22.16374686879502</v>
       </c>
-      <c r="FS45" t="n">
+      <c r="FU45" t="n">
         <v>22.24327583602598</v>
       </c>
-      <c r="FT45" t="n">
+      <c r="FV45" t="n">
         <v>0.388625826233246</v>
       </c>
-      <c r="FU45" t="n">
+      <c r="FW45" t="n">
         <v>22.24667053629268</v>
       </c>
     </row>
@@ -18017,40 +18467,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ46" t="n">
+      <c r="FJ46" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK46" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL46" t="n">
         <v>10.80137586815453</v>
       </c>
-      <c r="FK46" t="n">
+      <c r="FM46" t="n">
         <v>0.4299285338922029</v>
       </c>
-      <c r="FL46" t="n">
+      <c r="FN46" t="n">
         <v>10.80992873193</v>
       </c>
-      <c r="FM46" t="n">
+      <c r="FO46" t="n">
         <v>7.369149374544905</v>
       </c>
-      <c r="FN46" t="n">
+      <c r="FP46" t="n">
         <v>0.3178611798046603</v>
       </c>
-      <c r="FO46" t="n">
+      <c r="FQ46" t="n">
         <v>7.376001507184117</v>
       </c>
-      <c r="FP46" t="n">
+      <c r="FR46" t="n">
         <v>11.16010097870306</v>
       </c>
-      <c r="FQ46" t="n">
+      <c r="FS46" t="n">
         <v>0.4732286622183746</v>
       </c>
-      <c r="FR46" t="n">
+      <c r="FT46" t="n">
         <v>11.17012977639893</v>
       </c>
-      <c r="FS46" t="n">
+      <c r="FU46" t="n">
         <v>10.68672894599696</v>
       </c>
-      <c r="FT46" t="n">
+      <c r="FV46" t="n">
         <v>0.4601997783187081</v>
       </c>
-      <c r="FU46" t="n">
+      <c r="FW46" t="n">
         <v>10.69663308715289</v>
       </c>
     </row>
@@ -18404,40 +18864,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ47" t="n">
+      <c r="FJ47" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK47" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL47" t="n">
         <v>20.0538984245249</v>
       </c>
-      <c r="FK47" t="n">
+      <c r="FM47" t="n">
         <v>0.6238315334711194</v>
       </c>
-      <c r="FL47" t="n">
+      <c r="FN47" t="n">
         <v>20.06359907402745</v>
       </c>
-      <c r="FM47" t="n">
+      <c r="FO47" t="n">
         <v>18.93883142016285</v>
       </c>
-      <c r="FN47" t="n">
+      <c r="FP47" t="n">
         <v>0.2876654701510419</v>
       </c>
-      <c r="FO47" t="n">
+      <c r="FQ47" t="n">
         <v>18.94101599661604</v>
       </c>
-      <c r="FP47" t="n">
+      <c r="FR47" t="n">
         <v>20.09329570036371</v>
       </c>
-      <c r="FQ47" t="n">
+      <c r="FS47" t="n">
         <v>0.5554058093528184</v>
       </c>
-      <c r="FR47" t="n">
+      <c r="FT47" t="n">
         <v>20.10097031775625</v>
       </c>
-      <c r="FS47" t="n">
+      <c r="FU47" t="n">
         <v>20.44431434099486</v>
       </c>
-      <c r="FT47" t="n">
+      <c r="FV47" t="n">
         <v>0.2945979954100831</v>
       </c>
-      <c r="FU47" t="n">
+      <c r="FW47" t="n">
         <v>20.4464367764241</v>
       </c>
     </row>
@@ -18791,40 +19261,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ48" t="n">
+      <c r="FJ48" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK48" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL48" t="n">
         <v>11.6557707743052</v>
       </c>
-      <c r="FK48" t="n">
+      <c r="FM48" t="n">
         <v>7.956897178585111</v>
       </c>
-      <c r="FL48" t="n">
+      <c r="FN48" t="n">
         <v>14.11273201948237</v>
       </c>
-      <c r="FM48" t="n">
+      <c r="FO48" t="n">
         <v>7.335552251190117</v>
       </c>
-      <c r="FN48" t="n">
+      <c r="FP48" t="n">
         <v>0.9043763527409775</v>
       </c>
-      <c r="FO48" t="n">
+      <c r="FQ48" t="n">
         <v>7.391090813766088</v>
       </c>
-      <c r="FP48" t="n">
+      <c r="FR48" t="n">
         <v>11.15420111432968</v>
       </c>
-      <c r="FQ48" t="n">
+      <c r="FS48" t="n">
         <v>5.119030326065718</v>
       </c>
-      <c r="FR48" t="n">
+      <c r="FT48" t="n">
         <v>12.27276146505317</v>
       </c>
-      <c r="FS48" t="n">
+      <c r="FU48" t="n">
         <v>10.99012684447801</v>
       </c>
-      <c r="FT48" t="n">
+      <c r="FV48" t="n">
         <v>5.685465874996043</v>
       </c>
-      <c r="FU48" t="n">
+      <c r="FW48" t="n">
         <v>12.37365791807179</v>
       </c>
     </row>
@@ -19178,40 +19658,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ49" t="n">
+      <c r="FJ49" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK49" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL49" t="n">
         <v>10.22944205116218</v>
       </c>
-      <c r="FK49" t="n">
+      <c r="FM49" t="n">
         <v>0.5855189811064064</v>
       </c>
-      <c r="FL49" t="n">
+      <c r="FN49" t="n">
         <v>10.24618549291984</v>
       </c>
-      <c r="FM49" t="n">
+      <c r="FO49" t="n">
         <v>6.750917261273964</v>
       </c>
-      <c r="FN49" t="n">
+      <c r="FP49" t="n">
         <v>0.3410006127637463</v>
       </c>
-      <c r="FO49" t="n">
+      <c r="FQ49" t="n">
         <v>6.759524042894737</v>
       </c>
-      <c r="FP49" t="n">
+      <c r="FR49" t="n">
         <v>10.42054363713724</v>
       </c>
-      <c r="FQ49" t="n">
+      <c r="FS49" t="n">
         <v>0.5847952033898697</v>
       </c>
-      <c r="FR49" t="n">
+      <c r="FT49" t="n">
         <v>10.43693993100417</v>
       </c>
-      <c r="FS49" t="n">
+      <c r="FU49" t="n">
         <v>10.55796142883602</v>
       </c>
-      <c r="FT49" t="n">
+      <c r="FV49" t="n">
         <v>0.4337608478529744</v>
       </c>
-      <c r="FU49" t="n">
+      <c r="FW49" t="n">
         <v>10.56686793737479</v>
       </c>
     </row>
@@ -19565,40 +20055,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ50" t="n">
+      <c r="FJ50" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK50" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL50" t="n">
         <v>10.7366101191965</v>
       </c>
-      <c r="FK50" t="n">
+      <c r="FM50" t="n">
         <v>0.5538399442945444</v>
       </c>
-      <c r="FL50" t="n">
+      <c r="FN50" t="n">
         <v>10.75088533728869</v>
       </c>
-      <c r="FM50" t="n">
+      <c r="FO50" t="n">
         <v>7.027712361356873</v>
       </c>
-      <c r="FN50" t="n">
+      <c r="FP50" t="n">
         <v>0.3006050384792418</v>
       </c>
-      <c r="FO50" t="n">
+      <c r="FQ50" t="n">
         <v>7.034138499000948</v>
       </c>
-      <c r="FP50" t="n">
+      <c r="FR50" t="n">
         <v>10.93888332682259</v>
       </c>
-      <c r="FQ50" t="n">
+      <c r="FS50" t="n">
         <v>0.6301442808452384</v>
       </c>
-      <c r="FR50" t="n">
+      <c r="FT50" t="n">
         <v>10.95701831031231</v>
       </c>
-      <c r="FS50" t="n">
+      <c r="FU50" t="n">
         <v>10.27827711339434</v>
       </c>
-      <c r="FT50" t="n">
+      <c r="FV50" t="n">
         <v>0.4389302948807479</v>
       </c>
-      <c r="FU50" t="n">
+      <c r="FW50" t="n">
         <v>10.28764502806595</v>
       </c>
     </row>
@@ -19952,40 +20452,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ51" t="n">
+      <c r="FJ51" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK51" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL51" t="n">
         <v>11.22581721532976</v>
       </c>
-      <c r="FK51" t="n">
+      <c r="FM51" t="n">
         <v>6.94666798192139</v>
       </c>
-      <c r="FL51" t="n">
+      <c r="FN51" t="n">
         <v>13.20133206169157</v>
       </c>
-      <c r="FM51" t="n">
+      <c r="FO51" t="n">
         <v>6.999426226388422</v>
       </c>
-      <c r="FN51" t="n">
+      <c r="FP51" t="n">
         <v>0.8310790375417791</v>
       </c>
-      <c r="FO51" t="n">
+      <c r="FQ51" t="n">
         <v>7.048592757798923</v>
       </c>
-      <c r="FP51" t="n">
+      <c r="FR51" t="n">
         <v>11.8030922168786</v>
       </c>
-      <c r="FQ51" t="n">
+      <c r="FS51" t="n">
         <v>7.343032097777538</v>
       </c>
-      <c r="FR51" t="n">
+      <c r="FT51" t="n">
         <v>13.90083113591167</v>
       </c>
-      <c r="FS51" t="n">
+      <c r="FU51" t="n">
         <v>10.91978246879043</v>
       </c>
-      <c r="FT51" t="n">
+      <c r="FV51" t="n">
         <v>6.038078876048384</v>
       </c>
-      <c r="FU51" t="n">
+      <c r="FW51" t="n">
         <v>12.47798243623882</v>
       </c>
     </row>
@@ -20229,8 +20739,16 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ52" t="inlineStr"/>
-      <c r="FK52" t="inlineStr"/>
+      <c r="FJ52" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK52" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
       <c r="FL52" t="inlineStr"/>
       <c r="FM52" t="inlineStr"/>
       <c r="FN52" t="inlineStr"/>
@@ -20241,6 +20759,8 @@
       <c r="FS52" t="inlineStr"/>
       <c r="FT52" t="inlineStr"/>
       <c r="FU52" t="inlineStr"/>
+      <c r="FV52" t="inlineStr"/>
+      <c r="FW52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -20592,40 +21112,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ53" t="n">
+      <c r="FJ53" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK53" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL53" t="n">
         <v>20.17708854821833</v>
       </c>
-      <c r="FK53" t="n">
+      <c r="FM53" t="n">
         <v>6.686059177245952</v>
       </c>
-      <c r="FL53" t="n">
+      <c r="FN53" t="n">
         <v>21.25601772685274</v>
       </c>
-      <c r="FM53" t="n">
+      <c r="FO53" t="n">
         <v>18.0621203633565</v>
       </c>
-      <c r="FN53" t="n">
+      <c r="FP53" t="n">
         <v>0.7781402084262911</v>
       </c>
-      <c r="FO53" t="n">
+      <c r="FQ53" t="n">
         <v>18.07887425157737</v>
       </c>
-      <c r="FP53" t="n">
+      <c r="FR53" t="n">
         <v>20.20534763097545</v>
       </c>
-      <c r="FQ53" t="n">
+      <c r="FS53" t="n">
         <v>5.879779749053572</v>
       </c>
-      <c r="FR53" t="n">
+      <c r="FT53" t="n">
         <v>21.04347601481147</v>
       </c>
-      <c r="FS53" t="n">
+      <c r="FU53" t="n">
         <v>20.36824975109708</v>
       </c>
-      <c r="FT53" t="n">
+      <c r="FV53" t="n">
         <v>5.366600161202084</v>
       </c>
-      <c r="FU53" t="n">
+      <c r="FW53" t="n">
         <v>21.06338043176547</v>
       </c>
     </row>
@@ -20979,40 +21509,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ54" t="n">
+      <c r="FJ54" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK54" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL54" t="n">
         <v>22.5020510181746</v>
       </c>
-      <c r="FK54" t="n">
+      <c r="FM54" t="n">
         <v>3.934441801102209</v>
       </c>
-      <c r="FL54" t="n">
+      <c r="FN54" t="n">
         <v>22.84342645731574</v>
       </c>
-      <c r="FM54" t="n">
+      <c r="FO54" t="n">
         <v>15.56154852524487</v>
       </c>
-      <c r="FN54" t="n">
+      <c r="FP54" t="n">
         <v>0.8159737561248953</v>
       </c>
-      <c r="FO54" t="n">
+      <c r="FQ54" t="n">
         <v>15.5829267364714</v>
       </c>
-      <c r="FP54" t="n">
+      <c r="FR54" t="n">
         <v>21.89406239880842</v>
       </c>
-      <c r="FQ54" t="n">
+      <c r="FS54" t="n">
         <v>5.10820739219287</v>
       </c>
-      <c r="FR54" t="n">
+      <c r="FT54" t="n">
         <v>22.48207621828043</v>
       </c>
-      <c r="FS54" t="n">
+      <c r="FU54" t="n">
         <v>22.02470768810516</v>
       </c>
-      <c r="FT54" t="n">
+      <c r="FV54" t="n">
         <v>3.997794742610248</v>
       </c>
-      <c r="FU54" t="n">
+      <c r="FW54" t="n">
         <v>22.38459540734477</v>
       </c>
     </row>
@@ -21366,40 +21906,50 @@
           <t>PROCESSED-20260307-ProbPos4_31_FPV_2-tett6roof</t>
         </is>
       </c>
-      <c r="FJ55" t="n">
+      <c r="FJ55" t="inlineStr">
+        <is>
+          <t>9373/170</t>
+        </is>
+      </c>
+      <c r="FK55" t="inlineStr">
+        <is>
+          <t>12545</t>
+        </is>
+      </c>
+      <c r="FL55" t="n">
         <v>10.53190908141337</v>
       </c>
-      <c r="FK55" t="n">
+      <c r="FM55" t="n">
         <v>0.5231786458072176</v>
       </c>
-      <c r="FL55" t="n">
+      <c r="FN55" t="n">
         <v>10.54489567490291</v>
       </c>
-      <c r="FM55" t="n">
+      <c r="FO55" t="n">
         <v>7.096262651415318</v>
       </c>
-      <c r="FN55" t="n">
+      <c r="FP55" t="n">
         <v>0.3267813258420401</v>
       </c>
-      <c r="FO55" t="n">
+      <c r="FQ55" t="n">
         <v>7.103782770664589</v>
       </c>
-      <c r="FP55" t="n">
+      <c r="FR55" t="n">
         <v>10.78673999595023</v>
       </c>
-      <c r="FQ55" t="n">
+      <c r="FS55" t="n">
         <v>0.5690584475472223</v>
       </c>
-      <c r="FR55" t="n">
+      <c r="FT55" t="n">
         <v>10.80174001061668</v>
       </c>
-      <c r="FS55" t="n">
+      <c r="FU55" t="n">
         <v>10.38115647961444</v>
       </c>
-      <c r="FT55" t="n">
+      <c r="FV55" t="n">
         <v>0.3826566022420553</v>
       </c>
-      <c r="FU55" t="n">
+      <c r="FW55" t="n">
         <v>10.38820657907226</v>
       </c>
     </row>

</xml_diff>